<commit_message>
Fix: formato de dinero con puntos, NIT y cédula con puntos, limpieza y justificación de objeto
</commit_message>
<xml_diff>
--- a/plantillas/CUENTA_COBRO.xlsx
+++ b/plantillas/CUENTA_COBRO.xlsx
@@ -120,7 +120,7 @@
     <numFmt numFmtId="167" formatCode="##,###"/>
     <numFmt numFmtId="168" formatCode="&quot;$&quot;\ #,##0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -131,43 +131,51 @@
       <sz val="8"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Verdana"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Verdana"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Verdana"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Verdana"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Verdana"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -684,7 +692,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -735,24 +743,115 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -762,88 +861,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -876,7 +893,7 @@
         <xdr:cNvPr id="3" name="Shape 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000003000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -931,7 +948,7 @@
         <xdr:cNvPr id="4" name="Shape 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000004000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -986,7 +1003,7 @@
         <xdr:cNvPr id="2" name="Shape 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1041,7 +1058,7 @@
         <xdr:cNvPr id="5" name="Shape 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000005000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1096,7 +1113,7 @@
         <xdr:cNvPr id="6" name="Shape 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000006000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1197,7 +1214,7 @@
         <xdr:cNvPr id="7" name="Shape 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000007000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000007000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1216,7 +1233,7 @@
           <xdr:cNvPr id="8" name="Shape 6">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000008000000}"/>
+                <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000008000000}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
@@ -1235,7 +1252,7 @@
             <xdr:cNvPr id="9" name="Shape 7">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000009000000}"/>
+                  <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1278,7 +1295,7 @@
             <xdr:cNvPr id="10" name="Shape 8">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000A000000}"/>
+                  <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000A000000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1297,7 +1314,7 @@
               <xdr:cNvPr id="11" name="Shape 9">
                 <a:extLst>
                   <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000B000000}"/>
+                    <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000B000000}"/>
                   </a:ext>
                 </a:extLst>
               </xdr:cNvPr>
@@ -1342,7 +1359,7 @@
               <xdr:cNvPr id="12" name="Shape 10">
                 <a:extLst>
                   <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000C000000}"/>
+                    <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000C000000}"/>
                   </a:ext>
                 </a:extLst>
               </xdr:cNvPr>
@@ -1361,7 +1378,7 @@
                 <xdr:cNvPr id="13" name="Shape 11">
                   <a:extLst>
                     <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000D000000}"/>
+                      <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000D000000}"/>
                     </a:ext>
                   </a:extLst>
                 </xdr:cNvPr>
@@ -1406,7 +1423,7 @@
                 <xdr:cNvPr id="14" name="Shape 12">
                   <a:extLst>
                     <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000E000000}"/>
+                      <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000E000000}"/>
                     </a:ext>
                   </a:extLst>
                 </xdr:cNvPr>
@@ -1425,7 +1442,7 @@
                   <xdr:cNvPr id="15" name="Shape 13">
                     <a:extLst>
                       <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000F000000}"/>
+                        <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000F000000}"/>
                       </a:ext>
                     </a:extLst>
                   </xdr:cNvPr>
@@ -1470,7 +1487,7 @@
                   <xdr:cNvPr id="16" name="Shape 14">
                     <a:extLst>
                       <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000010000000}"/>
+                        <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000010000000}"/>
                       </a:ext>
                     </a:extLst>
                   </xdr:cNvPr>
@@ -1489,7 +1506,7 @@
                     <xdr:cNvPr id="17" name="Shape 15">
                       <a:extLst>
                         <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                          <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000011000000}"/>
+                          <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000011000000}"/>
                         </a:ext>
                       </a:extLst>
                     </xdr:cNvPr>
@@ -1534,7 +1551,7 @@
                     <xdr:cNvPr id="18" name="Shape 16">
                       <a:extLst>
                         <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                          <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000012000000}"/>
+                          <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000012000000}"/>
                         </a:ext>
                       </a:extLst>
                     </xdr:cNvPr>
@@ -1553,7 +1570,7 @@
                       <xdr:cNvPr id="19" name="Shape 17">
                         <a:extLst>
                           <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                            <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000013000000}"/>
+                            <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000013000000}"/>
                           </a:ext>
                         </a:extLst>
                       </xdr:cNvPr>
@@ -1598,7 +1615,7 @@
                       <xdr:cNvPr id="20" name="Shape 18">
                         <a:extLst>
                           <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                            <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000014000000}"/>
+                            <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000014000000}"/>
                           </a:ext>
                         </a:extLst>
                       </xdr:cNvPr>
@@ -1617,7 +1634,7 @@
                         <xdr:cNvPr id="21" name="Shape 19">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000015000000}"/>
+                              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000015000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -1668,7 +1685,7 @@
                         <xdr:cNvPr id="22" name="Shape 20">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000016000000}"/>
+                              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000016000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -1744,7 +1761,7 @@
                         <xdr:cNvPr id="23" name="Shape 21">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000017000000}"/>
+                              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000017000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -1812,7 +1829,7 @@
                         <xdr:cNvPr id="24" name="Shape 22">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000018000000}"/>
+                              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000018000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -1880,7 +1897,7 @@
                         <xdr:cNvPr id="25" name="Shape 23">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000019000000}"/>
+                              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000019000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -2055,7 +2072,7 @@
                       <xdr:cNvPr id="26" name="Shape 24" descr="escudo">
                         <a:extLst>
                           <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                            <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00001A000000}"/>
+                            <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001A000000}"/>
                           </a:ext>
                         </a:extLst>
                       </xdr:cNvPr>
@@ -2293,7 +2310,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="10.7109375" customWidth="1"/>
     <col min="4" max="4" width="8.7109375" customWidth="1"/>
@@ -2308,16 +2325,16 @@
     <col min="14" max="26" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="13.5" customHeight="1">
-      <c r="A1" s="23"/>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
+    <row r="1" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="70"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
@@ -2336,16 +2353,16 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="13.5" customHeight="1">
-      <c r="A2" s="24"/>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
+    <row r="2" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="56"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
@@ -2364,16 +2381,16 @@
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
     </row>
-    <row r="3" spans="1:26" ht="13.5" customHeight="1">
-      <c r="A3" s="24"/>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
+    <row r="3" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="56"/>
+      <c r="B3" s="56"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="56"/>
+      <c r="G3" s="56"/>
+      <c r="H3" s="56"/>
+      <c r="I3" s="56"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
@@ -2392,16 +2409,16 @@
       <c r="Y3" s="1"/>
       <c r="Z3" s="1"/>
     </row>
-    <row r="4" spans="1:26" ht="15" customHeight="1">
-      <c r="A4" s="24"/>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
-      <c r="G4" s="24"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="24"/>
+    <row r="4" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="56"/>
+      <c r="B4" s="56"/>
+      <c r="C4" s="56"/>
+      <c r="D4" s="56"/>
+      <c r="E4" s="56"/>
+      <c r="F4" s="56"/>
+      <c r="G4" s="56"/>
+      <c r="H4" s="56"/>
+      <c r="I4" s="56"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
@@ -2420,16 +2437,16 @@
       <c r="Y4" s="1"/>
       <c r="Z4" s="1"/>
     </row>
-    <row r="5" spans="1:26" ht="16.5" customHeight="1">
-      <c r="A5" s="24"/>
-      <c r="B5" s="24"/>
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="24"/>
-      <c r="H5" s="24"/>
-      <c r="I5" s="24"/>
+    <row r="5" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="56"/>
+      <c r="B5" s="56"/>
+      <c r="C5" s="56"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="56"/>
+      <c r="F5" s="56"/>
+      <c r="G5" s="56"/>
+      <c r="H5" s="56"/>
+      <c r="I5" s="56"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
@@ -2448,16 +2465,16 @@
       <c r="Y5" s="1"/>
       <c r="Z5" s="1"/>
     </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A6" s="24"/>
-      <c r="B6" s="24"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="24"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="24"/>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="56"/>
+      <c r="B6" s="56"/>
+      <c r="C6" s="56"/>
+      <c r="D6" s="56"/>
+      <c r="E6" s="56"/>
+      <c r="F6" s="56"/>
+      <c r="G6" s="56"/>
+      <c r="H6" s="56"/>
+      <c r="I6" s="56"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
@@ -2476,16 +2493,16 @@
       <c r="Y6" s="1"/>
       <c r="Z6" s="1"/>
     </row>
-    <row r="7" spans="1:26" ht="13.5" customHeight="1">
-      <c r="A7" s="24"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="24"/>
+    <row r="7" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="56"/>
+      <c r="B7" s="56"/>
+      <c r="C7" s="56"/>
+      <c r="D7" s="56"/>
+      <c r="E7" s="56"/>
+      <c r="F7" s="56"/>
+      <c r="G7" s="56"/>
+      <c r="H7" s="56"/>
+      <c r="I7" s="56"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
@@ -2504,16 +2521,16 @@
       <c r="Y7" s="1"/>
       <c r="Z7" s="1"/>
     </row>
-    <row r="8" spans="1:26" ht="13.5" customHeight="1">
-      <c r="A8" s="24"/>
-      <c r="B8" s="24"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="24"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="24"/>
+    <row r="8" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="56"/>
+      <c r="B8" s="56"/>
+      <c r="C8" s="56"/>
+      <c r="D8" s="56"/>
+      <c r="E8" s="56"/>
+      <c r="F8" s="56"/>
+      <c r="G8" s="56"/>
+      <c r="H8" s="56"/>
+      <c r="I8" s="56"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
@@ -2532,16 +2549,16 @@
       <c r="Y8" s="1"/>
       <c r="Z8" s="1"/>
     </row>
-    <row r="9" spans="1:26" ht="13.5" customHeight="1">
-      <c r="A9" s="24"/>
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="24"/>
-      <c r="H9" s="24"/>
-      <c r="I9" s="24"/>
+    <row r="9" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="56"/>
+      <c r="B9" s="56"/>
+      <c r="C9" s="56"/>
+      <c r="D9" s="56"/>
+      <c r="E9" s="56"/>
+      <c r="F9" s="56"/>
+      <c r="G9" s="56"/>
+      <c r="H9" s="56"/>
+      <c r="I9" s="56"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
@@ -2560,16 +2577,16 @@
       <c r="Y9" s="1"/>
       <c r="Z9" s="1"/>
     </row>
-    <row r="10" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A10" s="24"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="24"/>
+    <row r="10" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="56"/>
+      <c r="B10" s="56"/>
+      <c r="C10" s="56"/>
+      <c r="D10" s="56"/>
+      <c r="E10" s="56"/>
+      <c r="F10" s="56"/>
+      <c r="G10" s="56"/>
+      <c r="H10" s="56"/>
+      <c r="I10" s="56"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
@@ -2588,18 +2605,18 @@
       <c r="Y10" s="1"/>
       <c r="Z10" s="1"/>
     </row>
-    <row r="11" spans="1:26" ht="34.5" customHeight="1">
-      <c r="A11" s="25" t="s">
+    <row r="11" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="63" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="27"/>
+      <c r="B11" s="64"/>
+      <c r="C11" s="64"/>
+      <c r="D11" s="64"/>
+      <c r="E11" s="64"/>
+      <c r="F11" s="64"/>
+      <c r="G11" s="64"/>
+      <c r="H11" s="64"/>
+      <c r="I11" s="65"/>
       <c r="J11" s="17">
         <v>1</v>
       </c>
@@ -2620,14 +2637,14 @@
       <c r="Y11" s="2"/>
       <c r="Z11" s="2"/>
     </row>
-    <row r="12" spans="1:26" ht="39.75" customHeight="1">
-      <c r="A12" s="28" t="s">
+    <row r="12" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="29"/>
-      <c r="C12" s="30"/>
-      <c r="D12" s="31"/>
-      <c r="E12" s="32"/>
+      <c r="B12" s="72"/>
+      <c r="C12" s="73"/>
+      <c r="D12" s="74"/>
+      <c r="E12" s="75"/>
       <c r="F12" s="3" t="s">
         <v>2</v>
       </c>
@@ -2656,17 +2673,17 @@
       <c r="Y12" s="2"/>
       <c r="Z12" s="2"/>
     </row>
-    <row r="13" spans="1:26" ht="28.5" customHeight="1">
-      <c r="A13" s="33" t="s">
+    <row r="13" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="60" t="s">
         <v>4</v>
       </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="34" t="s">
+      <c r="B13" s="38"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="58" t="s">
         <v>5</v>
       </c>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="38"/>
       <c r="G13" s="7" t="s">
         <v>6</v>
       </c>
@@ -2694,24 +2711,24 @@
       <c r="Y13" s="2"/>
       <c r="Z13" s="2"/>
     </row>
-    <row r="14" spans="1:26" ht="28.5" customHeight="1">
-      <c r="A14" s="33" t="s">
+    <row r="14" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="19"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="18" t="s">
+      <c r="B14" s="38"/>
+      <c r="C14" s="39"/>
+      <c r="D14" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="19"/>
-      <c r="F14" s="20"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="39"/>
       <c r="G14" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="H14" s="21">
+      <c r="H14" s="62">
         <v>4121</v>
       </c>
-      <c r="I14" s="22"/>
+      <c r="I14" s="43"/>
       <c r="J14" s="6"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
@@ -2730,24 +2747,24 @@
       <c r="Y14" s="2"/>
       <c r="Z14" s="2"/>
     </row>
-    <row r="15" spans="1:26" ht="28.5" customHeight="1">
-      <c r="A15" s="33" t="s">
+    <row r="15" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="60" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="19"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="35" t="s">
+      <c r="B15" s="38"/>
+      <c r="C15" s="39"/>
+      <c r="D15" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="19"/>
-      <c r="F15" s="20"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="39"/>
       <c r="G15" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="21">
+      <c r="H15" s="62">
         <v>8896744</v>
       </c>
-      <c r="I15" s="22"/>
+      <c r="I15" s="43"/>
       <c r="J15" s="6"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
@@ -2766,18 +2783,18 @@
       <c r="Y15" s="2"/>
       <c r="Z15" s="2"/>
     </row>
-    <row r="16" spans="1:26" ht="34.5" customHeight="1">
-      <c r="A16" s="25" t="s">
+    <row r="16" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="26"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26"/>
-      <c r="H16" s="26"/>
-      <c r="I16" s="27"/>
+      <c r="B16" s="64"/>
+      <c r="C16" s="64"/>
+      <c r="D16" s="64"/>
+      <c r="E16" s="64"/>
+      <c r="F16" s="64"/>
+      <c r="G16" s="64"/>
+      <c r="H16" s="64"/>
+      <c r="I16" s="65"/>
       <c r="J16" s="17">
         <v>2</v>
       </c>
@@ -2798,15 +2815,15 @@
       <c r="Y16" s="2"/>
       <c r="Z16" s="2"/>
     </row>
-    <row r="17" spans="1:26" ht="45" customHeight="1">
-      <c r="A17" s="36" t="s">
+    <row r="17" spans="1:26" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="66" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="37"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="38"/>
+      <c r="B17" s="67"/>
+      <c r="C17" s="68"/>
+      <c r="D17" s="69"/>
+      <c r="E17" s="67"/>
+      <c r="F17" s="68"/>
       <c r="G17" s="11" t="s">
         <v>15</v>
       </c>
@@ -2830,20 +2847,20 @@
       <c r="Y17" s="2"/>
       <c r="Z17" s="2"/>
     </row>
-    <row r="18" spans="1:26" ht="28.5" customHeight="1">
-      <c r="A18" s="33" t="s">
+    <row r="18" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="60" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="19"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="20"/>
+      <c r="B18" s="38"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="58"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="39"/>
       <c r="G18" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="H18" s="18"/>
-      <c r="I18" s="22"/>
+      <c r="H18" s="59"/>
+      <c r="I18" s="43"/>
       <c r="J18" s="6"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
@@ -2862,20 +2879,20 @@
       <c r="Y18" s="2"/>
       <c r="Z18" s="2"/>
     </row>
-    <row r="19" spans="1:26" ht="28.5" customHeight="1">
-      <c r="A19" s="60" t="s">
+    <row r="19" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="43"/>
-      <c r="C19" s="41"/>
-      <c r="D19" s="61"/>
-      <c r="E19" s="43"/>
-      <c r="F19" s="41"/>
+      <c r="B19" s="19"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="20"/>
       <c r="G19" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="H19" s="62"/>
-      <c r="I19" s="44"/>
+      <c r="H19" s="22"/>
+      <c r="I19" s="23"/>
       <c r="J19" s="6"/>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
@@ -2894,18 +2911,18 @@
       <c r="Y19" s="2"/>
       <c r="Z19" s="2"/>
     </row>
-    <row r="20" spans="1:26" ht="34.5" customHeight="1">
-      <c r="A20" s="63" t="s">
+    <row r="20" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="64"/>
-      <c r="C20" s="64"/>
-      <c r="D20" s="64"/>
-      <c r="E20" s="64"/>
-      <c r="F20" s="64"/>
-      <c r="G20" s="64"/>
-      <c r="H20" s="64"/>
-      <c r="I20" s="65"/>
+      <c r="B20" s="25"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="25"/>
+      <c r="G20" s="25"/>
+      <c r="H20" s="25"/>
+      <c r="I20" s="26"/>
       <c r="J20" s="17">
         <v>3</v>
       </c>
@@ -2926,18 +2943,18 @@
       <c r="Y20" s="2"/>
       <c r="Z20" s="2"/>
     </row>
-    <row r="21" spans="1:26" ht="24.75" customHeight="1">
-      <c r="A21" s="66" t="s">
+    <row r="21" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="64"/>
-      <c r="C21" s="67"/>
-      <c r="D21" s="68"/>
-      <c r="E21" s="69"/>
-      <c r="F21" s="69"/>
-      <c r="G21" s="69"/>
-      <c r="H21" s="69"/>
-      <c r="I21" s="70"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="33"/>
+      <c r="G21" s="33"/>
+      <c r="H21" s="33"/>
+      <c r="I21" s="34"/>
       <c r="J21" s="17"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
@@ -2956,16 +2973,16 @@
       <c r="Y21" s="2"/>
       <c r="Z21" s="2"/>
     </row>
-    <row r="22" spans="1:26" ht="24.75" customHeight="1">
-      <c r="A22" s="49"/>
-      <c r="B22" s="50"/>
-      <c r="C22" s="51"/>
-      <c r="D22" s="71"/>
-      <c r="E22" s="71"/>
-      <c r="F22" s="71"/>
-      <c r="G22" s="71"/>
-      <c r="H22" s="71"/>
-      <c r="I22" s="72"/>
+    <row r="22" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="29"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="35"/>
+      <c r="E22" s="35"/>
+      <c r="F22" s="35"/>
+      <c r="G22" s="35"/>
+      <c r="H22" s="35"/>
+      <c r="I22" s="36"/>
       <c r="J22" s="17"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
@@ -2984,18 +3001,18 @@
       <c r="Y22" s="2"/>
       <c r="Z22" s="2"/>
     </row>
-    <row r="23" spans="1:26" ht="34.5" customHeight="1">
-      <c r="A23" s="45" t="s">
+    <row r="23" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="43"/>
-      <c r="C23" s="41"/>
-      <c r="D23" s="40"/>
-      <c r="E23" s="41"/>
-      <c r="F23" s="42"/>
-      <c r="G23" s="43"/>
-      <c r="H23" s="43"/>
-      <c r="I23" s="44"/>
+      <c r="B23" s="19"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="48"/>
+      <c r="G23" s="19"/>
+      <c r="H23" s="19"/>
+      <c r="I23" s="23"/>
       <c r="J23" s="17"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
@@ -3014,18 +3031,18 @@
       <c r="Y23" s="2"/>
       <c r="Z23" s="2"/>
     </row>
-    <row r="24" spans="1:26" ht="34.5" customHeight="1">
-      <c r="A24" s="54" t="s">
+    <row r="24" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="55" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="24"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="24"/>
-      <c r="H24" s="24"/>
-      <c r="I24" s="55"/>
+      <c r="B24" s="56"/>
+      <c r="C24" s="56"/>
+      <c r="D24" s="56"/>
+      <c r="E24" s="56"/>
+      <c r="F24" s="56"/>
+      <c r="G24" s="56"/>
+      <c r="H24" s="56"/>
+      <c r="I24" s="57"/>
       <c r="J24" s="17">
         <v>4</v>
       </c>
@@ -3046,20 +3063,20 @@
       <c r="Y24" s="2"/>
       <c r="Z24" s="2"/>
     </row>
-    <row r="25" spans="1:26" ht="28.5" customHeight="1">
-      <c r="A25" s="46" t="s">
+    <row r="25" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="47"/>
-      <c r="C25" s="48"/>
-      <c r="D25" s="52"/>
-      <c r="E25" s="47"/>
-      <c r="F25" s="48"/>
+      <c r="B25" s="51"/>
+      <c r="C25" s="52"/>
+      <c r="D25" s="53"/>
+      <c r="E25" s="51"/>
+      <c r="F25" s="52"/>
       <c r="G25" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="H25" s="58"/>
-      <c r="I25" s="22"/>
+      <c r="H25" s="42"/>
+      <c r="I25" s="43"/>
       <c r="J25" s="17"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
@@ -3078,18 +3095,18 @@
       <c r="Y25" s="2"/>
       <c r="Z25" s="2"/>
     </row>
-    <row r="26" spans="1:26" ht="28.5" customHeight="1">
-      <c r="A26" s="49"/>
-      <c r="B26" s="50"/>
-      <c r="C26" s="51"/>
-      <c r="D26" s="53"/>
-      <c r="E26" s="50"/>
-      <c r="F26" s="51"/>
+    <row r="26" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="29"/>
+      <c r="B26" s="30"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="54"/>
+      <c r="E26" s="30"/>
+      <c r="F26" s="31"/>
       <c r="G26" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="H26" s="58"/>
-      <c r="I26" s="22"/>
+      <c r="H26" s="42"/>
+      <c r="I26" s="43"/>
       <c r="J26" s="17"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
@@ -3108,18 +3125,18 @@
       <c r="Y26" s="2"/>
       <c r="Z26" s="2"/>
     </row>
-    <row r="27" spans="1:26" ht="90" customHeight="1">
-      <c r="A27" s="56" t="s">
+    <row r="27" spans="1:26" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="B27" s="19"/>
-      <c r="C27" s="20"/>
-      <c r="D27" s="35"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="19"/>
-      <c r="G27" s="19"/>
-      <c r="H27" s="19"/>
-      <c r="I27" s="22"/>
+      <c r="B27" s="38"/>
+      <c r="C27" s="39"/>
+      <c r="D27" s="44"/>
+      <c r="E27" s="45"/>
+      <c r="F27" s="45"/>
+      <c r="G27" s="45"/>
+      <c r="H27" s="45"/>
+      <c r="I27" s="46"/>
       <c r="J27" s="17"/>
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
@@ -3138,18 +3155,18 @@
       <c r="Y27" s="2"/>
       <c r="Z27" s="2"/>
     </row>
-    <row r="28" spans="1:26" ht="34.5" customHeight="1">
-      <c r="A28" s="57" t="s">
+    <row r="28" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="43"/>
-      <c r="C28" s="41"/>
-      <c r="D28" s="40"/>
-      <c r="E28" s="41"/>
-      <c r="F28" s="59"/>
-      <c r="G28" s="43"/>
-      <c r="H28" s="43"/>
-      <c r="I28" s="44"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="41"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="47"/>
+      <c r="G28" s="19"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="23"/>
       <c r="J28" s="17"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
@@ -3168,7 +3185,7 @@
       <c r="Y28" s="2"/>
       <c r="Z28" s="2"/>
     </row>
-    <row r="29" spans="1:26" ht="13.5" customHeight="1">
+    <row r="29" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -3196,7 +3213,7 @@
       <c r="Y29" s="2"/>
       <c r="Z29" s="2"/>
     </row>
-    <row r="30" spans="1:26" ht="13.5" customHeight="1">
+    <row r="30" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -3224,7 +3241,7 @@
       <c r="Y30" s="2"/>
       <c r="Z30" s="2"/>
     </row>
-    <row r="31" spans="1:26" ht="13.5" customHeight="1">
+    <row r="31" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -3252,7 +3269,7 @@
       <c r="Y31" s="2"/>
       <c r="Z31" s="2"/>
     </row>
-    <row r="32" spans="1:26" ht="13.5" customHeight="1">
+    <row r="32" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -3280,7 +3297,7 @@
       <c r="Y32" s="2"/>
       <c r="Z32" s="2"/>
     </row>
-    <row r="33" spans="1:26" ht="13.5" customHeight="1">
+    <row r="33" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -3308,7 +3325,7 @@
       <c r="Y33" s="2"/>
       <c r="Z33" s="2"/>
     </row>
-    <row r="34" spans="1:26" ht="13.5" customHeight="1">
+    <row r="34" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -3336,7 +3353,7 @@
       <c r="Y34" s="2"/>
       <c r="Z34" s="2"/>
     </row>
-    <row r="35" spans="1:26" ht="13.5" customHeight="1">
+    <row r="35" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -3364,7 +3381,7 @@
       <c r="Y35" s="2"/>
       <c r="Z35" s="2"/>
     </row>
-    <row r="36" spans="1:26" ht="13.5" customHeight="1">
+    <row r="36" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -3392,7 +3409,7 @@
       <c r="Y36" s="2"/>
       <c r="Z36" s="2"/>
     </row>
-    <row r="37" spans="1:26" ht="13.5" customHeight="1">
+    <row r="37" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -3420,7 +3437,7 @@
       <c r="Y37" s="2"/>
       <c r="Z37" s="2"/>
     </row>
-    <row r="38" spans="1:26" ht="13.5" customHeight="1">
+    <row r="38" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -3448,7 +3465,7 @@
       <c r="Y38" s="2"/>
       <c r="Z38" s="2"/>
     </row>
-    <row r="39" spans="1:26" ht="13.5" customHeight="1">
+    <row r="39" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -3476,7 +3493,7 @@
       <c r="Y39" s="2"/>
       <c r="Z39" s="2"/>
     </row>
-    <row r="40" spans="1:26" ht="13.5" customHeight="1">
+    <row r="40" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -3504,7 +3521,7 @@
       <c r="Y40" s="2"/>
       <c r="Z40" s="2"/>
     </row>
-    <row r="41" spans="1:26" ht="13.5" customHeight="1">
+    <row r="41" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -3532,7 +3549,7 @@
       <c r="Y41" s="2"/>
       <c r="Z41" s="2"/>
     </row>
-    <row r="42" spans="1:26" ht="13.5" customHeight="1">
+    <row r="42" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -3560,7 +3577,7 @@
       <c r="Y42" s="2"/>
       <c r="Z42" s="2"/>
     </row>
-    <row r="43" spans="1:26" ht="13.5" customHeight="1">
+    <row r="43" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -3588,7 +3605,7 @@
       <c r="Y43" s="2"/>
       <c r="Z43" s="2"/>
     </row>
-    <row r="44" spans="1:26" ht="13.5" customHeight="1">
+    <row r="44" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -3616,7 +3633,7 @@
       <c r="Y44" s="2"/>
       <c r="Z44" s="2"/>
     </row>
-    <row r="45" spans="1:26" ht="13.5" customHeight="1">
+    <row r="45" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -3644,7 +3661,7 @@
       <c r="Y45" s="2"/>
       <c r="Z45" s="2"/>
     </row>
-    <row r="46" spans="1:26" ht="13.5" customHeight="1">
+    <row r="46" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -3672,7 +3689,7 @@
       <c r="Y46" s="2"/>
       <c r="Z46" s="2"/>
     </row>
-    <row r="47" spans="1:26" ht="13.5" customHeight="1">
+    <row r="47" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
@@ -3700,7 +3717,7 @@
       <c r="Y47" s="2"/>
       <c r="Z47" s="2"/>
     </row>
-    <row r="48" spans="1:26" ht="13.5" customHeight="1">
+    <row r="48" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -3728,7 +3745,7 @@
       <c r="Y48" s="2"/>
       <c r="Z48" s="2"/>
     </row>
-    <row r="49" spans="1:26" ht="13.5" customHeight="1">
+    <row r="49" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -3756,7 +3773,7 @@
       <c r="Y49" s="2"/>
       <c r="Z49" s="2"/>
     </row>
-    <row r="50" spans="1:26" ht="13.5" customHeight="1">
+    <row r="50" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -3784,7 +3801,7 @@
       <c r="Y50" s="2"/>
       <c r="Z50" s="2"/>
     </row>
-    <row r="51" spans="1:26" ht="13.5" customHeight="1">
+    <row r="51" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
@@ -3812,7 +3829,7 @@
       <c r="Y51" s="2"/>
       <c r="Z51" s="2"/>
     </row>
-    <row r="52" spans="1:26" ht="13.5" customHeight="1">
+    <row r="52" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
@@ -3840,7 +3857,7 @@
       <c r="Y52" s="2"/>
       <c r="Z52" s="2"/>
     </row>
-    <row r="53" spans="1:26" ht="13.5" customHeight="1">
+    <row r="53" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
@@ -3868,7 +3885,7 @@
       <c r="Y53" s="2"/>
       <c r="Z53" s="2"/>
     </row>
-    <row r="54" spans="1:26" ht="13.5" customHeight="1">
+    <row r="54" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
@@ -3896,7 +3913,7 @@
       <c r="Y54" s="2"/>
       <c r="Z54" s="2"/>
     </row>
-    <row r="55" spans="1:26" ht="13.5" customHeight="1">
+    <row r="55" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -3924,7 +3941,7 @@
       <c r="Y55" s="2"/>
       <c r="Z55" s="2"/>
     </row>
-    <row r="56" spans="1:26" ht="13.5" customHeight="1">
+    <row r="56" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
@@ -3952,7 +3969,7 @@
       <c r="Y56" s="2"/>
       <c r="Z56" s="2"/>
     </row>
-    <row r="57" spans="1:26" ht="13.5" customHeight="1">
+    <row r="57" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
@@ -3980,7 +3997,7 @@
       <c r="Y57" s="2"/>
       <c r="Z57" s="2"/>
     </row>
-    <row r="58" spans="1:26" ht="13.5" customHeight="1">
+    <row r="58" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
@@ -4008,7 +4025,7 @@
       <c r="Y58" s="2"/>
       <c r="Z58" s="2"/>
     </row>
-    <row r="59" spans="1:26" ht="13.5" customHeight="1">
+    <row r="59" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
@@ -4036,7 +4053,7 @@
       <c r="Y59" s="2"/>
       <c r="Z59" s="2"/>
     </row>
-    <row r="60" spans="1:26" ht="13.5" customHeight="1">
+    <row r="60" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
@@ -4064,7 +4081,7 @@
       <c r="Y60" s="2"/>
       <c r="Z60" s="2"/>
     </row>
-    <row r="61" spans="1:26" ht="13.5" customHeight="1">
+    <row r="61" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
@@ -4092,7 +4109,7 @@
       <c r="Y61" s="2"/>
       <c r="Z61" s="2"/>
     </row>
-    <row r="62" spans="1:26" ht="13.5" customHeight="1">
+    <row r="62" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
@@ -4120,7 +4137,7 @@
       <c r="Y62" s="2"/>
       <c r="Z62" s="2"/>
     </row>
-    <row r="63" spans="1:26" ht="13.5" customHeight="1">
+    <row r="63" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -4148,7 +4165,7 @@
       <c r="Y63" s="2"/>
       <c r="Z63" s="2"/>
     </row>
-    <row r="64" spans="1:26" ht="13.5" customHeight="1">
+    <row r="64" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
@@ -4176,7 +4193,7 @@
       <c r="Y64" s="2"/>
       <c r="Z64" s="2"/>
     </row>
-    <row r="65" spans="1:26" ht="13.5" customHeight="1">
+    <row r="65" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
@@ -4204,7 +4221,7 @@
       <c r="Y65" s="2"/>
       <c r="Z65" s="2"/>
     </row>
-    <row r="66" spans="1:26" ht="13.5" customHeight="1">
+    <row r="66" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
@@ -4232,7 +4249,7 @@
       <c r="Y66" s="2"/>
       <c r="Z66" s="2"/>
     </row>
-    <row r="67" spans="1:26" ht="13.5" customHeight="1">
+    <row r="67" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
@@ -4260,7 +4277,7 @@
       <c r="Y67" s="2"/>
       <c r="Z67" s="2"/>
     </row>
-    <row r="68" spans="1:26" ht="13.5" customHeight="1">
+    <row r="68" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
@@ -4288,7 +4305,7 @@
       <c r="Y68" s="2"/>
       <c r="Z68" s="2"/>
     </row>
-    <row r="69" spans="1:26" ht="13.5" customHeight="1">
+    <row r="69" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
@@ -4316,7 +4333,7 @@
       <c r="Y69" s="2"/>
       <c r="Z69" s="2"/>
     </row>
-    <row r="70" spans="1:26" ht="13.5" customHeight="1">
+    <row r="70" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
@@ -4344,7 +4361,7 @@
       <c r="Y70" s="2"/>
       <c r="Z70" s="2"/>
     </row>
-    <row r="71" spans="1:26" ht="13.5" customHeight="1">
+    <row r="71" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
@@ -4372,7 +4389,7 @@
       <c r="Y71" s="2"/>
       <c r="Z71" s="2"/>
     </row>
-    <row r="72" spans="1:26" ht="13.5" customHeight="1">
+    <row r="72" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
@@ -4400,7 +4417,7 @@
       <c r="Y72" s="2"/>
       <c r="Z72" s="2"/>
     </row>
-    <row r="73" spans="1:26" ht="13.5" customHeight="1">
+    <row r="73" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
@@ -4428,7 +4445,7 @@
       <c r="Y73" s="2"/>
       <c r="Z73" s="2"/>
     </row>
-    <row r="74" spans="1:26" ht="13.5" customHeight="1">
+    <row r="74" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2"/>
       <c r="B74" s="2"/>
       <c r="C74" s="2"/>
@@ -4456,7 +4473,7 @@
       <c r="Y74" s="2"/>
       <c r="Z74" s="2"/>
     </row>
-    <row r="75" spans="1:26" ht="13.5" customHeight="1">
+    <row r="75" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
@@ -4484,7 +4501,7 @@
       <c r="Y75" s="2"/>
       <c r="Z75" s="2"/>
     </row>
-    <row r="76" spans="1:26" ht="13.5" customHeight="1">
+    <row r="76" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
@@ -4512,7 +4529,7 @@
       <c r="Y76" s="2"/>
       <c r="Z76" s="2"/>
     </row>
-    <row r="77" spans="1:26" ht="13.5" customHeight="1">
+    <row r="77" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
@@ -4540,7 +4557,7 @@
       <c r="Y77" s="2"/>
       <c r="Z77" s="2"/>
     </row>
-    <row r="78" spans="1:26" ht="13.5" customHeight="1">
+    <row r="78" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
@@ -4568,7 +4585,7 @@
       <c r="Y78" s="2"/>
       <c r="Z78" s="2"/>
     </row>
-    <row r="79" spans="1:26" ht="13.5" customHeight="1">
+    <row r="79" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
@@ -4596,7 +4613,7 @@
       <c r="Y79" s="2"/>
       <c r="Z79" s="2"/>
     </row>
-    <row r="80" spans="1:26" ht="13.5" customHeight="1">
+    <row r="80" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
@@ -4624,7 +4641,7 @@
       <c r="Y80" s="2"/>
       <c r="Z80" s="2"/>
     </row>
-    <row r="81" spans="1:26" ht="13.5" customHeight="1">
+    <row r="81" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
@@ -4652,7 +4669,7 @@
       <c r="Y81" s="2"/>
       <c r="Z81" s="2"/>
     </row>
-    <row r="82" spans="1:26" ht="13.5" customHeight="1">
+    <row r="82" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
@@ -4680,7 +4697,7 @@
       <c r="Y82" s="2"/>
       <c r="Z82" s="2"/>
     </row>
-    <row r="83" spans="1:26" ht="13.5" customHeight="1">
+    <row r="83" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
@@ -4708,7 +4725,7 @@
       <c r="Y83" s="2"/>
       <c r="Z83" s="2"/>
     </row>
-    <row r="84" spans="1:26" ht="13.5" customHeight="1">
+    <row r="84" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
@@ -4736,7 +4753,7 @@
       <c r="Y84" s="2"/>
       <c r="Z84" s="2"/>
     </row>
-    <row r="85" spans="1:26" ht="13.5" customHeight="1">
+    <row r="85" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
@@ -4764,7 +4781,7 @@
       <c r="Y85" s="2"/>
       <c r="Z85" s="2"/>
     </row>
-    <row r="86" spans="1:26" ht="13.5" customHeight="1">
+    <row r="86" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
@@ -4792,7 +4809,7 @@
       <c r="Y86" s="2"/>
       <c r="Z86" s="2"/>
     </row>
-    <row r="87" spans="1:26" ht="13.5" customHeight="1">
+    <row r="87" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
@@ -4820,7 +4837,7 @@
       <c r="Y87" s="2"/>
       <c r="Z87" s="2"/>
     </row>
-    <row r="88" spans="1:26" ht="13.5" customHeight="1">
+    <row r="88" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
@@ -4848,7 +4865,7 @@
       <c r="Y88" s="2"/>
       <c r="Z88" s="2"/>
     </row>
-    <row r="89" spans="1:26" ht="13.5" customHeight="1">
+    <row r="89" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
@@ -4876,7 +4893,7 @@
       <c r="Y89" s="2"/>
       <c r="Z89" s="2"/>
     </row>
-    <row r="90" spans="1:26" ht="13.5" customHeight="1">
+    <row r="90" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
@@ -4904,7 +4921,7 @@
       <c r="Y90" s="2"/>
       <c r="Z90" s="2"/>
     </row>
-    <row r="91" spans="1:26" ht="13.5" customHeight="1">
+    <row r="91" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
@@ -4932,7 +4949,7 @@
       <c r="Y91" s="2"/>
       <c r="Z91" s="2"/>
     </row>
-    <row r="92" spans="1:26" ht="13.5" customHeight="1">
+    <row r="92" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
@@ -4960,7 +4977,7 @@
       <c r="Y92" s="2"/>
       <c r="Z92" s="2"/>
     </row>
-    <row r="93" spans="1:26" ht="13.5" customHeight="1">
+    <row r="93" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
@@ -4988,7 +5005,7 @@
       <c r="Y93" s="2"/>
       <c r="Z93" s="2"/>
     </row>
-    <row r="94" spans="1:26" ht="13.5" customHeight="1">
+    <row r="94" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
@@ -5016,7 +5033,7 @@
       <c r="Y94" s="2"/>
       <c r="Z94" s="2"/>
     </row>
-    <row r="95" spans="1:26" ht="13.5" customHeight="1">
+    <row r="95" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
@@ -5044,7 +5061,7 @@
       <c r="Y95" s="2"/>
       <c r="Z95" s="2"/>
     </row>
-    <row r="96" spans="1:26" ht="13.5" customHeight="1">
+    <row r="96" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
@@ -5072,7 +5089,7 @@
       <c r="Y96" s="2"/>
       <c r="Z96" s="2"/>
     </row>
-    <row r="97" spans="1:26" ht="13.5" customHeight="1">
+    <row r="97" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
@@ -5100,7 +5117,7 @@
       <c r="Y97" s="2"/>
       <c r="Z97" s="2"/>
     </row>
-    <row r="98" spans="1:26" ht="13.5" customHeight="1">
+    <row r="98" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
@@ -5128,7 +5145,7 @@
       <c r="Y98" s="2"/>
       <c r="Z98" s="2"/>
     </row>
-    <row r="99" spans="1:26" ht="13.5" customHeight="1">
+    <row r="99" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
@@ -5156,7 +5173,7 @@
       <c r="Y99" s="2"/>
       <c r="Z99" s="2"/>
     </row>
-    <row r="100" spans="1:26" ht="13.5" customHeight="1">
+    <row r="100" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
@@ -5184,7 +5201,7 @@
       <c r="Y100" s="2"/>
       <c r="Z100" s="2"/>
     </row>
-    <row r="101" spans="1:26" ht="13.5" customHeight="1">
+    <row r="101" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2"/>
       <c r="B101" s="2"/>
       <c r="C101" s="2"/>
@@ -5212,7 +5229,7 @@
       <c r="Y101" s="2"/>
       <c r="Z101" s="2"/>
     </row>
-    <row r="102" spans="1:26" ht="13.5" customHeight="1">
+    <row r="102" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="2"/>
       <c r="B102" s="2"/>
       <c r="C102" s="2"/>
@@ -5240,7 +5257,7 @@
       <c r="Y102" s="2"/>
       <c r="Z102" s="2"/>
     </row>
-    <row r="103" spans="1:26" ht="13.5" customHeight="1">
+    <row r="103" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="2"/>
       <c r="B103" s="2"/>
       <c r="C103" s="2"/>
@@ -5268,7 +5285,7 @@
       <c r="Y103" s="2"/>
       <c r="Z103" s="2"/>
     </row>
-    <row r="104" spans="1:26" ht="13.5" customHeight="1">
+    <row r="104" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="2"/>
       <c r="B104" s="2"/>
       <c r="C104" s="2"/>
@@ -5296,7 +5313,7 @@
       <c r="Y104" s="2"/>
       <c r="Z104" s="2"/>
     </row>
-    <row r="105" spans="1:26" ht="13.5" customHeight="1">
+    <row r="105" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="2"/>
       <c r="B105" s="2"/>
       <c r="C105" s="2"/>
@@ -5324,7 +5341,7 @@
       <c r="Y105" s="2"/>
       <c r="Z105" s="2"/>
     </row>
-    <row r="106" spans="1:26" ht="13.5" customHeight="1">
+    <row r="106" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="2"/>
       <c r="B106" s="2"/>
       <c r="C106" s="2"/>
@@ -5352,7 +5369,7 @@
       <c r="Y106" s="2"/>
       <c r="Z106" s="2"/>
     </row>
-    <row r="107" spans="1:26" ht="13.5" customHeight="1">
+    <row r="107" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="2"/>
       <c r="B107" s="2"/>
       <c r="C107" s="2"/>
@@ -5380,7 +5397,7 @@
       <c r="Y107" s="2"/>
       <c r="Z107" s="2"/>
     </row>
-    <row r="108" spans="1:26" ht="13.5" customHeight="1">
+    <row r="108" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="2"/>
       <c r="B108" s="2"/>
       <c r="C108" s="2"/>
@@ -5408,7 +5425,7 @@
       <c r="Y108" s="2"/>
       <c r="Z108" s="2"/>
     </row>
-    <row r="109" spans="1:26" ht="13.5" customHeight="1">
+    <row r="109" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="2"/>
       <c r="B109" s="2"/>
       <c r="C109" s="2"/>
@@ -5436,7 +5453,7 @@
       <c r="Y109" s="2"/>
       <c r="Z109" s="2"/>
     </row>
-    <row r="110" spans="1:26" ht="13.5" customHeight="1">
+    <row r="110" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="2"/>
       <c r="B110" s="2"/>
       <c r="C110" s="2"/>
@@ -5464,7 +5481,7 @@
       <c r="Y110" s="2"/>
       <c r="Z110" s="2"/>
     </row>
-    <row r="111" spans="1:26" ht="13.5" customHeight="1">
+    <row r="111" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
       <c r="C111" s="2"/>
@@ -5492,7 +5509,7 @@
       <c r="Y111" s="2"/>
       <c r="Z111" s="2"/>
     </row>
-    <row r="112" spans="1:26" ht="13.5" customHeight="1">
+    <row r="112" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="C112" s="2"/>
@@ -5520,7 +5537,7 @@
       <c r="Y112" s="2"/>
       <c r="Z112" s="2"/>
     </row>
-    <row r="113" spans="1:26" ht="13.5" customHeight="1">
+    <row r="113" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="2"/>
@@ -5548,7 +5565,7 @@
       <c r="Y113" s="2"/>
       <c r="Z113" s="2"/>
     </row>
-    <row r="114" spans="1:26" ht="13.5" customHeight="1">
+    <row r="114" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="2"/>
@@ -5576,7 +5593,7 @@
       <c r="Y114" s="2"/>
       <c r="Z114" s="2"/>
     </row>
-    <row r="115" spans="1:26" ht="13.5" customHeight="1">
+    <row r="115" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2"/>
       <c r="B115" s="2"/>
       <c r="C115" s="2"/>
@@ -5604,7 +5621,7 @@
       <c r="Y115" s="2"/>
       <c r="Z115" s="2"/>
     </row>
-    <row r="116" spans="1:26" ht="13.5" customHeight="1">
+    <row r="116" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2"/>
       <c r="B116" s="2"/>
       <c r="C116" s="2"/>
@@ -5632,7 +5649,7 @@
       <c r="Y116" s="2"/>
       <c r="Z116" s="2"/>
     </row>
-    <row r="117" spans="1:26" ht="13.5" customHeight="1">
+    <row r="117" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2"/>
       <c r="B117" s="2"/>
       <c r="C117" s="2"/>
@@ -5660,7 +5677,7 @@
       <c r="Y117" s="2"/>
       <c r="Z117" s="2"/>
     </row>
-    <row r="118" spans="1:26" ht="13.5" customHeight="1">
+    <row r="118" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2"/>
       <c r="B118" s="2"/>
       <c r="C118" s="2"/>
@@ -5688,7 +5705,7 @@
       <c r="Y118" s="2"/>
       <c r="Z118" s="2"/>
     </row>
-    <row r="119" spans="1:26" ht="13.5" customHeight="1">
+    <row r="119" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2"/>
       <c r="B119" s="2"/>
       <c r="C119" s="2"/>
@@ -5716,7 +5733,7 @@
       <c r="Y119" s="2"/>
       <c r="Z119" s="2"/>
     </row>
-    <row r="120" spans="1:26" ht="13.5" customHeight="1">
+    <row r="120" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2"/>
       <c r="B120" s="2"/>
       <c r="C120" s="2"/>
@@ -5744,7 +5761,7 @@
       <c r="Y120" s="2"/>
       <c r="Z120" s="2"/>
     </row>
-    <row r="121" spans="1:26" ht="13.5" customHeight="1">
+    <row r="121" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2"/>
       <c r="B121" s="2"/>
       <c r="C121" s="2"/>
@@ -5772,7 +5789,7 @@
       <c r="Y121" s="2"/>
       <c r="Z121" s="2"/>
     </row>
-    <row r="122" spans="1:26" ht="13.5" customHeight="1">
+    <row r="122" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2"/>
       <c r="B122" s="2"/>
       <c r="C122" s="2"/>
@@ -5800,7 +5817,7 @@
       <c r="Y122" s="2"/>
       <c r="Z122" s="2"/>
     </row>
-    <row r="123" spans="1:26" ht="13.5" customHeight="1">
+    <row r="123" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2"/>
       <c r="B123" s="2"/>
       <c r="C123" s="2"/>
@@ -5828,7 +5845,7 @@
       <c r="Y123" s="2"/>
       <c r="Z123" s="2"/>
     </row>
-    <row r="124" spans="1:26" ht="13.5" customHeight="1">
+    <row r="124" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2"/>
       <c r="B124" s="2"/>
       <c r="C124" s="2"/>
@@ -5856,7 +5873,7 @@
       <c r="Y124" s="2"/>
       <c r="Z124" s="2"/>
     </row>
-    <row r="125" spans="1:26" ht="13.5" customHeight="1">
+    <row r="125" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2"/>
       <c r="B125" s="2"/>
       <c r="C125" s="2"/>
@@ -5884,7 +5901,7 @@
       <c r="Y125" s="2"/>
       <c r="Z125" s="2"/>
     </row>
-    <row r="126" spans="1:26" ht="13.5" customHeight="1">
+    <row r="126" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2"/>
       <c r="B126" s="2"/>
       <c r="C126" s="2"/>
@@ -5912,7 +5929,7 @@
       <c r="Y126" s="2"/>
       <c r="Z126" s="2"/>
     </row>
-    <row r="127" spans="1:26" ht="13.5" customHeight="1">
+    <row r="127" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2"/>
       <c r="B127" s="2"/>
       <c r="C127" s="2"/>
@@ -5940,7 +5957,7 @@
       <c r="Y127" s="2"/>
       <c r="Z127" s="2"/>
     </row>
-    <row r="128" spans="1:26" ht="13.5" customHeight="1">
+    <row r="128" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2"/>
       <c r="B128" s="2"/>
       <c r="C128" s="2"/>
@@ -5968,7 +5985,7 @@
       <c r="Y128" s="2"/>
       <c r="Z128" s="2"/>
     </row>
-    <row r="129" spans="1:26" ht="13.5" customHeight="1">
+    <row r="129" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2"/>
       <c r="B129" s="2"/>
       <c r="C129" s="2"/>
@@ -5996,7 +6013,7 @@
       <c r="Y129" s="2"/>
       <c r="Z129" s="2"/>
     </row>
-    <row r="130" spans="1:26" ht="13.5" customHeight="1">
+    <row r="130" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2"/>
       <c r="B130" s="2"/>
       <c r="C130" s="2"/>
@@ -6024,7 +6041,7 @@
       <c r="Y130" s="2"/>
       <c r="Z130" s="2"/>
     </row>
-    <row r="131" spans="1:26" ht="13.5" customHeight="1">
+    <row r="131" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2"/>
       <c r="B131" s="2"/>
       <c r="C131" s="2"/>
@@ -6052,7 +6069,7 @@
       <c r="Y131" s="2"/>
       <c r="Z131" s="2"/>
     </row>
-    <row r="132" spans="1:26" ht="13.5" customHeight="1">
+    <row r="132" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2"/>
       <c r="B132" s="2"/>
       <c r="C132" s="2"/>
@@ -6080,7 +6097,7 @@
       <c r="Y132" s="2"/>
       <c r="Z132" s="2"/>
     </row>
-    <row r="133" spans="1:26" ht="13.5" customHeight="1">
+    <row r="133" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2"/>
       <c r="B133" s="2"/>
       <c r="C133" s="2"/>
@@ -6108,7 +6125,7 @@
       <c r="Y133" s="2"/>
       <c r="Z133" s="2"/>
     </row>
-    <row r="134" spans="1:26" ht="13.5" customHeight="1">
+    <row r="134" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="2"/>
       <c r="B134" s="2"/>
       <c r="C134" s="2"/>
@@ -6136,7 +6153,7 @@
       <c r="Y134" s="2"/>
       <c r="Z134" s="2"/>
     </row>
-    <row r="135" spans="1:26" ht="13.5" customHeight="1">
+    <row r="135" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="2"/>
       <c r="B135" s="2"/>
       <c r="C135" s="2"/>
@@ -6164,7 +6181,7 @@
       <c r="Y135" s="2"/>
       <c r="Z135" s="2"/>
     </row>
-    <row r="136" spans="1:26" ht="13.5" customHeight="1">
+    <row r="136" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="2"/>
       <c r="B136" s="2"/>
       <c r="C136" s="2"/>
@@ -6192,7 +6209,7 @@
       <c r="Y136" s="2"/>
       <c r="Z136" s="2"/>
     </row>
-    <row r="137" spans="1:26" ht="13.5" customHeight="1">
+    <row r="137" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="2"/>
       <c r="B137" s="2"/>
       <c r="C137" s="2"/>
@@ -6220,7 +6237,7 @@
       <c r="Y137" s="2"/>
       <c r="Z137" s="2"/>
     </row>
-    <row r="138" spans="1:26" ht="13.5" customHeight="1">
+    <row r="138" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="2"/>
       <c r="B138" s="2"/>
       <c r="C138" s="2"/>
@@ -6248,7 +6265,7 @@
       <c r="Y138" s="2"/>
       <c r="Z138" s="2"/>
     </row>
-    <row r="139" spans="1:26" ht="13.5" customHeight="1">
+    <row r="139" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="2"/>
       <c r="B139" s="2"/>
       <c r="C139" s="2"/>
@@ -6276,7 +6293,7 @@
       <c r="Y139" s="2"/>
       <c r="Z139" s="2"/>
     </row>
-    <row r="140" spans="1:26" ht="13.5" customHeight="1">
+    <row r="140" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="2"/>
       <c r="B140" s="2"/>
       <c r="C140" s="2"/>
@@ -6304,7 +6321,7 @@
       <c r="Y140" s="2"/>
       <c r="Z140" s="2"/>
     </row>
-    <row r="141" spans="1:26" ht="13.5" customHeight="1">
+    <row r="141" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="2"/>
       <c r="B141" s="2"/>
       <c r="C141" s="2"/>
@@ -6332,7 +6349,7 @@
       <c r="Y141" s="2"/>
       <c r="Z141" s="2"/>
     </row>
-    <row r="142" spans="1:26" ht="13.5" customHeight="1">
+    <row r="142" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="2"/>
       <c r="B142" s="2"/>
       <c r="C142" s="2"/>
@@ -6360,7 +6377,7 @@
       <c r="Y142" s="2"/>
       <c r="Z142" s="2"/>
     </row>
-    <row r="143" spans="1:26" ht="13.5" customHeight="1">
+    <row r="143" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="2"/>
       <c r="B143" s="2"/>
       <c r="C143" s="2"/>
@@ -6388,7 +6405,7 @@
       <c r="Y143" s="2"/>
       <c r="Z143" s="2"/>
     </row>
-    <row r="144" spans="1:26" ht="13.5" customHeight="1">
+    <row r="144" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="2"/>
       <c r="B144" s="2"/>
       <c r="C144" s="2"/>
@@ -6416,7 +6433,7 @@
       <c r="Y144" s="2"/>
       <c r="Z144" s="2"/>
     </row>
-    <row r="145" spans="1:26" ht="13.5" customHeight="1">
+    <row r="145" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="2"/>
       <c r="B145" s="2"/>
       <c r="C145" s="2"/>
@@ -6444,7 +6461,7 @@
       <c r="Y145" s="2"/>
       <c r="Z145" s="2"/>
     </row>
-    <row r="146" spans="1:26" ht="13.5" customHeight="1">
+    <row r="146" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="2"/>
       <c r="B146" s="2"/>
       <c r="C146" s="2"/>
@@ -6472,7 +6489,7 @@
       <c r="Y146" s="2"/>
       <c r="Z146" s="2"/>
     </row>
-    <row r="147" spans="1:26" ht="13.5" customHeight="1">
+    <row r="147" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="2"/>
       <c r="B147" s="2"/>
       <c r="C147" s="2"/>
@@ -6500,7 +6517,7 @@
       <c r="Y147" s="2"/>
       <c r="Z147" s="2"/>
     </row>
-    <row r="148" spans="1:26" ht="13.5" customHeight="1">
+    <row r="148" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="2"/>
       <c r="B148" s="2"/>
       <c r="C148" s="2"/>
@@ -6528,7 +6545,7 @@
       <c r="Y148" s="2"/>
       <c r="Z148" s="2"/>
     </row>
-    <row r="149" spans="1:26" ht="13.5" customHeight="1">
+    <row r="149" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="2"/>
       <c r="B149" s="2"/>
       <c r="C149" s="2"/>
@@ -6556,7 +6573,7 @@
       <c r="Y149" s="2"/>
       <c r="Z149" s="2"/>
     </row>
-    <row r="150" spans="1:26" ht="13.5" customHeight="1">
+    <row r="150" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="2"/>
       <c r="B150" s="2"/>
       <c r="C150" s="2"/>
@@ -6584,7 +6601,7 @@
       <c r="Y150" s="2"/>
       <c r="Z150" s="2"/>
     </row>
-    <row r="151" spans="1:26" ht="13.5" customHeight="1">
+    <row r="151" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="2"/>
       <c r="B151" s="2"/>
       <c r="C151" s="2"/>
@@ -6612,7 +6629,7 @@
       <c r="Y151" s="2"/>
       <c r="Z151" s="2"/>
     </row>
-    <row r="152" spans="1:26" ht="13.5" customHeight="1">
+    <row r="152" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="2"/>
       <c r="B152" s="2"/>
       <c r="C152" s="2"/>
@@ -6640,7 +6657,7 @@
       <c r="Y152" s="2"/>
       <c r="Z152" s="2"/>
     </row>
-    <row r="153" spans="1:26" ht="13.5" customHeight="1">
+    <row r="153" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="2"/>
       <c r="B153" s="2"/>
       <c r="C153" s="2"/>
@@ -6668,7 +6685,7 @@
       <c r="Y153" s="2"/>
       <c r="Z153" s="2"/>
     </row>
-    <row r="154" spans="1:26" ht="13.5" customHeight="1">
+    <row r="154" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="2"/>
       <c r="B154" s="2"/>
       <c r="C154" s="2"/>
@@ -6696,7 +6713,7 @@
       <c r="Y154" s="2"/>
       <c r="Z154" s="2"/>
     </row>
-    <row r="155" spans="1:26" ht="13.5" customHeight="1">
+    <row r="155" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="2"/>
       <c r="B155" s="2"/>
       <c r="C155" s="2"/>
@@ -6724,7 +6741,7 @@
       <c r="Y155" s="2"/>
       <c r="Z155" s="2"/>
     </row>
-    <row r="156" spans="1:26" ht="13.5" customHeight="1">
+    <row r="156" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="2"/>
       <c r="B156" s="2"/>
       <c r="C156" s="2"/>
@@ -6752,7 +6769,7 @@
       <c r="Y156" s="2"/>
       <c r="Z156" s="2"/>
     </row>
-    <row r="157" spans="1:26" ht="13.5" customHeight="1">
+    <row r="157" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="2"/>
       <c r="B157" s="2"/>
       <c r="C157" s="2"/>
@@ -6780,7 +6797,7 @@
       <c r="Y157" s="2"/>
       <c r="Z157" s="2"/>
     </row>
-    <row r="158" spans="1:26" ht="13.5" customHeight="1">
+    <row r="158" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="2"/>
       <c r="B158" s="2"/>
       <c r="C158" s="2"/>
@@ -6808,7 +6825,7 @@
       <c r="Y158" s="2"/>
       <c r="Z158" s="2"/>
     </row>
-    <row r="159" spans="1:26" ht="13.5" customHeight="1">
+    <row r="159" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="2"/>
       <c r="B159" s="2"/>
       <c r="C159" s="2"/>
@@ -6836,7 +6853,7 @@
       <c r="Y159" s="2"/>
       <c r="Z159" s="2"/>
     </row>
-    <row r="160" spans="1:26" ht="13.5" customHeight="1">
+    <row r="160" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="2"/>
       <c r="B160" s="2"/>
       <c r="C160" s="2"/>
@@ -6864,7 +6881,7 @@
       <c r="Y160" s="2"/>
       <c r="Z160" s="2"/>
     </row>
-    <row r="161" spans="1:26" ht="13.5" customHeight="1">
+    <row r="161" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="2"/>
       <c r="B161" s="2"/>
       <c r="C161" s="2"/>
@@ -6892,7 +6909,7 @@
       <c r="Y161" s="2"/>
       <c r="Z161" s="2"/>
     </row>
-    <row r="162" spans="1:26" ht="13.5" customHeight="1">
+    <row r="162" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="2"/>
       <c r="B162" s="2"/>
       <c r="C162" s="2"/>
@@ -6920,7 +6937,7 @@
       <c r="Y162" s="2"/>
       <c r="Z162" s="2"/>
     </row>
-    <row r="163" spans="1:26" ht="13.5" customHeight="1">
+    <row r="163" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="2"/>
       <c r="B163" s="2"/>
       <c r="C163" s="2"/>
@@ -6948,7 +6965,7 @@
       <c r="Y163" s="2"/>
       <c r="Z163" s="2"/>
     </row>
-    <row r="164" spans="1:26" ht="13.5" customHeight="1">
+    <row r="164" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="2"/>
       <c r="B164" s="2"/>
       <c r="C164" s="2"/>
@@ -6976,7 +6993,7 @@
       <c r="Y164" s="2"/>
       <c r="Z164" s="2"/>
     </row>
-    <row r="165" spans="1:26" ht="13.5" customHeight="1">
+    <row r="165" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="2"/>
       <c r="B165" s="2"/>
       <c r="C165" s="2"/>
@@ -7004,7 +7021,7 @@
       <c r="Y165" s="2"/>
       <c r="Z165" s="2"/>
     </row>
-    <row r="166" spans="1:26" ht="13.5" customHeight="1">
+    <row r="166" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="2"/>
       <c r="B166" s="2"/>
       <c r="C166" s="2"/>
@@ -7032,7 +7049,7 @@
       <c r="Y166" s="2"/>
       <c r="Z166" s="2"/>
     </row>
-    <row r="167" spans="1:26" ht="13.5" customHeight="1">
+    <row r="167" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="2"/>
       <c r="B167" s="2"/>
       <c r="C167" s="2"/>
@@ -7060,7 +7077,7 @@
       <c r="Y167" s="2"/>
       <c r="Z167" s="2"/>
     </row>
-    <row r="168" spans="1:26" ht="13.5" customHeight="1">
+    <row r="168" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="2"/>
       <c r="B168" s="2"/>
       <c r="C168" s="2"/>
@@ -7088,7 +7105,7 @@
       <c r="Y168" s="2"/>
       <c r="Z168" s="2"/>
     </row>
-    <row r="169" spans="1:26" ht="13.5" customHeight="1">
+    <row r="169" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="2"/>
       <c r="B169" s="2"/>
       <c r="C169" s="2"/>
@@ -7116,7 +7133,7 @@
       <c r="Y169" s="2"/>
       <c r="Z169" s="2"/>
     </row>
-    <row r="170" spans="1:26" ht="13.5" customHeight="1">
+    <row r="170" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="2"/>
       <c r="B170" s="2"/>
       <c r="C170" s="2"/>
@@ -7144,7 +7161,7 @@
       <c r="Y170" s="2"/>
       <c r="Z170" s="2"/>
     </row>
-    <row r="171" spans="1:26" ht="13.5" customHeight="1">
+    <row r="171" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="2"/>
       <c r="B171" s="2"/>
       <c r="C171" s="2"/>
@@ -7172,7 +7189,7 @@
       <c r="Y171" s="2"/>
       <c r="Z171" s="2"/>
     </row>
-    <row r="172" spans="1:26" ht="13.5" customHeight="1">
+    <row r="172" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="2"/>
       <c r="B172" s="2"/>
       <c r="C172" s="2"/>
@@ -7200,7 +7217,7 @@
       <c r="Y172" s="2"/>
       <c r="Z172" s="2"/>
     </row>
-    <row r="173" spans="1:26" ht="13.5" customHeight="1">
+    <row r="173" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="2"/>
       <c r="B173" s="2"/>
       <c r="C173" s="2"/>
@@ -7228,7 +7245,7 @@
       <c r="Y173" s="2"/>
       <c r="Z173" s="2"/>
     </row>
-    <row r="174" spans="1:26" ht="13.5" customHeight="1">
+    <row r="174" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A174" s="2"/>
       <c r="B174" s="2"/>
       <c r="C174" s="2"/>
@@ -7256,7 +7273,7 @@
       <c r="Y174" s="2"/>
       <c r="Z174" s="2"/>
     </row>
-    <row r="175" spans="1:26" ht="13.5" customHeight="1">
+    <row r="175" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="2"/>
       <c r="B175" s="2"/>
       <c r="C175" s="2"/>
@@ -7284,7 +7301,7 @@
       <c r="Y175" s="2"/>
       <c r="Z175" s="2"/>
     </row>
-    <row r="176" spans="1:26" ht="13.5" customHeight="1">
+    <row r="176" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="2"/>
       <c r="B176" s="2"/>
       <c r="C176" s="2"/>
@@ -7312,7 +7329,7 @@
       <c r="Y176" s="2"/>
       <c r="Z176" s="2"/>
     </row>
-    <row r="177" spans="1:26" ht="13.5" customHeight="1">
+    <row r="177" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="2"/>
       <c r="B177" s="2"/>
       <c r="C177" s="2"/>
@@ -7340,7 +7357,7 @@
       <c r="Y177" s="2"/>
       <c r="Z177" s="2"/>
     </row>
-    <row r="178" spans="1:26" ht="13.5" customHeight="1">
+    <row r="178" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="2"/>
       <c r="B178" s="2"/>
       <c r="C178" s="2"/>
@@ -7368,7 +7385,7 @@
       <c r="Y178" s="2"/>
       <c r="Z178" s="2"/>
     </row>
-    <row r="179" spans="1:26" ht="13.5" customHeight="1">
+    <row r="179" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="2"/>
       <c r="B179" s="2"/>
       <c r="C179" s="2"/>
@@ -7396,7 +7413,7 @@
       <c r="Y179" s="2"/>
       <c r="Z179" s="2"/>
     </row>
-    <row r="180" spans="1:26" ht="13.5" customHeight="1">
+    <row r="180" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="2"/>
       <c r="B180" s="2"/>
       <c r="C180" s="2"/>
@@ -7424,7 +7441,7 @@
       <c r="Y180" s="2"/>
       <c r="Z180" s="2"/>
     </row>
-    <row r="181" spans="1:26" ht="13.5" customHeight="1">
+    <row r="181" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="2"/>
       <c r="B181" s="2"/>
       <c r="C181" s="2"/>
@@ -7452,7 +7469,7 @@
       <c r="Y181" s="2"/>
       <c r="Z181" s="2"/>
     </row>
-    <row r="182" spans="1:26" ht="13.5" customHeight="1">
+    <row r="182" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="2"/>
       <c r="B182" s="2"/>
       <c r="C182" s="2"/>
@@ -7480,7 +7497,7 @@
       <c r="Y182" s="2"/>
       <c r="Z182" s="2"/>
     </row>
-    <row r="183" spans="1:26" ht="13.5" customHeight="1">
+    <row r="183" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="2"/>
       <c r="B183" s="2"/>
       <c r="C183" s="2"/>
@@ -7508,7 +7525,7 @@
       <c r="Y183" s="2"/>
       <c r="Z183" s="2"/>
     </row>
-    <row r="184" spans="1:26" ht="13.5" customHeight="1">
+    <row r="184" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A184" s="2"/>
       <c r="B184" s="2"/>
       <c r="C184" s="2"/>
@@ -7536,7 +7553,7 @@
       <c r="Y184" s="2"/>
       <c r="Z184" s="2"/>
     </row>
-    <row r="185" spans="1:26" ht="13.5" customHeight="1">
+    <row r="185" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A185" s="2"/>
       <c r="B185" s="2"/>
       <c r="C185" s="2"/>
@@ -7564,7 +7581,7 @@
       <c r="Y185" s="2"/>
       <c r="Z185" s="2"/>
     </row>
-    <row r="186" spans="1:26" ht="13.5" customHeight="1">
+    <row r="186" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A186" s="2"/>
       <c r="B186" s="2"/>
       <c r="C186" s="2"/>
@@ -7592,7 +7609,7 @@
       <c r="Y186" s="2"/>
       <c r="Z186" s="2"/>
     </row>
-    <row r="187" spans="1:26" ht="13.5" customHeight="1">
+    <row r="187" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="2"/>
       <c r="B187" s="2"/>
       <c r="C187" s="2"/>
@@ -7620,7 +7637,7 @@
       <c r="Y187" s="2"/>
       <c r="Z187" s="2"/>
     </row>
-    <row r="188" spans="1:26" ht="13.5" customHeight="1">
+    <row r="188" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A188" s="2"/>
       <c r="B188" s="2"/>
       <c r="C188" s="2"/>
@@ -7648,7 +7665,7 @@
       <c r="Y188" s="2"/>
       <c r="Z188" s="2"/>
     </row>
-    <row r="189" spans="1:26" ht="13.5" customHeight="1">
+    <row r="189" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A189" s="2"/>
       <c r="B189" s="2"/>
       <c r="C189" s="2"/>
@@ -7676,7 +7693,7 @@
       <c r="Y189" s="2"/>
       <c r="Z189" s="2"/>
     </row>
-    <row r="190" spans="1:26" ht="13.5" customHeight="1">
+    <row r="190" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A190" s="2"/>
       <c r="B190" s="2"/>
       <c r="C190" s="2"/>
@@ -7704,7 +7721,7 @@
       <c r="Y190" s="2"/>
       <c r="Z190" s="2"/>
     </row>
-    <row r="191" spans="1:26" ht="13.5" customHeight="1">
+    <row r="191" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A191" s="2"/>
       <c r="B191" s="2"/>
       <c r="C191" s="2"/>
@@ -7732,7 +7749,7 @@
       <c r="Y191" s="2"/>
       <c r="Z191" s="2"/>
     </row>
-    <row r="192" spans="1:26" ht="13.5" customHeight="1">
+    <row r="192" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="2"/>
       <c r="B192" s="2"/>
       <c r="C192" s="2"/>
@@ -7760,7 +7777,7 @@
       <c r="Y192" s="2"/>
       <c r="Z192" s="2"/>
     </row>
-    <row r="193" spans="1:26" ht="13.5" customHeight="1">
+    <row r="193" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="2"/>
       <c r="B193" s="2"/>
       <c r="C193" s="2"/>
@@ -7788,7 +7805,7 @@
       <c r="Y193" s="2"/>
       <c r="Z193" s="2"/>
     </row>
-    <row r="194" spans="1:26" ht="13.5" customHeight="1">
+    <row r="194" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A194" s="2"/>
       <c r="B194" s="2"/>
       <c r="C194" s="2"/>
@@ -7816,7 +7833,7 @@
       <c r="Y194" s="2"/>
       <c r="Z194" s="2"/>
     </row>
-    <row r="195" spans="1:26" ht="13.5" customHeight="1">
+    <row r="195" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A195" s="2"/>
       <c r="B195" s="2"/>
       <c r="C195" s="2"/>
@@ -7844,7 +7861,7 @@
       <c r="Y195" s="2"/>
       <c r="Z195" s="2"/>
     </row>
-    <row r="196" spans="1:26" ht="13.5" customHeight="1">
+    <row r="196" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A196" s="2"/>
       <c r="B196" s="2"/>
       <c r="C196" s="2"/>
@@ -7872,7 +7889,7 @@
       <c r="Y196" s="2"/>
       <c r="Z196" s="2"/>
     </row>
-    <row r="197" spans="1:26" ht="13.5" customHeight="1">
+    <row r="197" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="2"/>
       <c r="B197" s="2"/>
       <c r="C197" s="2"/>
@@ -7900,7 +7917,7 @@
       <c r="Y197" s="2"/>
       <c r="Z197" s="2"/>
     </row>
-    <row r="198" spans="1:26" ht="13.5" customHeight="1">
+    <row r="198" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A198" s="2"/>
       <c r="B198" s="2"/>
       <c r="C198" s="2"/>
@@ -7928,7 +7945,7 @@
       <c r="Y198" s="2"/>
       <c r="Z198" s="2"/>
     </row>
-    <row r="199" spans="1:26" ht="13.5" customHeight="1">
+    <row r="199" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="2"/>
       <c r="B199" s="2"/>
       <c r="C199" s="2"/>
@@ -7956,7 +7973,7 @@
       <c r="Y199" s="2"/>
       <c r="Z199" s="2"/>
     </row>
-    <row r="200" spans="1:26" ht="13.5" customHeight="1">
+    <row r="200" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A200" s="2"/>
       <c r="B200" s="2"/>
       <c r="C200" s="2"/>
@@ -7984,7 +8001,7 @@
       <c r="Y200" s="2"/>
       <c r="Z200" s="2"/>
     </row>
-    <row r="201" spans="1:26" ht="13.5" customHeight="1">
+    <row r="201" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A201" s="2"/>
       <c r="B201" s="2"/>
       <c r="C201" s="2"/>
@@ -8012,7 +8029,7 @@
       <c r="Y201" s="2"/>
       <c r="Z201" s="2"/>
     </row>
-    <row r="202" spans="1:26" ht="13.5" customHeight="1">
+    <row r="202" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A202" s="2"/>
       <c r="B202" s="2"/>
       <c r="C202" s="2"/>
@@ -8040,7 +8057,7 @@
       <c r="Y202" s="2"/>
       <c r="Z202" s="2"/>
     </row>
-    <row r="203" spans="1:26" ht="13.5" customHeight="1">
+    <row r="203" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A203" s="2"/>
       <c r="B203" s="2"/>
       <c r="C203" s="2"/>
@@ -8068,7 +8085,7 @@
       <c r="Y203" s="2"/>
       <c r="Z203" s="2"/>
     </row>
-    <row r="204" spans="1:26" ht="13.5" customHeight="1">
+    <row r="204" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A204" s="2"/>
       <c r="B204" s="2"/>
       <c r="C204" s="2"/>
@@ -8096,7 +8113,7 @@
       <c r="Y204" s="2"/>
       <c r="Z204" s="2"/>
     </row>
-    <row r="205" spans="1:26" ht="13.5" customHeight="1">
+    <row r="205" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A205" s="2"/>
       <c r="B205" s="2"/>
       <c r="C205" s="2"/>
@@ -8124,7 +8141,7 @@
       <c r="Y205" s="2"/>
       <c r="Z205" s="2"/>
     </row>
-    <row r="206" spans="1:26" ht="13.5" customHeight="1">
+    <row r="206" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A206" s="2"/>
       <c r="B206" s="2"/>
       <c r="C206" s="2"/>
@@ -8152,7 +8169,7 @@
       <c r="Y206" s="2"/>
       <c r="Z206" s="2"/>
     </row>
-    <row r="207" spans="1:26" ht="13.5" customHeight="1">
+    <row r="207" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A207" s="2"/>
       <c r="B207" s="2"/>
       <c r="C207" s="2"/>
@@ -8180,7 +8197,7 @@
       <c r="Y207" s="2"/>
       <c r="Z207" s="2"/>
     </row>
-    <row r="208" spans="1:26" ht="13.5" customHeight="1">
+    <row r="208" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A208" s="2"/>
       <c r="B208" s="2"/>
       <c r="C208" s="2"/>
@@ -8208,7 +8225,7 @@
       <c r="Y208" s="2"/>
       <c r="Z208" s="2"/>
     </row>
-    <row r="209" spans="1:26" ht="13.5" customHeight="1">
+    <row r="209" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A209" s="2"/>
       <c r="B209" s="2"/>
       <c r="C209" s="2"/>
@@ -8236,7 +8253,7 @@
       <c r="Y209" s="2"/>
       <c r="Z209" s="2"/>
     </row>
-    <row r="210" spans="1:26" ht="13.5" customHeight="1">
+    <row r="210" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A210" s="2"/>
       <c r="B210" s="2"/>
       <c r="C210" s="2"/>
@@ -8264,7 +8281,7 @@
       <c r="Y210" s="2"/>
       <c r="Z210" s="2"/>
     </row>
-    <row r="211" spans="1:26" ht="13.5" customHeight="1">
+    <row r="211" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A211" s="2"/>
       <c r="B211" s="2"/>
       <c r="C211" s="2"/>
@@ -8292,7 +8309,7 @@
       <c r="Y211" s="2"/>
       <c r="Z211" s="2"/>
     </row>
-    <row r="212" spans="1:26" ht="13.5" customHeight="1">
+    <row r="212" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A212" s="2"/>
       <c r="B212" s="2"/>
       <c r="C212" s="2"/>
@@ -8320,7 +8337,7 @@
       <c r="Y212" s="2"/>
       <c r="Z212" s="2"/>
     </row>
-    <row r="213" spans="1:26" ht="13.5" customHeight="1">
+    <row r="213" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A213" s="2"/>
       <c r="B213" s="2"/>
       <c r="C213" s="2"/>
@@ -8348,7 +8365,7 @@
       <c r="Y213" s="2"/>
       <c r="Z213" s="2"/>
     </row>
-    <row r="214" spans="1:26" ht="13.5" customHeight="1">
+    <row r="214" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A214" s="2"/>
       <c r="B214" s="2"/>
       <c r="C214" s="2"/>
@@ -8376,7 +8393,7 @@
       <c r="Y214" s="2"/>
       <c r="Z214" s="2"/>
     </row>
-    <row r="215" spans="1:26" ht="13.5" customHeight="1">
+    <row r="215" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A215" s="2"/>
       <c r="B215" s="2"/>
       <c r="C215" s="2"/>
@@ -8404,7 +8421,7 @@
       <c r="Y215" s="2"/>
       <c r="Z215" s="2"/>
     </row>
-    <row r="216" spans="1:26" ht="13.5" customHeight="1">
+    <row r="216" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A216" s="2"/>
       <c r="B216" s="2"/>
       <c r="C216" s="2"/>
@@ -8432,7 +8449,7 @@
       <c r="Y216" s="2"/>
       <c r="Z216" s="2"/>
     </row>
-    <row r="217" spans="1:26" ht="13.5" customHeight="1">
+    <row r="217" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A217" s="2"/>
       <c r="B217" s="2"/>
       <c r="C217" s="2"/>
@@ -8460,7 +8477,7 @@
       <c r="Y217" s="2"/>
       <c r="Z217" s="2"/>
     </row>
-    <row r="218" spans="1:26" ht="13.5" customHeight="1">
+    <row r="218" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A218" s="2"/>
       <c r="B218" s="2"/>
       <c r="C218" s="2"/>
@@ -8488,7 +8505,7 @@
       <c r="Y218" s="2"/>
       <c r="Z218" s="2"/>
     </row>
-    <row r="219" spans="1:26" ht="13.5" customHeight="1">
+    <row r="219" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A219" s="2"/>
       <c r="B219" s="2"/>
       <c r="C219" s="2"/>
@@ -8516,7 +8533,7 @@
       <c r="Y219" s="2"/>
       <c r="Z219" s="2"/>
     </row>
-    <row r="220" spans="1:26" ht="13.5" customHeight="1">
+    <row r="220" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A220" s="2"/>
       <c r="B220" s="2"/>
       <c r="C220" s="2"/>
@@ -8544,7 +8561,7 @@
       <c r="Y220" s="2"/>
       <c r="Z220" s="2"/>
     </row>
-    <row r="221" spans="1:26" ht="13.5" customHeight="1">
+    <row r="221" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A221" s="2"/>
       <c r="B221" s="2"/>
       <c r="C221" s="2"/>
@@ -8572,7 +8589,7 @@
       <c r="Y221" s="2"/>
       <c r="Z221" s="2"/>
     </row>
-    <row r="222" spans="1:26" ht="13.5" customHeight="1">
+    <row r="222" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A222" s="2"/>
       <c r="B222" s="2"/>
       <c r="C222" s="2"/>
@@ -8600,7 +8617,7 @@
       <c r="Y222" s="2"/>
       <c r="Z222" s="2"/>
     </row>
-    <row r="223" spans="1:26" ht="13.5" customHeight="1">
+    <row r="223" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A223" s="2"/>
       <c r="B223" s="2"/>
       <c r="C223" s="2"/>
@@ -8628,7 +8645,7 @@
       <c r="Y223" s="2"/>
       <c r="Z223" s="2"/>
     </row>
-    <row r="224" spans="1:26" ht="13.5" customHeight="1">
+    <row r="224" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A224" s="2"/>
       <c r="B224" s="2"/>
       <c r="C224" s="2"/>
@@ -8656,7 +8673,7 @@
       <c r="Y224" s="2"/>
       <c r="Z224" s="2"/>
     </row>
-    <row r="225" spans="1:26" ht="13.5" customHeight="1">
+    <row r="225" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A225" s="2"/>
       <c r="B225" s="2"/>
       <c r="C225" s="2"/>
@@ -8684,7 +8701,7 @@
       <c r="Y225" s="2"/>
       <c r="Z225" s="2"/>
     </row>
-    <row r="226" spans="1:26" ht="13.5" customHeight="1">
+    <row r="226" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A226" s="2"/>
       <c r="B226" s="2"/>
       <c r="C226" s="2"/>
@@ -8712,7 +8729,7 @@
       <c r="Y226" s="2"/>
       <c r="Z226" s="2"/>
     </row>
-    <row r="227" spans="1:26" ht="13.5" customHeight="1">
+    <row r="227" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A227" s="2"/>
       <c r="B227" s="2"/>
       <c r="C227" s="2"/>
@@ -8740,7 +8757,7 @@
       <c r="Y227" s="2"/>
       <c r="Z227" s="2"/>
     </row>
-    <row r="228" spans="1:26" ht="13.5" customHeight="1">
+    <row r="228" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A228" s="2"/>
       <c r="B228" s="2"/>
       <c r="C228" s="2"/>
@@ -8768,799 +8785,789 @@
       <c r="Y228" s="2"/>
       <c r="Z228" s="2"/>
     </row>
-    <row r="229" spans="1:26" ht="15.75" customHeight="1"/>
-    <row r="230" spans="1:26" ht="15.75" customHeight="1"/>
-    <row r="231" spans="1:26" ht="15.75" customHeight="1"/>
-    <row r="232" spans="1:26" ht="15.75" customHeight="1"/>
-    <row r="233" spans="1:26" ht="15.75" customHeight="1"/>
-    <row r="234" spans="1:26" ht="15.75" customHeight="1"/>
-    <row r="235" spans="1:26" ht="15.75" customHeight="1"/>
-    <row r="236" spans="1:26" ht="15.75" customHeight="1"/>
-    <row r="237" spans="1:26" ht="15.75" customHeight="1"/>
-    <row r="238" spans="1:26" ht="15.75" customHeight="1"/>
-    <row r="239" spans="1:26" ht="15.75" customHeight="1"/>
-    <row r="240" spans="1:26" ht="15.75" customHeight="1"/>
-    <row r="241" ht="15.75" customHeight="1"/>
-    <row r="242" ht="15.75" customHeight="1"/>
-    <row r="243" ht="15.75" customHeight="1"/>
-    <row r="244" ht="15.75" customHeight="1"/>
-    <row r="245" ht="15.75" customHeight="1"/>
-    <row r="246" ht="15.75" customHeight="1"/>
-    <row r="247" ht="15.75" customHeight="1"/>
-    <row r="248" ht="15.75" customHeight="1"/>
-    <row r="249" ht="15.75" customHeight="1"/>
-    <row r="250" ht="15.75" customHeight="1"/>
-    <row r="251" ht="15.75" customHeight="1"/>
-    <row r="252" ht="15.75" customHeight="1"/>
-    <row r="253" ht="15.75" customHeight="1"/>
-    <row r="254" ht="15.75" customHeight="1"/>
-    <row r="255" ht="15.75" customHeight="1"/>
-    <row r="256" ht="15.75" customHeight="1"/>
-    <row r="257" ht="15.75" customHeight="1"/>
-    <row r="258" ht="15.75" customHeight="1"/>
-    <row r="259" ht="15.75" customHeight="1"/>
-    <row r="260" ht="15.75" customHeight="1"/>
-    <row r="261" ht="15.75" customHeight="1"/>
-    <row r="262" ht="15.75" customHeight="1"/>
-    <row r="263" ht="15.75" customHeight="1"/>
-    <row r="264" ht="15.75" customHeight="1"/>
-    <row r="265" ht="15.75" customHeight="1"/>
-    <row r="266" ht="15.75" customHeight="1"/>
-    <row r="267" ht="15.75" customHeight="1"/>
-    <row r="268" ht="15.75" customHeight="1"/>
-    <row r="269" ht="15.75" customHeight="1"/>
-    <row r="270" ht="15.75" customHeight="1"/>
-    <row r="271" ht="15.75" customHeight="1"/>
-    <row r="272" ht="15.75" customHeight="1"/>
-    <row r="273" ht="15.75" customHeight="1"/>
-    <row r="274" ht="15.75" customHeight="1"/>
-    <row r="275" ht="15.75" customHeight="1"/>
-    <row r="276" ht="15.75" customHeight="1"/>
-    <row r="277" ht="15.75" customHeight="1"/>
-    <row r="278" ht="15.75" customHeight="1"/>
-    <row r="279" ht="15.75" customHeight="1"/>
-    <row r="280" ht="15.75" customHeight="1"/>
-    <row r="281" ht="15.75" customHeight="1"/>
-    <row r="282" ht="15.75" customHeight="1"/>
-    <row r="283" ht="15.75" customHeight="1"/>
-    <row r="284" ht="15.75" customHeight="1"/>
-    <row r="285" ht="15.75" customHeight="1"/>
-    <row r="286" ht="15.75" customHeight="1"/>
-    <row r="287" ht="15.75" customHeight="1"/>
-    <row r="288" ht="15.75" customHeight="1"/>
-    <row r="289" ht="15.75" customHeight="1"/>
-    <row r="290" ht="15.75" customHeight="1"/>
-    <row r="291" ht="15.75" customHeight="1"/>
-    <row r="292" ht="15.75" customHeight="1"/>
-    <row r="293" ht="15.75" customHeight="1"/>
-    <row r="294" ht="15.75" customHeight="1"/>
-    <row r="295" ht="15.75" customHeight="1"/>
-    <row r="296" ht="15.75" customHeight="1"/>
-    <row r="297" ht="15.75" customHeight="1"/>
-    <row r="298" ht="15.75" customHeight="1"/>
-    <row r="299" ht="15.75" customHeight="1"/>
-    <row r="300" ht="15.75" customHeight="1"/>
-    <row r="301" ht="15.75" customHeight="1"/>
-    <row r="302" ht="15.75" customHeight="1"/>
-    <row r="303" ht="15.75" customHeight="1"/>
-    <row r="304" ht="15.75" customHeight="1"/>
-    <row r="305" ht="15.75" customHeight="1"/>
-    <row r="306" ht="15.75" customHeight="1"/>
-    <row r="307" ht="15.75" customHeight="1"/>
-    <row r="308" ht="15.75" customHeight="1"/>
-    <row r="309" ht="15.75" customHeight="1"/>
-    <row r="310" ht="15.75" customHeight="1"/>
-    <row r="311" ht="15.75" customHeight="1"/>
-    <row r="312" ht="15.75" customHeight="1"/>
-    <row r="313" ht="15.75" customHeight="1"/>
-    <row r="314" ht="15.75" customHeight="1"/>
-    <row r="315" ht="15.75" customHeight="1"/>
-    <row r="316" ht="15.75" customHeight="1"/>
-    <row r="317" ht="15.75" customHeight="1"/>
-    <row r="318" ht="15.75" customHeight="1"/>
-    <row r="319" ht="15.75" customHeight="1"/>
-    <row r="320" ht="15.75" customHeight="1"/>
-    <row r="321" ht="15.75" customHeight="1"/>
-    <row r="322" ht="15.75" customHeight="1"/>
-    <row r="323" ht="15.75" customHeight="1"/>
-    <row r="324" ht="15.75" customHeight="1"/>
-    <row r="325" ht="15.75" customHeight="1"/>
-    <row r="326" ht="15.75" customHeight="1"/>
-    <row r="327" ht="15.75" customHeight="1"/>
-    <row r="328" ht="15.75" customHeight="1"/>
-    <row r="329" ht="15.75" customHeight="1"/>
-    <row r="330" ht="15.75" customHeight="1"/>
-    <row r="331" ht="15.75" customHeight="1"/>
-    <row r="332" ht="15.75" customHeight="1"/>
-    <row r="333" ht="15.75" customHeight="1"/>
-    <row r="334" ht="15.75" customHeight="1"/>
-    <row r="335" ht="15.75" customHeight="1"/>
-    <row r="336" ht="15.75" customHeight="1"/>
-    <row r="337" ht="15.75" customHeight="1"/>
-    <row r="338" ht="15.75" customHeight="1"/>
-    <row r="339" ht="15.75" customHeight="1"/>
-    <row r="340" ht="15.75" customHeight="1"/>
-    <row r="341" ht="15.75" customHeight="1"/>
-    <row r="342" ht="15.75" customHeight="1"/>
-    <row r="343" ht="15.75" customHeight="1"/>
-    <row r="344" ht="15.75" customHeight="1"/>
-    <row r="345" ht="15.75" customHeight="1"/>
-    <row r="346" ht="15.75" customHeight="1"/>
-    <row r="347" ht="15.75" customHeight="1"/>
-    <row r="348" ht="15.75" customHeight="1"/>
-    <row r="349" ht="15.75" customHeight="1"/>
-    <row r="350" ht="15.75" customHeight="1"/>
-    <row r="351" ht="15.75" customHeight="1"/>
-    <row r="352" ht="15.75" customHeight="1"/>
-    <row r="353" ht="15.75" customHeight="1"/>
-    <row r="354" ht="15.75" customHeight="1"/>
-    <row r="355" ht="15.75" customHeight="1"/>
-    <row r="356" ht="15.75" customHeight="1"/>
-    <row r="357" ht="15.75" customHeight="1"/>
-    <row r="358" ht="15.75" customHeight="1"/>
-    <row r="359" ht="15.75" customHeight="1"/>
-    <row r="360" ht="15.75" customHeight="1"/>
-    <row r="361" ht="15.75" customHeight="1"/>
-    <row r="362" ht="15.75" customHeight="1"/>
-    <row r="363" ht="15.75" customHeight="1"/>
-    <row r="364" ht="15.75" customHeight="1"/>
-    <row r="365" ht="15.75" customHeight="1"/>
-    <row r="366" ht="15.75" customHeight="1"/>
-    <row r="367" ht="15.75" customHeight="1"/>
-    <row r="368" ht="15.75" customHeight="1"/>
-    <row r="369" ht="15.75" customHeight="1"/>
-    <row r="370" ht="15.75" customHeight="1"/>
-    <row r="371" ht="15.75" customHeight="1"/>
-    <row r="372" ht="15.75" customHeight="1"/>
-    <row r="373" ht="15.75" customHeight="1"/>
-    <row r="374" ht="15.75" customHeight="1"/>
-    <row r="375" ht="15.75" customHeight="1"/>
-    <row r="376" ht="15.75" customHeight="1"/>
-    <row r="377" ht="15.75" customHeight="1"/>
-    <row r="378" ht="15.75" customHeight="1"/>
-    <row r="379" ht="15.75" customHeight="1"/>
-    <row r="380" ht="15.75" customHeight="1"/>
-    <row r="381" ht="15.75" customHeight="1"/>
-    <row r="382" ht="15.75" customHeight="1"/>
-    <row r="383" ht="15.75" customHeight="1"/>
-    <row r="384" ht="15.75" customHeight="1"/>
-    <row r="385" ht="15.75" customHeight="1"/>
-    <row r="386" ht="15.75" customHeight="1"/>
-    <row r="387" ht="15.75" customHeight="1"/>
-    <row r="388" ht="15.75" customHeight="1"/>
-    <row r="389" ht="15.75" customHeight="1"/>
-    <row r="390" ht="15.75" customHeight="1"/>
-    <row r="391" ht="15.75" customHeight="1"/>
-    <row r="392" ht="15.75" customHeight="1"/>
-    <row r="393" ht="15.75" customHeight="1"/>
-    <row r="394" ht="15.75" customHeight="1"/>
-    <row r="395" ht="15.75" customHeight="1"/>
-    <row r="396" ht="15.75" customHeight="1"/>
-    <row r="397" ht="15.75" customHeight="1"/>
-    <row r="398" ht="15.75" customHeight="1"/>
-    <row r="399" ht="15.75" customHeight="1"/>
-    <row r="400" ht="15.75" customHeight="1"/>
-    <row r="401" ht="15.75" customHeight="1"/>
-    <row r="402" ht="15.75" customHeight="1"/>
-    <row r="403" ht="15.75" customHeight="1"/>
-    <row r="404" ht="15.75" customHeight="1"/>
-    <row r="405" ht="15.75" customHeight="1"/>
-    <row r="406" ht="15.75" customHeight="1"/>
-    <row r="407" ht="15.75" customHeight="1"/>
-    <row r="408" ht="15.75" customHeight="1"/>
-    <row r="409" ht="15.75" customHeight="1"/>
-    <row r="410" ht="15.75" customHeight="1"/>
-    <row r="411" ht="15.75" customHeight="1"/>
-    <row r="412" ht="15.75" customHeight="1"/>
-    <row r="413" ht="15.75" customHeight="1"/>
-    <row r="414" ht="15.75" customHeight="1"/>
-    <row r="415" ht="15.75" customHeight="1"/>
-    <row r="416" ht="15.75" customHeight="1"/>
-    <row r="417" ht="15.75" customHeight="1"/>
-    <row r="418" ht="15.75" customHeight="1"/>
-    <row r="419" ht="15.75" customHeight="1"/>
-    <row r="420" ht="15.75" customHeight="1"/>
-    <row r="421" ht="15.75" customHeight="1"/>
-    <row r="422" ht="15.75" customHeight="1"/>
-    <row r="423" ht="15.75" customHeight="1"/>
-    <row r="424" ht="15.75" customHeight="1"/>
-    <row r="425" ht="15.75" customHeight="1"/>
-    <row r="426" ht="15.75" customHeight="1"/>
-    <row r="427" ht="15.75" customHeight="1"/>
-    <row r="428" ht="15.75" customHeight="1"/>
-    <row r="429" ht="15.75" customHeight="1"/>
-    <row r="430" ht="15.75" customHeight="1"/>
-    <row r="431" ht="15.75" customHeight="1"/>
-    <row r="432" ht="15.75" customHeight="1"/>
-    <row r="433" ht="15.75" customHeight="1"/>
-    <row r="434" ht="15.75" customHeight="1"/>
-    <row r="435" ht="15.75" customHeight="1"/>
-    <row r="436" ht="15.75" customHeight="1"/>
-    <row r="437" ht="15.75" customHeight="1"/>
-    <row r="438" ht="15.75" customHeight="1"/>
-    <row r="439" ht="15.75" customHeight="1"/>
-    <row r="440" ht="15.75" customHeight="1"/>
-    <row r="441" ht="15.75" customHeight="1"/>
-    <row r="442" ht="15.75" customHeight="1"/>
-    <row r="443" ht="15.75" customHeight="1"/>
-    <row r="444" ht="15.75" customHeight="1"/>
-    <row r="445" ht="15.75" customHeight="1"/>
-    <row r="446" ht="15.75" customHeight="1"/>
-    <row r="447" ht="15.75" customHeight="1"/>
-    <row r="448" ht="15.75" customHeight="1"/>
-    <row r="449" ht="15.75" customHeight="1"/>
-    <row r="450" ht="15.75" customHeight="1"/>
-    <row r="451" ht="15.75" customHeight="1"/>
-    <row r="452" ht="15.75" customHeight="1"/>
-    <row r="453" ht="15.75" customHeight="1"/>
-    <row r="454" ht="15.75" customHeight="1"/>
-    <row r="455" ht="15.75" customHeight="1"/>
-    <row r="456" ht="15.75" customHeight="1"/>
-    <row r="457" ht="15.75" customHeight="1"/>
-    <row r="458" ht="15.75" customHeight="1"/>
-    <row r="459" ht="15.75" customHeight="1"/>
-    <row r="460" ht="15.75" customHeight="1"/>
-    <row r="461" ht="15.75" customHeight="1"/>
-    <row r="462" ht="15.75" customHeight="1"/>
-    <row r="463" ht="15.75" customHeight="1"/>
-    <row r="464" ht="15.75" customHeight="1"/>
-    <row r="465" ht="15.75" customHeight="1"/>
-    <row r="466" ht="15.75" customHeight="1"/>
-    <row r="467" ht="15.75" customHeight="1"/>
-    <row r="468" ht="15.75" customHeight="1"/>
-    <row r="469" ht="15.75" customHeight="1"/>
-    <row r="470" ht="15.75" customHeight="1"/>
-    <row r="471" ht="15.75" customHeight="1"/>
-    <row r="472" ht="15.75" customHeight="1"/>
-    <row r="473" ht="15.75" customHeight="1"/>
-    <row r="474" ht="15.75" customHeight="1"/>
-    <row r="475" ht="15.75" customHeight="1"/>
-    <row r="476" ht="15.75" customHeight="1"/>
-    <row r="477" ht="15.75" customHeight="1"/>
-    <row r="478" ht="15.75" customHeight="1"/>
-    <row r="479" ht="15.75" customHeight="1"/>
-    <row r="480" ht="15.75" customHeight="1"/>
-    <row r="481" ht="15.75" customHeight="1"/>
-    <row r="482" ht="15.75" customHeight="1"/>
-    <row r="483" ht="15.75" customHeight="1"/>
-    <row r="484" ht="15.75" customHeight="1"/>
-    <row r="485" ht="15.75" customHeight="1"/>
-    <row r="486" ht="15.75" customHeight="1"/>
-    <row r="487" ht="15.75" customHeight="1"/>
-    <row r="488" ht="15.75" customHeight="1"/>
-    <row r="489" ht="15.75" customHeight="1"/>
-    <row r="490" ht="15.75" customHeight="1"/>
-    <row r="491" ht="15.75" customHeight="1"/>
-    <row r="492" ht="15.75" customHeight="1"/>
-    <row r="493" ht="15.75" customHeight="1"/>
-    <row r="494" ht="15.75" customHeight="1"/>
-    <row r="495" ht="15.75" customHeight="1"/>
-    <row r="496" ht="15.75" customHeight="1"/>
-    <row r="497" ht="15.75" customHeight="1"/>
-    <row r="498" ht="15.75" customHeight="1"/>
-    <row r="499" ht="15.75" customHeight="1"/>
-    <row r="500" ht="15.75" customHeight="1"/>
-    <row r="501" ht="15.75" customHeight="1"/>
-    <row r="502" ht="15.75" customHeight="1"/>
-    <row r="503" ht="15.75" customHeight="1"/>
-    <row r="504" ht="15.75" customHeight="1"/>
-    <row r="505" ht="15.75" customHeight="1"/>
-    <row r="506" ht="15.75" customHeight="1"/>
-    <row r="507" ht="15.75" customHeight="1"/>
-    <row r="508" ht="15.75" customHeight="1"/>
-    <row r="509" ht="15.75" customHeight="1"/>
-    <row r="510" ht="15.75" customHeight="1"/>
-    <row r="511" ht="15.75" customHeight="1"/>
-    <row r="512" ht="15.75" customHeight="1"/>
-    <row r="513" ht="15.75" customHeight="1"/>
-    <row r="514" ht="15.75" customHeight="1"/>
-    <row r="515" ht="15.75" customHeight="1"/>
-    <row r="516" ht="15.75" customHeight="1"/>
-    <row r="517" ht="15.75" customHeight="1"/>
-    <row r="518" ht="15.75" customHeight="1"/>
-    <row r="519" ht="15.75" customHeight="1"/>
-    <row r="520" ht="15.75" customHeight="1"/>
-    <row r="521" ht="15.75" customHeight="1"/>
-    <row r="522" ht="15.75" customHeight="1"/>
-    <row r="523" ht="15.75" customHeight="1"/>
-    <row r="524" ht="15.75" customHeight="1"/>
-    <row r="525" ht="15.75" customHeight="1"/>
-    <row r="526" ht="15.75" customHeight="1"/>
-    <row r="527" ht="15.75" customHeight="1"/>
-    <row r="528" ht="15.75" customHeight="1"/>
-    <row r="529" ht="15.75" customHeight="1"/>
-    <row r="530" ht="15.75" customHeight="1"/>
-    <row r="531" ht="15.75" customHeight="1"/>
-    <row r="532" ht="15.75" customHeight="1"/>
-    <row r="533" ht="15.75" customHeight="1"/>
-    <row r="534" ht="15.75" customHeight="1"/>
-    <row r="535" ht="15.75" customHeight="1"/>
-    <row r="536" ht="15.75" customHeight="1"/>
-    <row r="537" ht="15.75" customHeight="1"/>
-    <row r="538" ht="15.75" customHeight="1"/>
-    <row r="539" ht="15.75" customHeight="1"/>
-    <row r="540" ht="15.75" customHeight="1"/>
-    <row r="541" ht="15.75" customHeight="1"/>
-    <row r="542" ht="15.75" customHeight="1"/>
-    <row r="543" ht="15.75" customHeight="1"/>
-    <row r="544" ht="15.75" customHeight="1"/>
-    <row r="545" ht="15.75" customHeight="1"/>
-    <row r="546" ht="15.75" customHeight="1"/>
-    <row r="547" ht="15.75" customHeight="1"/>
-    <row r="548" ht="15.75" customHeight="1"/>
-    <row r="549" ht="15.75" customHeight="1"/>
-    <row r="550" ht="15.75" customHeight="1"/>
-    <row r="551" ht="15.75" customHeight="1"/>
-    <row r="552" ht="15.75" customHeight="1"/>
-    <row r="553" ht="15.75" customHeight="1"/>
-    <row r="554" ht="15.75" customHeight="1"/>
-    <row r="555" ht="15.75" customHeight="1"/>
-    <row r="556" ht="15.75" customHeight="1"/>
-    <row r="557" ht="15.75" customHeight="1"/>
-    <row r="558" ht="15.75" customHeight="1"/>
-    <row r="559" ht="15.75" customHeight="1"/>
-    <row r="560" ht="15.75" customHeight="1"/>
-    <row r="561" ht="15.75" customHeight="1"/>
-    <row r="562" ht="15.75" customHeight="1"/>
-    <row r="563" ht="15.75" customHeight="1"/>
-    <row r="564" ht="15.75" customHeight="1"/>
-    <row r="565" ht="15.75" customHeight="1"/>
-    <row r="566" ht="15.75" customHeight="1"/>
-    <row r="567" ht="15.75" customHeight="1"/>
-    <row r="568" ht="15.75" customHeight="1"/>
-    <row r="569" ht="15.75" customHeight="1"/>
-    <row r="570" ht="15.75" customHeight="1"/>
-    <row r="571" ht="15.75" customHeight="1"/>
-    <row r="572" ht="15.75" customHeight="1"/>
-    <row r="573" ht="15.75" customHeight="1"/>
-    <row r="574" ht="15.75" customHeight="1"/>
-    <row r="575" ht="15.75" customHeight="1"/>
-    <row r="576" ht="15.75" customHeight="1"/>
-    <row r="577" ht="15.75" customHeight="1"/>
-    <row r="578" ht="15.75" customHeight="1"/>
-    <row r="579" ht="15.75" customHeight="1"/>
-    <row r="580" ht="15.75" customHeight="1"/>
-    <row r="581" ht="15.75" customHeight="1"/>
-    <row r="582" ht="15.75" customHeight="1"/>
-    <row r="583" ht="15.75" customHeight="1"/>
-    <row r="584" ht="15.75" customHeight="1"/>
-    <row r="585" ht="15.75" customHeight="1"/>
-    <row r="586" ht="15.75" customHeight="1"/>
-    <row r="587" ht="15.75" customHeight="1"/>
-    <row r="588" ht="15.75" customHeight="1"/>
-    <row r="589" ht="15.75" customHeight="1"/>
-    <row r="590" ht="15.75" customHeight="1"/>
-    <row r="591" ht="15.75" customHeight="1"/>
-    <row r="592" ht="15.75" customHeight="1"/>
-    <row r="593" ht="15.75" customHeight="1"/>
-    <row r="594" ht="15.75" customHeight="1"/>
-    <row r="595" ht="15.75" customHeight="1"/>
-    <row r="596" ht="15.75" customHeight="1"/>
-    <row r="597" ht="15.75" customHeight="1"/>
-    <row r="598" ht="15.75" customHeight="1"/>
-    <row r="599" ht="15.75" customHeight="1"/>
-    <row r="600" ht="15.75" customHeight="1"/>
-    <row r="601" ht="15.75" customHeight="1"/>
-    <row r="602" ht="15.75" customHeight="1"/>
-    <row r="603" ht="15.75" customHeight="1"/>
-    <row r="604" ht="15.75" customHeight="1"/>
-    <row r="605" ht="15.75" customHeight="1"/>
-    <row r="606" ht="15.75" customHeight="1"/>
-    <row r="607" ht="15.75" customHeight="1"/>
-    <row r="608" ht="15.75" customHeight="1"/>
-    <row r="609" ht="15.75" customHeight="1"/>
-    <row r="610" ht="15.75" customHeight="1"/>
-    <row r="611" ht="15.75" customHeight="1"/>
-    <row r="612" ht="15.75" customHeight="1"/>
-    <row r="613" ht="15.75" customHeight="1"/>
-    <row r="614" ht="15.75" customHeight="1"/>
-    <row r="615" ht="15.75" customHeight="1"/>
-    <row r="616" ht="15.75" customHeight="1"/>
-    <row r="617" ht="15.75" customHeight="1"/>
-    <row r="618" ht="15.75" customHeight="1"/>
-    <row r="619" ht="15.75" customHeight="1"/>
-    <row r="620" ht="15.75" customHeight="1"/>
-    <row r="621" ht="15.75" customHeight="1"/>
-    <row r="622" ht="15.75" customHeight="1"/>
-    <row r="623" ht="15.75" customHeight="1"/>
-    <row r="624" ht="15.75" customHeight="1"/>
-    <row r="625" ht="15.75" customHeight="1"/>
-    <row r="626" ht="15.75" customHeight="1"/>
-    <row r="627" ht="15.75" customHeight="1"/>
-    <row r="628" ht="15.75" customHeight="1"/>
-    <row r="629" ht="15.75" customHeight="1"/>
-    <row r="630" ht="15.75" customHeight="1"/>
-    <row r="631" ht="15.75" customHeight="1"/>
-    <row r="632" ht="15.75" customHeight="1"/>
-    <row r="633" ht="15.75" customHeight="1"/>
-    <row r="634" ht="15.75" customHeight="1"/>
-    <row r="635" ht="15.75" customHeight="1"/>
-    <row r="636" ht="15.75" customHeight="1"/>
-    <row r="637" ht="15.75" customHeight="1"/>
-    <row r="638" ht="15.75" customHeight="1"/>
-    <row r="639" ht="15.75" customHeight="1"/>
-    <row r="640" ht="15.75" customHeight="1"/>
-    <row r="641" ht="15.75" customHeight="1"/>
-    <row r="642" ht="15.75" customHeight="1"/>
-    <row r="643" ht="15.75" customHeight="1"/>
-    <row r="644" ht="15.75" customHeight="1"/>
-    <row r="645" ht="15.75" customHeight="1"/>
-    <row r="646" ht="15.75" customHeight="1"/>
-    <row r="647" ht="15.75" customHeight="1"/>
-    <row r="648" ht="15.75" customHeight="1"/>
-    <row r="649" ht="15.75" customHeight="1"/>
-    <row r="650" ht="15.75" customHeight="1"/>
-    <row r="651" ht="15.75" customHeight="1"/>
-    <row r="652" ht="15.75" customHeight="1"/>
-    <row r="653" ht="15.75" customHeight="1"/>
-    <row r="654" ht="15.75" customHeight="1"/>
-    <row r="655" ht="15.75" customHeight="1"/>
-    <row r="656" ht="15.75" customHeight="1"/>
-    <row r="657" ht="15.75" customHeight="1"/>
-    <row r="658" ht="15.75" customHeight="1"/>
-    <row r="659" ht="15.75" customHeight="1"/>
-    <row r="660" ht="15.75" customHeight="1"/>
-    <row r="661" ht="15.75" customHeight="1"/>
-    <row r="662" ht="15.75" customHeight="1"/>
-    <row r="663" ht="15.75" customHeight="1"/>
-    <row r="664" ht="15.75" customHeight="1"/>
-    <row r="665" ht="15.75" customHeight="1"/>
-    <row r="666" ht="15.75" customHeight="1"/>
-    <row r="667" ht="15.75" customHeight="1"/>
-    <row r="668" ht="15.75" customHeight="1"/>
-    <row r="669" ht="15.75" customHeight="1"/>
-    <row r="670" ht="15.75" customHeight="1"/>
-    <row r="671" ht="15.75" customHeight="1"/>
-    <row r="672" ht="15.75" customHeight="1"/>
-    <row r="673" ht="15.75" customHeight="1"/>
-    <row r="674" ht="15.75" customHeight="1"/>
-    <row r="675" ht="15.75" customHeight="1"/>
-    <row r="676" ht="15.75" customHeight="1"/>
-    <row r="677" ht="15.75" customHeight="1"/>
-    <row r="678" ht="15.75" customHeight="1"/>
-    <row r="679" ht="15.75" customHeight="1"/>
-    <row r="680" ht="15.75" customHeight="1"/>
-    <row r="681" ht="15.75" customHeight="1"/>
-    <row r="682" ht="15.75" customHeight="1"/>
-    <row r="683" ht="15.75" customHeight="1"/>
-    <row r="684" ht="15.75" customHeight="1"/>
-    <row r="685" ht="15.75" customHeight="1"/>
-    <row r="686" ht="15.75" customHeight="1"/>
-    <row r="687" ht="15.75" customHeight="1"/>
-    <row r="688" ht="15.75" customHeight="1"/>
-    <row r="689" ht="15.75" customHeight="1"/>
-    <row r="690" ht="15.75" customHeight="1"/>
-    <row r="691" ht="15.75" customHeight="1"/>
-    <row r="692" ht="15.75" customHeight="1"/>
-    <row r="693" ht="15.75" customHeight="1"/>
-    <row r="694" ht="15.75" customHeight="1"/>
-    <row r="695" ht="15.75" customHeight="1"/>
-    <row r="696" ht="15.75" customHeight="1"/>
-    <row r="697" ht="15.75" customHeight="1"/>
-    <row r="698" ht="15.75" customHeight="1"/>
-    <row r="699" ht="15.75" customHeight="1"/>
-    <row r="700" ht="15.75" customHeight="1"/>
-    <row r="701" ht="15.75" customHeight="1"/>
-    <row r="702" ht="15.75" customHeight="1"/>
-    <row r="703" ht="15.75" customHeight="1"/>
-    <row r="704" ht="15.75" customHeight="1"/>
-    <row r="705" ht="15.75" customHeight="1"/>
-    <row r="706" ht="15.75" customHeight="1"/>
-    <row r="707" ht="15.75" customHeight="1"/>
-    <row r="708" ht="15.75" customHeight="1"/>
-    <row r="709" ht="15.75" customHeight="1"/>
-    <row r="710" ht="15.75" customHeight="1"/>
-    <row r="711" ht="15.75" customHeight="1"/>
-    <row r="712" ht="15.75" customHeight="1"/>
-    <row r="713" ht="15.75" customHeight="1"/>
-    <row r="714" ht="15.75" customHeight="1"/>
-    <row r="715" ht="15.75" customHeight="1"/>
-    <row r="716" ht="15.75" customHeight="1"/>
-    <row r="717" ht="15.75" customHeight="1"/>
-    <row r="718" ht="15.75" customHeight="1"/>
-    <row r="719" ht="15.75" customHeight="1"/>
-    <row r="720" ht="15.75" customHeight="1"/>
-    <row r="721" ht="15.75" customHeight="1"/>
-    <row r="722" ht="15.75" customHeight="1"/>
-    <row r="723" ht="15.75" customHeight="1"/>
-    <row r="724" ht="15.75" customHeight="1"/>
-    <row r="725" ht="15.75" customHeight="1"/>
-    <row r="726" ht="15.75" customHeight="1"/>
-    <row r="727" ht="15.75" customHeight="1"/>
-    <row r="728" ht="15.75" customHeight="1"/>
-    <row r="729" ht="15.75" customHeight="1"/>
-    <row r="730" ht="15.75" customHeight="1"/>
-    <row r="731" ht="15.75" customHeight="1"/>
-    <row r="732" ht="15.75" customHeight="1"/>
-    <row r="733" ht="15.75" customHeight="1"/>
-    <row r="734" ht="15.75" customHeight="1"/>
-    <row r="735" ht="15.75" customHeight="1"/>
-    <row r="736" ht="15.75" customHeight="1"/>
-    <row r="737" ht="15.75" customHeight="1"/>
-    <row r="738" ht="15.75" customHeight="1"/>
-    <row r="739" ht="15.75" customHeight="1"/>
-    <row r="740" ht="15.75" customHeight="1"/>
-    <row r="741" ht="15.75" customHeight="1"/>
-    <row r="742" ht="15.75" customHeight="1"/>
-    <row r="743" ht="15.75" customHeight="1"/>
-    <row r="744" ht="15.75" customHeight="1"/>
-    <row r="745" ht="15.75" customHeight="1"/>
-    <row r="746" ht="15.75" customHeight="1"/>
-    <row r="747" ht="15.75" customHeight="1"/>
-    <row r="748" ht="15.75" customHeight="1"/>
-    <row r="749" ht="15.75" customHeight="1"/>
-    <row r="750" ht="15.75" customHeight="1"/>
-    <row r="751" ht="15.75" customHeight="1"/>
-    <row r="752" ht="15.75" customHeight="1"/>
-    <row r="753" ht="15.75" customHeight="1"/>
-    <row r="754" ht="15.75" customHeight="1"/>
-    <row r="755" ht="15.75" customHeight="1"/>
-    <row r="756" ht="15.75" customHeight="1"/>
-    <row r="757" ht="15.75" customHeight="1"/>
-    <row r="758" ht="15.75" customHeight="1"/>
-    <row r="759" ht="15.75" customHeight="1"/>
-    <row r="760" ht="15.75" customHeight="1"/>
-    <row r="761" ht="15.75" customHeight="1"/>
-    <row r="762" ht="15.75" customHeight="1"/>
-    <row r="763" ht="15.75" customHeight="1"/>
-    <row r="764" ht="15.75" customHeight="1"/>
-    <row r="765" ht="15.75" customHeight="1"/>
-    <row r="766" ht="15.75" customHeight="1"/>
-    <row r="767" ht="15.75" customHeight="1"/>
-    <row r="768" ht="15.75" customHeight="1"/>
-    <row r="769" ht="15.75" customHeight="1"/>
-    <row r="770" ht="15.75" customHeight="1"/>
-    <row r="771" ht="15.75" customHeight="1"/>
-    <row r="772" ht="15.75" customHeight="1"/>
-    <row r="773" ht="15.75" customHeight="1"/>
-    <row r="774" ht="15.75" customHeight="1"/>
-    <row r="775" ht="15.75" customHeight="1"/>
-    <row r="776" ht="15.75" customHeight="1"/>
-    <row r="777" ht="15.75" customHeight="1"/>
-    <row r="778" ht="15.75" customHeight="1"/>
-    <row r="779" ht="15.75" customHeight="1"/>
-    <row r="780" ht="15.75" customHeight="1"/>
-    <row r="781" ht="15.75" customHeight="1"/>
-    <row r="782" ht="15.75" customHeight="1"/>
-    <row r="783" ht="15.75" customHeight="1"/>
-    <row r="784" ht="15.75" customHeight="1"/>
-    <row r="785" ht="15.75" customHeight="1"/>
-    <row r="786" ht="15.75" customHeight="1"/>
-    <row r="787" ht="15.75" customHeight="1"/>
-    <row r="788" ht="15.75" customHeight="1"/>
-    <row r="789" ht="15.75" customHeight="1"/>
-    <row r="790" ht="15.75" customHeight="1"/>
-    <row r="791" ht="15.75" customHeight="1"/>
-    <row r="792" ht="15.75" customHeight="1"/>
-    <row r="793" ht="15.75" customHeight="1"/>
-    <row r="794" ht="15.75" customHeight="1"/>
-    <row r="795" ht="15.75" customHeight="1"/>
-    <row r="796" ht="15.75" customHeight="1"/>
-    <row r="797" ht="15.75" customHeight="1"/>
-    <row r="798" ht="15.75" customHeight="1"/>
-    <row r="799" ht="15.75" customHeight="1"/>
-    <row r="800" ht="15.75" customHeight="1"/>
-    <row r="801" ht="15.75" customHeight="1"/>
-    <row r="802" ht="15.75" customHeight="1"/>
-    <row r="803" ht="15.75" customHeight="1"/>
-    <row r="804" ht="15.75" customHeight="1"/>
-    <row r="805" ht="15.75" customHeight="1"/>
-    <row r="806" ht="15.75" customHeight="1"/>
-    <row r="807" ht="15.75" customHeight="1"/>
-    <row r="808" ht="15.75" customHeight="1"/>
-    <row r="809" ht="15.75" customHeight="1"/>
-    <row r="810" ht="15.75" customHeight="1"/>
-    <row r="811" ht="15.75" customHeight="1"/>
-    <row r="812" ht="15.75" customHeight="1"/>
-    <row r="813" ht="15.75" customHeight="1"/>
-    <row r="814" ht="15.75" customHeight="1"/>
-    <row r="815" ht="15.75" customHeight="1"/>
-    <row r="816" ht="15.75" customHeight="1"/>
-    <row r="817" ht="15.75" customHeight="1"/>
-    <row r="818" ht="15.75" customHeight="1"/>
-    <row r="819" ht="15.75" customHeight="1"/>
-    <row r="820" ht="15.75" customHeight="1"/>
-    <row r="821" ht="15.75" customHeight="1"/>
-    <row r="822" ht="15.75" customHeight="1"/>
-    <row r="823" ht="15.75" customHeight="1"/>
-    <row r="824" ht="15.75" customHeight="1"/>
-    <row r="825" ht="15.75" customHeight="1"/>
-    <row r="826" ht="15.75" customHeight="1"/>
-    <row r="827" ht="15.75" customHeight="1"/>
-    <row r="828" ht="15.75" customHeight="1"/>
-    <row r="829" ht="15.75" customHeight="1"/>
-    <row r="830" ht="15.75" customHeight="1"/>
-    <row r="831" ht="15.75" customHeight="1"/>
-    <row r="832" ht="15.75" customHeight="1"/>
-    <row r="833" ht="15.75" customHeight="1"/>
-    <row r="834" ht="15.75" customHeight="1"/>
-    <row r="835" ht="15.75" customHeight="1"/>
-    <row r="836" ht="15.75" customHeight="1"/>
-    <row r="837" ht="15.75" customHeight="1"/>
-    <row r="838" ht="15.75" customHeight="1"/>
-    <row r="839" ht="15.75" customHeight="1"/>
-    <row r="840" ht="15.75" customHeight="1"/>
-    <row r="841" ht="15.75" customHeight="1"/>
-    <row r="842" ht="15.75" customHeight="1"/>
-    <row r="843" ht="15.75" customHeight="1"/>
-    <row r="844" ht="15.75" customHeight="1"/>
-    <row r="845" ht="15.75" customHeight="1"/>
-    <row r="846" ht="15.75" customHeight="1"/>
-    <row r="847" ht="15.75" customHeight="1"/>
-    <row r="848" ht="15.75" customHeight="1"/>
-    <row r="849" ht="15.75" customHeight="1"/>
-    <row r="850" ht="15.75" customHeight="1"/>
-    <row r="851" ht="15.75" customHeight="1"/>
-    <row r="852" ht="15.75" customHeight="1"/>
-    <row r="853" ht="15.75" customHeight="1"/>
-    <row r="854" ht="15.75" customHeight="1"/>
-    <row r="855" ht="15.75" customHeight="1"/>
-    <row r="856" ht="15.75" customHeight="1"/>
-    <row r="857" ht="15.75" customHeight="1"/>
-    <row r="858" ht="15.75" customHeight="1"/>
-    <row r="859" ht="15.75" customHeight="1"/>
-    <row r="860" ht="15.75" customHeight="1"/>
-    <row r="861" ht="15.75" customHeight="1"/>
-    <row r="862" ht="15.75" customHeight="1"/>
-    <row r="863" ht="15.75" customHeight="1"/>
-    <row r="864" ht="15.75" customHeight="1"/>
-    <row r="865" ht="15.75" customHeight="1"/>
-    <row r="866" ht="15.75" customHeight="1"/>
-    <row r="867" ht="15.75" customHeight="1"/>
-    <row r="868" ht="15.75" customHeight="1"/>
-    <row r="869" ht="15.75" customHeight="1"/>
-    <row r="870" ht="15.75" customHeight="1"/>
-    <row r="871" ht="15.75" customHeight="1"/>
-    <row r="872" ht="15.75" customHeight="1"/>
-    <row r="873" ht="15.75" customHeight="1"/>
-    <row r="874" ht="15.75" customHeight="1"/>
-    <row r="875" ht="15.75" customHeight="1"/>
-    <row r="876" ht="15.75" customHeight="1"/>
-    <row r="877" ht="15.75" customHeight="1"/>
-    <row r="878" ht="15.75" customHeight="1"/>
-    <row r="879" ht="15.75" customHeight="1"/>
-    <row r="880" ht="15.75" customHeight="1"/>
-    <row r="881" ht="15.75" customHeight="1"/>
-    <row r="882" ht="15.75" customHeight="1"/>
-    <row r="883" ht="15.75" customHeight="1"/>
-    <row r="884" ht="15.75" customHeight="1"/>
-    <row r="885" ht="15.75" customHeight="1"/>
-    <row r="886" ht="15.75" customHeight="1"/>
-    <row r="887" ht="15.75" customHeight="1"/>
-    <row r="888" ht="15.75" customHeight="1"/>
-    <row r="889" ht="15.75" customHeight="1"/>
-    <row r="890" ht="15.75" customHeight="1"/>
-    <row r="891" ht="15.75" customHeight="1"/>
-    <row r="892" ht="15.75" customHeight="1"/>
-    <row r="893" ht="15.75" customHeight="1"/>
-    <row r="894" ht="15.75" customHeight="1"/>
-    <row r="895" ht="15.75" customHeight="1"/>
-    <row r="896" ht="15.75" customHeight="1"/>
-    <row r="897" ht="15.75" customHeight="1"/>
-    <row r="898" ht="15.75" customHeight="1"/>
-    <row r="899" ht="15.75" customHeight="1"/>
-    <row r="900" ht="15.75" customHeight="1"/>
-    <row r="901" ht="15.75" customHeight="1"/>
-    <row r="902" ht="15.75" customHeight="1"/>
-    <row r="903" ht="15.75" customHeight="1"/>
-    <row r="904" ht="15.75" customHeight="1"/>
-    <row r="905" ht="15.75" customHeight="1"/>
-    <row r="906" ht="15.75" customHeight="1"/>
-    <row r="907" ht="15.75" customHeight="1"/>
-    <row r="908" ht="15.75" customHeight="1"/>
-    <row r="909" ht="15.75" customHeight="1"/>
-    <row r="910" ht="15.75" customHeight="1"/>
-    <row r="911" ht="15.75" customHeight="1"/>
-    <row r="912" ht="15.75" customHeight="1"/>
-    <row r="913" ht="15.75" customHeight="1"/>
-    <row r="914" ht="15.75" customHeight="1"/>
-    <row r="915" ht="15.75" customHeight="1"/>
-    <row r="916" ht="15.75" customHeight="1"/>
-    <row r="917" ht="15.75" customHeight="1"/>
-    <row r="918" ht="15.75" customHeight="1"/>
-    <row r="919" ht="15.75" customHeight="1"/>
-    <row r="920" ht="15.75" customHeight="1"/>
-    <row r="921" ht="15.75" customHeight="1"/>
-    <row r="922" ht="15.75" customHeight="1"/>
-    <row r="923" ht="15.75" customHeight="1"/>
-    <row r="924" ht="15.75" customHeight="1"/>
-    <row r="925" ht="15.75" customHeight="1"/>
-    <row r="926" ht="15.75" customHeight="1"/>
-    <row r="927" ht="15.75" customHeight="1"/>
-    <row r="928" ht="15.75" customHeight="1"/>
-    <row r="929" ht="15.75" customHeight="1"/>
-    <row r="930" ht="15.75" customHeight="1"/>
-    <row r="931" ht="15.75" customHeight="1"/>
-    <row r="932" ht="15.75" customHeight="1"/>
-    <row r="933" ht="15.75" customHeight="1"/>
-    <row r="934" ht="15.75" customHeight="1"/>
-    <row r="935" ht="15.75" customHeight="1"/>
-    <row r="936" ht="15.75" customHeight="1"/>
-    <row r="937" ht="15.75" customHeight="1"/>
-    <row r="938" ht="15.75" customHeight="1"/>
-    <row r="939" ht="15.75" customHeight="1"/>
-    <row r="940" ht="15.75" customHeight="1"/>
-    <row r="941" ht="15.75" customHeight="1"/>
-    <row r="942" ht="15.75" customHeight="1"/>
-    <row r="943" ht="15.75" customHeight="1"/>
-    <row r="944" ht="15.75" customHeight="1"/>
-    <row r="945" ht="15.75" customHeight="1"/>
-    <row r="946" ht="15.75" customHeight="1"/>
-    <row r="947" ht="15.75" customHeight="1"/>
-    <row r="948" ht="15.75" customHeight="1"/>
-    <row r="949" ht="15.75" customHeight="1"/>
-    <row r="950" ht="15.75" customHeight="1"/>
-    <row r="951" ht="15.75" customHeight="1"/>
-    <row r="952" ht="15.75" customHeight="1"/>
-    <row r="953" ht="15.75" customHeight="1"/>
-    <row r="954" ht="15.75" customHeight="1"/>
-    <row r="955" ht="15.75" customHeight="1"/>
-    <row r="956" ht="15.75" customHeight="1"/>
-    <row r="957" ht="15.75" customHeight="1"/>
-    <row r="958" ht="15.75" customHeight="1"/>
-    <row r="959" ht="15.75" customHeight="1"/>
-    <row r="960" ht="15.75" customHeight="1"/>
-    <row r="961" ht="15.75" customHeight="1"/>
-    <row r="962" ht="15.75" customHeight="1"/>
-    <row r="963" ht="15.75" customHeight="1"/>
-    <row r="964" ht="15.75" customHeight="1"/>
-    <row r="965" ht="15.75" customHeight="1"/>
-    <row r="966" ht="15.75" customHeight="1"/>
-    <row r="967" ht="15.75" customHeight="1"/>
-    <row r="968" ht="15.75" customHeight="1"/>
-    <row r="969" ht="15.75" customHeight="1"/>
-    <row r="970" ht="15.75" customHeight="1"/>
-    <row r="971" ht="15.75" customHeight="1"/>
-    <row r="972" ht="15.75" customHeight="1"/>
-    <row r="973" ht="15.75" customHeight="1"/>
-    <row r="974" ht="15.75" customHeight="1"/>
-    <row r="975" ht="15.75" customHeight="1"/>
-    <row r="976" ht="15.75" customHeight="1"/>
-    <row r="977" ht="15.75" customHeight="1"/>
-    <row r="978" ht="15.75" customHeight="1"/>
-    <row r="979" ht="15.75" customHeight="1"/>
-    <row r="980" ht="15.75" customHeight="1"/>
-    <row r="981" ht="15.75" customHeight="1"/>
-    <row r="982" ht="15.75" customHeight="1"/>
-    <row r="983" ht="15.75" customHeight="1"/>
-    <row r="984" ht="15.75" customHeight="1"/>
-    <row r="985" ht="15.75" customHeight="1"/>
-    <row r="986" ht="15.75" customHeight="1"/>
-    <row r="987" ht="15.75" customHeight="1"/>
-    <row r="988" ht="15.75" customHeight="1"/>
-    <row r="989" ht="15.75" customHeight="1"/>
-    <row r="990" ht="15.75" customHeight="1"/>
-    <row r="991" ht="15.75" customHeight="1"/>
-    <row r="992" ht="15.75" customHeight="1"/>
-    <row r="993" ht="15.75" customHeight="1"/>
-    <row r="994" ht="15.75" customHeight="1"/>
-    <row r="995" ht="15.75" customHeight="1"/>
-    <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
+    <row r="229" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="230" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="231" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="232" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="233" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="234" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="235" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="236" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="237" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="238" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="239" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="240" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="A20:I20"/>
-    <mergeCell ref="A21:C22"/>
-    <mergeCell ref="D21:I22"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="D27:I27"/>
-    <mergeCell ref="F28:I28"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F23:I23"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A25:C26"/>
-    <mergeCell ref="D25:F26"/>
-    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="A1:I10"/>
+    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="A14:C14"/>
     <mergeCell ref="D18:F18"/>
     <mergeCell ref="H18:I18"/>
     <mergeCell ref="A15:C15"/>
@@ -9570,15 +9577,25 @@
     <mergeCell ref="A17:C17"/>
     <mergeCell ref="D17:F17"/>
     <mergeCell ref="A18:C18"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="A1:I10"/>
-    <mergeCell ref="A11:I11"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F23:I23"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A25:C26"/>
+    <mergeCell ref="D25:F26"/>
+    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="D27:I27"/>
+    <mergeCell ref="F28:I28"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A21:C22"/>
+    <mergeCell ref="D21:I22"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.78740157480314965" right="0.78740157480314965" top="0.59055118110236227" bottom="0.39370078740157483" header="0" footer="0"/>

</xml_diff>

<commit_message>
Ajustar diseño de plantilla de Cuenta de Cobro (alineación de logo y tamaño de fuente) para perfecta conversión a PDF en Linux
</commit_message>
<xml_diff>
--- a/plantillas/CUENTA_COBRO.xlsx
+++ b/plantillas/CUENTA_COBRO.xlsx
@@ -8,16 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Soporte y Desarrollo\Documents\NetBeansProjects\combinacion\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0601C33E-B26B-4C5D-A19D-AB5C1BA76F05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F7446E9-C919-4861-BB31-27169EB1E251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Documento Equivalente" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Documento Equivalente'!$A$1:$I$28</definedName>
-  </definedNames>
   <calcPr calcId="0"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
@@ -193,7 +190,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="36">
+  <borders count="37">
     <border>
       <left/>
       <right/>
@@ -593,6 +590,19 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -604,167 +614,169 @@
   </cellStyleXfs>
   <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="12" fontId="4" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="12" fontId="4" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="12" fontId="4" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="12" fontId="4" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1108,11 +1120,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>2</xdr:colOff>
+      <xdr:colOff>9525</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>66675</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="8391524" cy="1790700"/>
+    <xdr:ext cx="8391525" cy="1790700"/>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
         <xdr:cNvPr id="7" name="Shape 2">
@@ -1126,8 +1138,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="2" y="0"/>
-          <a:ext cx="8391524" cy="1790700"/>
+          <a:off x="9525" y="66675"/>
+          <a:ext cx="8391525" cy="1790700"/>
           <a:chOff x="1469325" y="2884650"/>
           <a:chExt cx="7753350" cy="1790700"/>
         </a:xfrm>
@@ -1181,7 +1193,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
-              <a:pPr marL="0" lvl="0" indent="0" algn="l" rtl="0">
+              <a:pPr marL="0" lvl="0" indent="0" algn="ctr" rtl="0">
                 <a:spcBef>
                   <a:spcPts val="0"/>
                 </a:spcBef>
@@ -1243,7 +1255,7 @@
               </a:bodyPr>
               <a:lstStyle/>
               <a:p>
-                <a:pPr marL="0" lvl="0" indent="0" algn="l" rtl="0">
+                <a:pPr marL="0" lvl="0" indent="0" algn="ctr" rtl="0">
                   <a:spcBef>
                     <a:spcPts val="0"/>
                   </a:spcBef>
@@ -1307,7 +1319,7 @@
                 </a:bodyPr>
                 <a:lstStyle/>
                 <a:p>
-                  <a:pPr marL="0" lvl="0" indent="0" algn="l" rtl="0">
+                  <a:pPr marL="0" lvl="0" indent="0" algn="ctr" rtl="0">
                     <a:spcBef>
                       <a:spcPts val="0"/>
                     </a:spcBef>
@@ -1371,7 +1383,7 @@
                   </a:bodyPr>
                   <a:lstStyle/>
                   <a:p>
-                    <a:pPr marL="0" lvl="0" indent="0" algn="l" rtl="0">
+                    <a:pPr marL="0" lvl="0" indent="0" algn="ctr" rtl="0">
                       <a:spcBef>
                         <a:spcPts val="0"/>
                       </a:spcBef>
@@ -1435,7 +1447,7 @@
                     </a:bodyPr>
                     <a:lstStyle/>
                     <a:p>
-                      <a:pPr marL="0" lvl="0" indent="0" algn="l" rtl="0">
+                      <a:pPr marL="0" lvl="0" indent="0" algn="ctr" rtl="0">
                         <a:spcBef>
                           <a:spcPts val="0"/>
                         </a:spcBef>
@@ -1499,7 +1511,7 @@
                       </a:bodyPr>
                       <a:lstStyle/>
                       <a:p>
-                        <a:pPr marL="0" lvl="0" indent="0" algn="l" rtl="0">
+                        <a:pPr marL="0" lvl="0" indent="0" algn="ctr" rtl="0">
                           <a:spcBef>
                             <a:spcPts val="0"/>
                           </a:spcBef>
@@ -1569,7 +1581,7 @@
                         </a:bodyPr>
                         <a:lstStyle/>
                         <a:p>
-                          <a:pPr marL="0" lvl="0" indent="0" algn="l" rtl="0">
+                          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" rtl="0">
                             <a:spcBef>
                               <a:spcPts val="0"/>
                             </a:spcBef>
@@ -2213,6 +2225,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2226,208 +2241,208 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
+      <c r="A1" s="20"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
     </row>
     <row r="2" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
+      <c r="A2" s="20"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
     </row>
     <row r="3" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
+      <c r="A3" s="20"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
     </row>
     <row r="4" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
+      <c r="A4" s="20"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
     </row>
     <row r="5" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
+      <c r="A5" s="20"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
     </row>
     <row r="6" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
+      <c r="A6" s="20"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
     </row>
     <row r="7" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
+      <c r="A7" s="20"/>
+      <c r="B7" s="20"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="20"/>
     </row>
     <row r="8" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
+      <c r="A8" s="20"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
     </row>
     <row r="9" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
+      <c r="A9" s="20"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
     </row>
     <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
+      <c r="A10" s="20"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="20"/>
+      <c r="I10" s="20"/>
     </row>
     <row r="11" spans="1:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="7"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="22"/>
+      <c r="I11" s="23"/>
     </row>
     <row r="12" spans="1:9" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="39" t="s">
+      <c r="A12" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="41" t="s">
+      <c r="B12" s="22"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="G12" s="45" t="s">
+      <c r="G12" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="H12" s="47">
+      <c r="H12" s="13">
         <v>4121</v>
       </c>
-      <c r="I12" s="48"/>
+      <c r="I12" s="14"/>
     </row>
     <row r="13" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="27" t="s">
         <v>4</v>
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="17"/>
-      <c r="D13" s="42" t="s">
+      <c r="D13" s="28" t="s">
         <v>5</v>
       </c>
       <c r="E13" s="16"/>
       <c r="F13" s="17"/>
-      <c r="G13" s="44" t="s">
+      <c r="G13" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H13" s="46">
+      <c r="H13" s="6">
         <v>890399011</v>
       </c>
-      <c r="I13" s="37">
+      <c r="I13" s="3">
         <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="39" t="s">
+      <c r="A14" s="27" t="s">
         <v>7</v>
       </c>
       <c r="B14" s="16"/>
       <c r="C14" s="17"/>
-      <c r="D14" s="43" t="s">
+      <c r="D14" s="15" t="s">
         <v>8</v>
       </c>
       <c r="E14" s="16"/>
       <c r="F14" s="17"/>
-      <c r="G14" s="44" t="s">
+      <c r="G14" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="H14" s="49">
+      <c r="H14" s="18">
         <v>4121</v>
       </c>
-      <c r="I14" s="34"/>
+      <c r="I14" s="19"/>
     </row>
     <row r="15" spans="1:9" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="39" t="s">
+      <c r="A15" s="27" t="s">
         <v>10</v>
       </c>
       <c r="B15" s="16"/>
       <c r="C15" s="17"/>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="32" t="s">
         <v>11</v>
       </c>
       <c r="E15" s="16"/>
       <c r="F15" s="17"/>
-      <c r="G15" s="44" t="s">
+      <c r="G15" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="50">
+      <c r="H15" s="33">
         <v>8896744</v>
       </c>
       <c r="I15" s="17"/>
     </row>
     <row r="16" spans="1:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="34" t="s">
         <v>13</v>
       </c>
       <c r="B16" s="16"/>
@@ -2440,52 +2455,52 @@
       <c r="I16" s="17"/>
     </row>
     <row r="17" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="63" t="s">
+      <c r="A17" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="64"/>
-      <c r="C17" s="65"/>
-      <c r="D17" s="35"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="36" t="s">
+      <c r="B17" s="36"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="39"/>
+      <c r="F17" s="40"/>
+      <c r="G17" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H17" s="54"/>
-      <c r="I17" s="55"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="10"/>
     </row>
     <row r="18" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="66" t="s">
+      <c r="A18" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="1"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="53" t="s">
+      <c r="B18" s="30"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H18" s="43"/>
+      <c r="H18" s="15"/>
       <c r="I18" s="17"/>
     </row>
     <row r="19" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="67" t="s">
+      <c r="A19" s="61" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="68"/>
-      <c r="C19" s="69"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="51" t="s">
+      <c r="B19" s="62"/>
+      <c r="C19" s="63"/>
+      <c r="D19" s="64"/>
+      <c r="E19" s="65"/>
+      <c r="F19" s="66"/>
+      <c r="G19" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="H19" s="52"/>
+      <c r="H19" s="67"/>
       <c r="I19" s="17"/>
     </row>
     <row r="20" spans="1:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="15" t="s">
+      <c r="A20" s="52" t="s">
         <v>20</v>
       </c>
       <c r="B20" s="16"/>
@@ -2498,108 +2513,108 @@
       <c r="I20" s="17"/>
     </row>
     <row r="21" spans="1:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="31" t="s">
+      <c r="A21" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="22"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="33"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="22"/>
-      <c r="I21" s="23"/>
+      <c r="B21" s="49"/>
+      <c r="C21" s="50"/>
+      <c r="D21" s="69"/>
+      <c r="E21" s="49"/>
+      <c r="F21" s="49"/>
+      <c r="G21" s="49"/>
+      <c r="H21" s="49"/>
+      <c r="I21" s="50"/>
     </row>
     <row r="22" spans="1:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="24"/>
-      <c r="B22" s="6"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="7"/>
+      <c r="A22" s="47"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="47"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="22"/>
+      <c r="H22" s="22"/>
+      <c r="I22" s="23"/>
     </row>
     <row r="23" spans="1:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="32" t="s">
+      <c r="A23" s="44" t="s">
         <v>22</v>
       </c>
       <c r="B23" s="16"/>
       <c r="C23" s="17"/>
-      <c r="D23" s="20"/>
+      <c r="D23" s="42"/>
       <c r="E23" s="17"/>
-      <c r="F23" s="18"/>
+      <c r="F23" s="43"/>
       <c r="G23" s="16"/>
       <c r="H23" s="16"/>
       <c r="I23" s="17"/>
     </row>
     <row r="24" spans="1:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="15" t="s">
+      <c r="A24" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="27"/>
-      <c r="C24" s="27"/>
-      <c r="D24" s="27"/>
-      <c r="E24" s="27"/>
-      <c r="F24" s="27"/>
-      <c r="G24" s="27"/>
-      <c r="H24" s="27"/>
+      <c r="B24" s="53"/>
+      <c r="C24" s="53"/>
+      <c r="D24" s="53"/>
+      <c r="E24" s="53"/>
+      <c r="F24" s="53"/>
+      <c r="G24" s="53"/>
+      <c r="H24" s="53"/>
       <c r="I24" s="17"/>
     </row>
     <row r="25" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="25" t="s">
+      <c r="A25" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="14"/>
+      <c r="B25" s="46"/>
       <c r="C25" s="26"/>
-      <c r="D25" s="28"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="23"/>
-      <c r="G25" s="30" t="s">
+      <c r="D25" s="48"/>
+      <c r="E25" s="49"/>
+      <c r="F25" s="50"/>
+      <c r="G25" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="H25" s="29"/>
+      <c r="H25" s="56"/>
       <c r="I25" s="17"/>
     </row>
     <row r="26" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="24"/>
-      <c r="B26" s="6"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="56"/>
-      <c r="E26" s="14"/>
+      <c r="A26" s="47"/>
+      <c r="B26" s="22"/>
+      <c r="C26" s="23"/>
+      <c r="D26" s="51"/>
+      <c r="E26" s="46"/>
       <c r="F26" s="26"/>
-      <c r="G26" s="57" t="s">
+      <c r="G26" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="H26" s="28"/>
-      <c r="I26" s="23"/>
+      <c r="H26" s="48"/>
+      <c r="I26" s="50"/>
     </row>
     <row r="27" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="21" t="s">
+      <c r="A27" s="54" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="16"/>
       <c r="C27" s="16"/>
-      <c r="D27" s="60"/>
-      <c r="E27" s="61"/>
-      <c r="F27" s="61"/>
-      <c r="G27" s="61"/>
-      <c r="H27" s="61"/>
-      <c r="I27" s="62"/>
+      <c r="D27" s="57"/>
+      <c r="E27" s="58"/>
+      <c r="F27" s="58"/>
+      <c r="G27" s="58"/>
+      <c r="H27" s="58"/>
+      <c r="I27" s="59"/>
     </row>
     <row r="28" spans="1:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="21" t="s">
+      <c r="A28" s="54" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="16"/>
       <c r="C28" s="17"/>
-      <c r="D28" s="58"/>
-      <c r="E28" s="6"/>
-      <c r="F28" s="59"/>
-      <c r="G28" s="6"/>
-      <c r="H28" s="6"/>
-      <c r="I28" s="7"/>
+      <c r="D28" s="55"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="60"/>
+      <c r="G28" s="22"/>
+      <c r="H28" s="22"/>
+      <c r="I28" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="37">
@@ -2643,7 +2658,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.78740157480314965" right="0.78740157480314965" top="0.59055118110236227" bottom="0.39370078740157483" header="0" footer="0"/>
-  <pageSetup scale="75" orientation="portrait" r:id="rId1"/>
+  <pageSetup scale="75" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;LEste documento es propiedad de la Administración Central del Distrito de Santiago de Cali. Prohibida su reproducción por cualquier medio, sin previa autorización del señor Alcalde. &amp;C &amp;RPágina &amp;P de 1</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
Ajustes de bugs en radicacion, observaciones_tecnicas por defecto en N/A, limpiezas de HTML
</commit_message>
<xml_diff>
--- a/plantillas/CUENTA_COBRO.xlsx
+++ b/plantillas/CUENTA_COBRO.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Soporte y Desarrollo\Documents\NetBeansProjects\combinacion\plantillas\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81717961-126E-49D4-9AB9-C464D1D8D3E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11160"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Documento Equivalente" sheetId="1" r:id="rId1"/>
@@ -115,13 +121,13 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;\ * #,##0.00_);_(&quot;$&quot;\ * \(#,##0.00\);_(&quot;$&quot;\ * &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="dd\-mm\-yyyy"/>
-    <numFmt numFmtId="167" formatCode="##,###"/>
-    <numFmt numFmtId="168" formatCode="&quot;$&quot;\ #,##0"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;\ * #,##0.00_);_(&quot;$&quot;\ * \(#,##0.00\);_(&quot;$&quot;\ * &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="dd\-mm\-yyyy"/>
+    <numFmt numFmtId="165" formatCode="##,###"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;\ #,##0"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -201,49 +207,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="43">
+  <borders count="18">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -254,99 +223,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
       <right/>
       <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -365,256 +246,6 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
       <right/>
       <top/>
       <bottom style="thin">
@@ -625,55 +256,6 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -691,179 +273,282 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="12" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="12" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="12" fontId="6" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="12" fontId="6" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -896,7 +581,7 @@
         <xdr:cNvPr id="3" name="Shape 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -951,7 +636,7 @@
         <xdr:cNvPr id="4" name="Shape 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000004000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1006,7 +691,7 @@
         <xdr:cNvPr id="2" name="Shape 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1061,7 +746,7 @@
         <xdr:cNvPr id="5" name="Shape 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000005000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1116,7 +801,7 @@
         <xdr:cNvPr id="6" name="Shape 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000006000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1211,13 +896,13 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="7810500" cy="1790700"/>
+    <xdr:ext cx="8362950" cy="1724025"/>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
         <xdr:cNvPr id="7" name="Shape 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000007000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000007000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1226,7 +911,7 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="7810500" cy="1790700"/>
+          <a:ext cx="8362950" cy="1724025"/>
           <a:chOff x="1469325" y="2884650"/>
           <a:chExt cx="7753350" cy="1790700"/>
         </a:xfrm>
@@ -1236,7 +921,7 @@
           <xdr:cNvPr id="8" name="Shape 6">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000008000000}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000008000000}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
@@ -1255,7 +940,7 @@
             <xdr:cNvPr id="9" name="Shape 7">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000009000000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1298,7 +983,7 @@
             <xdr:cNvPr id="10" name="Shape 8">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000A000000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000A000000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1317,7 +1002,7 @@
               <xdr:cNvPr id="11" name="Shape 9">
                 <a:extLst>
                   <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000B000000}"/>
+                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000B000000}"/>
                   </a:ext>
                 </a:extLst>
               </xdr:cNvPr>
@@ -1362,7 +1047,7 @@
               <xdr:cNvPr id="12" name="Shape 10">
                 <a:extLst>
                   <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000C000000}"/>
+                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000C000000}"/>
                   </a:ext>
                 </a:extLst>
               </xdr:cNvPr>
@@ -1381,7 +1066,7 @@
                 <xdr:cNvPr id="13" name="Shape 11">
                   <a:extLst>
                     <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000D000000}"/>
+                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000D000000}"/>
                     </a:ext>
                   </a:extLst>
                 </xdr:cNvPr>
@@ -1426,7 +1111,7 @@
                 <xdr:cNvPr id="14" name="Shape 12">
                   <a:extLst>
                     <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000E000000}"/>
+                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000E000000}"/>
                     </a:ext>
                   </a:extLst>
                 </xdr:cNvPr>
@@ -1445,7 +1130,7 @@
                   <xdr:cNvPr id="15" name="Shape 13">
                     <a:extLst>
                       <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000F000000}"/>
+                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000F000000}"/>
                       </a:ext>
                     </a:extLst>
                   </xdr:cNvPr>
@@ -1490,7 +1175,7 @@
                   <xdr:cNvPr id="16" name="Shape 14">
                     <a:extLst>
                       <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000010000000}"/>
+                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000010000000}"/>
                       </a:ext>
                     </a:extLst>
                   </xdr:cNvPr>
@@ -1509,7 +1194,7 @@
                     <xdr:cNvPr id="17" name="Shape 15">
                       <a:extLst>
                         <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                          <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000011000000}"/>
+                          <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000011000000}"/>
                         </a:ext>
                       </a:extLst>
                     </xdr:cNvPr>
@@ -1554,7 +1239,7 @@
                     <xdr:cNvPr id="18" name="Shape 16">
                       <a:extLst>
                         <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                          <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000012000000}"/>
+                          <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000012000000}"/>
                         </a:ext>
                       </a:extLst>
                     </xdr:cNvPr>
@@ -1573,7 +1258,7 @@
                       <xdr:cNvPr id="19" name="Shape 17">
                         <a:extLst>
                           <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                            <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000013000000}"/>
+                            <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000013000000}"/>
                           </a:ext>
                         </a:extLst>
                       </xdr:cNvPr>
@@ -1618,7 +1303,7 @@
                       <xdr:cNvPr id="20" name="Shape 18">
                         <a:extLst>
                           <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                            <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000014000000}"/>
+                            <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000014000000}"/>
                           </a:ext>
                         </a:extLst>
                       </xdr:cNvPr>
@@ -1637,7 +1322,7 @@
                         <xdr:cNvPr id="21" name="Shape 19">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000015000000}"/>
+                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000015000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -1688,7 +1373,7 @@
                         <xdr:cNvPr id="22" name="Shape 20">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000016000000}"/>
+                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000016000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -1764,7 +1449,7 @@
                         <xdr:cNvPr id="23" name="Shape 21">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000017000000}"/>
+                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000017000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -1832,7 +1517,7 @@
                         <xdr:cNvPr id="24" name="Shape 22">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000018000000}"/>
+                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000018000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -1900,7 +1585,7 @@
                         <xdr:cNvPr id="25" name="Shape 23">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000019000000}"/>
+                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000019000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -2075,7 +1760,7 @@
                       <xdr:cNvPr id="26" name="Shape 24" descr="escudo">
                         <a:extLst>
                           <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                            <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00001A000000}"/>
+                            <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001A000000}"/>
                           </a:ext>
                         </a:extLst>
                       </xdr:cNvPr>
@@ -2311,7 +1996,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2329,15 +2014,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="23"/>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
+      <c r="A1" s="57"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="58"/>
+      <c r="I1" s="58"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
@@ -2357,15 +2042,15 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="24"/>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
+      <c r="A2" s="58"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
@@ -2385,15 +2070,15 @@
       <c r="Z2" s="1"/>
     </row>
     <row r="3" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="24"/>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
+      <c r="A3" s="58"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="58"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
@@ -2413,15 +2098,15 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="24"/>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
-      <c r="G4" s="24"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="24"/>
+      <c r="A4" s="58"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="58"/>
+      <c r="H4" s="58"/>
+      <c r="I4" s="58"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
@@ -2441,15 +2126,15 @@
       <c r="Z4" s="1"/>
     </row>
     <row r="5" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="24"/>
-      <c r="B5" s="24"/>
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="24"/>
-      <c r="H5" s="24"/>
-      <c r="I5" s="24"/>
+      <c r="A5" s="58"/>
+      <c r="B5" s="58"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="58"/>
+      <c r="E5" s="58"/>
+      <c r="F5" s="58"/>
+      <c r="G5" s="58"/>
+      <c r="H5" s="58"/>
+      <c r="I5" s="58"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
@@ -2469,15 +2154,15 @@
       <c r="Z5" s="1"/>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="24"/>
-      <c r="B6" s="24"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="24"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="24"/>
+      <c r="A6" s="58"/>
+      <c r="B6" s="58"/>
+      <c r="C6" s="58"/>
+      <c r="D6" s="58"/>
+      <c r="E6" s="58"/>
+      <c r="F6" s="58"/>
+      <c r="G6" s="58"/>
+      <c r="H6" s="58"/>
+      <c r="I6" s="58"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
@@ -2497,15 +2182,15 @@
       <c r="Z6" s="1"/>
     </row>
     <row r="7" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="24"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="24"/>
+      <c r="A7" s="58"/>
+      <c r="B7" s="58"/>
+      <c r="C7" s="58"/>
+      <c r="D7" s="58"/>
+      <c r="E7" s="58"/>
+      <c r="F7" s="58"/>
+      <c r="G7" s="58"/>
+      <c r="H7" s="58"/>
+      <c r="I7" s="58"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
@@ -2525,15 +2210,15 @@
       <c r="Z7" s="1"/>
     </row>
     <row r="8" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="24"/>
-      <c r="B8" s="24"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="24"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="24"/>
+      <c r="A8" s="58"/>
+      <c r="B8" s="58"/>
+      <c r="C8" s="58"/>
+      <c r="D8" s="58"/>
+      <c r="E8" s="58"/>
+      <c r="F8" s="58"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="58"/>
+      <c r="I8" s="58"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
@@ -2553,15 +2238,15 @@
       <c r="Z8" s="1"/>
     </row>
     <row r="9" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="24"/>
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="24"/>
-      <c r="H9" s="24"/>
-      <c r="I9" s="24"/>
+      <c r="A9" s="58"/>
+      <c r="B9" s="58"/>
+      <c r="C9" s="58"/>
+      <c r="D9" s="58"/>
+      <c r="E9" s="58"/>
+      <c r="F9" s="58"/>
+      <c r="G9" s="58"/>
+      <c r="H9" s="58"/>
+      <c r="I9" s="58"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
@@ -2581,15 +2266,15 @@
       <c r="Z9" s="1"/>
     </row>
     <row r="10" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="24"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="24"/>
+      <c r="A10" s="58"/>
+      <c r="B10" s="58"/>
+      <c r="C10" s="58"/>
+      <c r="D10" s="58"/>
+      <c r="E10" s="58"/>
+      <c r="F10" s="58"/>
+      <c r="G10" s="58"/>
+      <c r="H10" s="58"/>
+      <c r="I10" s="58"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
@@ -2609,18 +2294,18 @@
       <c r="Z10" s="1"/>
     </row>
     <row r="11" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="27"/>
-      <c r="J11" s="17">
+      <c r="B11" s="19"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="20"/>
+      <c r="J11" s="5">
         <v>1</v>
       </c>
       <c r="K11" s="2"/>
@@ -2641,24 +2326,24 @@
       <c r="Z11" s="2"/>
     </row>
     <row r="12" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="28" t="s">
+      <c r="A12" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="29"/>
-      <c r="C12" s="30"/>
-      <c r="D12" s="31"/>
-      <c r="E12" s="32"/>
-      <c r="F12" s="3" t="s">
+      <c r="B12" s="19"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="59"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="16">
         <v>4121</v>
       </c>
-      <c r="I12" s="16"/>
-      <c r="J12" s="6"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="3"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
@@ -2677,26 +2362,26 @@
       <c r="Z12" s="2"/>
     </row>
     <row r="13" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="18" t="s">
         <v>4</v>
       </c>
       <c r="B13" s="19"/>
       <c r="C13" s="20"/>
-      <c r="D13" s="34" t="s">
+      <c r="D13" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="7" t="s">
+      <c r="E13" s="54"/>
+      <c r="F13" s="54"/>
+      <c r="G13" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H13" s="8">
+      <c r="H13" s="17">
         <v>890399011</v>
       </c>
       <c r="I13" s="9">
         <v>3</v>
       </c>
-      <c r="J13" s="6"/>
+      <c r="J13" s="3"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
@@ -2715,24 +2400,24 @@
       <c r="Z13" s="2"/>
     </row>
     <row r="14" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="33" t="s">
+      <c r="A14" s="18" t="s">
         <v>7</v>
       </c>
       <c r="B14" s="19"/>
       <c r="C14" s="20"/>
-      <c r="D14" s="18" t="s">
+      <c r="D14" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="19"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="10" t="s">
+      <c r="E14" s="56"/>
+      <c r="F14" s="56"/>
+      <c r="G14" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="H14" s="21">
+      <c r="H14" s="51">
         <v>4121</v>
       </c>
-      <c r="I14" s="22"/>
-      <c r="J14" s="6"/>
+      <c r="I14" s="20"/>
+      <c r="J14" s="3"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
@@ -2751,24 +2436,24 @@
       <c r="Z14" s="2"/>
     </row>
     <row r="15" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="33" t="s">
+      <c r="A15" s="18" t="s">
         <v>10</v>
       </c>
       <c r="B15" s="19"/>
       <c r="C15" s="20"/>
-      <c r="D15" s="35" t="s">
+      <c r="D15" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="19"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="10" t="s">
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="21">
+      <c r="H15" s="51">
         <v>8896744</v>
       </c>
-      <c r="I15" s="22"/>
-      <c r="J15" s="6"/>
+      <c r="I15" s="20"/>
+      <c r="J15" s="3"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
@@ -2787,18 +2472,18 @@
       <c r="Z15" s="2"/>
     </row>
     <row r="16" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="25" t="s">
+      <c r="A16" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="26"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26"/>
-      <c r="H16" s="26"/>
-      <c r="I16" s="27"/>
-      <c r="J16" s="17">
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="5">
         <v>2</v>
       </c>
       <c r="K16" s="2"/>
@@ -2819,23 +2504,23 @@
       <c r="Z16" s="2"/>
     </row>
     <row r="17" spans="1:26" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="36" t="s">
+      <c r="A17" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="37"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="38"/>
-      <c r="G17" s="11" t="s">
+      <c r="B17" s="19"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="53"/>
+      <c r="E17" s="54"/>
+      <c r="F17" s="54"/>
+      <c r="G17" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H17" s="12"/>
-      <c r="I17" s="13"/>
-      <c r="J17" s="6"/>
+      <c r="H17" s="13"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="3"/>
       <c r="K17" s="2"/>
       <c r="L17" s="2"/>
-      <c r="M17" s="14"/>
+      <c r="M17" s="4"/>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
       <c r="P17" s="2"/>
@@ -2851,23 +2536,23 @@
       <c r="Z17" s="2"/>
     </row>
     <row r="18" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="33" t="s">
+      <c r="A18" s="18" t="s">
         <v>16</v>
       </c>
       <c r="B18" s="19"/>
       <c r="C18" s="20"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="10" t="s">
+      <c r="D18" s="47"/>
+      <c r="E18" s="48"/>
+      <c r="F18" s="48"/>
+      <c r="G18" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="H18" s="18"/>
-      <c r="I18" s="22"/>
-      <c r="J18" s="6"/>
+      <c r="H18" s="49"/>
+      <c r="I18" s="20"/>
+      <c r="J18" s="3"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
-      <c r="M18" s="14"/>
+      <c r="M18" s="4"/>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
       <c r="P18" s="2"/>
@@ -2883,23 +2568,23 @@
       <c r="Z18" s="2"/>
     </row>
     <row r="19" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="63" t="s">
+      <c r="A19" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="43"/>
-      <c r="C19" s="41"/>
-      <c r="D19" s="64"/>
-      <c r="E19" s="43"/>
-      <c r="F19" s="41"/>
-      <c r="G19" s="10" t="s">
+      <c r="B19" s="19"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="H19" s="65"/>
-      <c r="I19" s="44"/>
-      <c r="J19" s="6"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="20"/>
+      <c r="J19" s="3"/>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
-      <c r="M19" s="14"/>
+      <c r="M19" s="4"/>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
       <c r="P19" s="2"/>
@@ -2915,18 +2600,18 @@
       <c r="Z19" s="2"/>
     </row>
     <row r="20" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="66" t="s">
+      <c r="A20" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="67"/>
-      <c r="C20" s="67"/>
-      <c r="D20" s="67"/>
-      <c r="E20" s="67"/>
-      <c r="F20" s="67"/>
-      <c r="G20" s="67"/>
-      <c r="H20" s="67"/>
-      <c r="I20" s="68"/>
-      <c r="J20" s="17">
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="20"/>
+      <c r="J20" s="5">
         <v>3</v>
       </c>
       <c r="K20" s="2"/>
@@ -2947,18 +2632,18 @@
       <c r="Z20" s="2"/>
     </row>
     <row r="21" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="69" t="s">
+      <c r="A21" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="67"/>
-      <c r="C21" s="70"/>
-      <c r="D21" s="71"/>
-      <c r="E21" s="72"/>
-      <c r="F21" s="72"/>
-      <c r="G21" s="72"/>
-      <c r="H21" s="72"/>
-      <c r="I21" s="73"/>
-      <c r="J21" s="17"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="26"/>
+      <c r="I21" s="27"/>
+      <c r="J21" s="5"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
@@ -2977,16 +2662,16 @@
       <c r="Z21" s="2"/>
     </row>
     <row r="22" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="49"/>
-      <c r="B22" s="50"/>
-      <c r="C22" s="51"/>
-      <c r="D22" s="74"/>
-      <c r="E22" s="74"/>
-      <c r="F22" s="74"/>
-      <c r="G22" s="74"/>
-      <c r="H22" s="74"/>
-      <c r="I22" s="75"/>
-      <c r="J22" s="17"/>
+      <c r="A22" s="28"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="29"/>
+      <c r="I22" s="30"/>
+      <c r="J22" s="5"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
@@ -3005,18 +2690,18 @@
       <c r="Z22" s="2"/>
     </row>
     <row r="23" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="45" t="s">
+      <c r="A23" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="43"/>
-      <c r="C23" s="41"/>
-      <c r="D23" s="40"/>
-      <c r="E23" s="41"/>
-      <c r="F23" s="42"/>
-      <c r="G23" s="43"/>
-      <c r="H23" s="43"/>
-      <c r="I23" s="44"/>
-      <c r="J23" s="17"/>
+      <c r="B23" s="19"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="39"/>
+      <c r="E23" s="40"/>
+      <c r="F23" s="41"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="29"/>
+      <c r="I23" s="30"/>
+      <c r="J23" s="5"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
       <c r="M23" s="2"/>
@@ -3035,18 +2720,18 @@
       <c r="Z23" s="2"/>
     </row>
     <row r="24" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="54" t="s">
+      <c r="A24" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="24"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="24"/>
-      <c r="H24" s="24"/>
-      <c r="I24" s="55"/>
-      <c r="J24" s="17">
+      <c r="B24" s="46"/>
+      <c r="C24" s="46"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="46"/>
+      <c r="G24" s="46"/>
+      <c r="H24" s="46"/>
+      <c r="I24" s="20"/>
+      <c r="J24" s="5">
         <v>4</v>
       </c>
       <c r="K24" s="2"/>
@@ -3067,20 +2752,20 @@
       <c r="Z24" s="2"/>
     </row>
     <row r="25" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="46" t="s">
+      <c r="A25" s="43" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="47"/>
-      <c r="C25" s="48"/>
-      <c r="D25" s="52"/>
-      <c r="E25" s="47"/>
-      <c r="F25" s="48"/>
-      <c r="G25" s="15" t="s">
+      <c r="B25" s="26"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="45"/>
+      <c r="G25" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="H25" s="58"/>
-      <c r="I25" s="22"/>
-      <c r="J25" s="17"/>
+      <c r="H25" s="34"/>
+      <c r="I25" s="20"/>
+      <c r="J25" s="5"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
@@ -3099,18 +2784,18 @@
       <c r="Z25" s="2"/>
     </row>
     <row r="26" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="49"/>
-      <c r="B26" s="50"/>
-      <c r="C26" s="51"/>
-      <c r="D26" s="53"/>
-      <c r="E26" s="50"/>
-      <c r="F26" s="51"/>
-      <c r="G26" s="15" t="s">
+      <c r="A26" s="28"/>
+      <c r="B26" s="29"/>
+      <c r="C26" s="30"/>
+      <c r="D26" s="40"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="45"/>
+      <c r="G26" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="H26" s="58"/>
-      <c r="I26" s="22"/>
-      <c r="J26" s="17"/>
+      <c r="H26" s="34"/>
+      <c r="I26" s="20"/>
+      <c r="J26" s="5"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
@@ -3129,18 +2814,18 @@
       <c r="Z26" s="2"/>
     </row>
     <row r="27" spans="1:26" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="56" t="s">
+      <c r="A27" s="32" t="s">
         <v>27</v>
       </c>
       <c r="B27" s="19"/>
       <c r="C27" s="20"/>
-      <c r="D27" s="59"/>
-      <c r="E27" s="60"/>
-      <c r="F27" s="60"/>
-      <c r="G27" s="60"/>
-      <c r="H27" s="60"/>
-      <c r="I27" s="61"/>
-      <c r="J27" s="17"/>
+      <c r="D27" s="35"/>
+      <c r="E27" s="36"/>
+      <c r="F27" s="36"/>
+      <c r="G27" s="36"/>
+      <c r="H27" s="36"/>
+      <c r="I27" s="37"/>
+      <c r="J27" s="5"/>
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
       <c r="M27" s="2"/>
@@ -3159,18 +2844,18 @@
       <c r="Z27" s="2"/>
     </row>
     <row r="28" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="57" t="s">
+      <c r="A28" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="43"/>
-      <c r="C28" s="41"/>
-      <c r="D28" s="40"/>
-      <c r="E28" s="41"/>
-      <c r="F28" s="62"/>
-      <c r="G28" s="43"/>
-      <c r="H28" s="43"/>
-      <c r="I28" s="44"/>
-      <c r="J28" s="17"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="38"/>
+      <c r="G28" s="19"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="20"/>
+      <c r="J28" s="5"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
@@ -3198,7 +2883,7 @@
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
       <c r="I29" s="2"/>
-      <c r="J29" s="6"/>
+      <c r="J29" s="3"/>
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
       <c r="M29" s="2"/>
@@ -3226,7 +2911,7 @@
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
-      <c r="J30" s="6"/>
+      <c r="J30" s="3"/>
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
       <c r="M30" s="2"/>
@@ -3254,7 +2939,7 @@
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
-      <c r="J31" s="6"/>
+      <c r="J31" s="3"/>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
       <c r="M31" s="2"/>
@@ -3282,7 +2967,7 @@
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
-      <c r="J32" s="6"/>
+      <c r="J32" s="3"/>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
       <c r="M32" s="2"/>
@@ -3310,7 +2995,7 @@
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
-      <c r="J33" s="6"/>
+      <c r="J33" s="3"/>
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
       <c r="M33" s="2"/>
@@ -3338,7 +3023,7 @@
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
-      <c r="J34" s="6"/>
+      <c r="J34" s="3"/>
       <c r="K34" s="2"/>
       <c r="L34" s="2"/>
       <c r="M34" s="2"/>
@@ -3366,7 +3051,7 @@
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
-      <c r="J35" s="6"/>
+      <c r="J35" s="3"/>
       <c r="K35" s="2"/>
       <c r="L35" s="2"/>
       <c r="M35" s="2"/>
@@ -3394,7 +3079,7 @@
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
-      <c r="J36" s="6"/>
+      <c r="J36" s="3"/>
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
       <c r="M36" s="2"/>
@@ -3422,7 +3107,7 @@
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
-      <c r="J37" s="6"/>
+      <c r="J37" s="3"/>
       <c r="K37" s="2"/>
       <c r="L37" s="2"/>
       <c r="M37" s="2"/>
@@ -3450,7 +3135,7 @@
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
-      <c r="J38" s="6"/>
+      <c r="J38" s="3"/>
       <c r="K38" s="2"/>
       <c r="L38" s="2"/>
       <c r="M38" s="2"/>
@@ -3478,7 +3163,7 @@
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
-      <c r="J39" s="6"/>
+      <c r="J39" s="3"/>
       <c r="K39" s="2"/>
       <c r="L39" s="2"/>
       <c r="M39" s="2"/>
@@ -3506,7 +3191,7 @@
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
-      <c r="J40" s="6"/>
+      <c r="J40" s="3"/>
       <c r="K40" s="2"/>
       <c r="L40" s="2"/>
       <c r="M40" s="2"/>
@@ -3534,7 +3219,7 @@
       <c r="G41" s="2"/>
       <c r="H41" s="2"/>
       <c r="I41" s="2"/>
-      <c r="J41" s="6"/>
+      <c r="J41" s="3"/>
       <c r="K41" s="2"/>
       <c r="L41" s="2"/>
       <c r="M41" s="2"/>
@@ -3562,7 +3247,7 @@
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
-      <c r="J42" s="6"/>
+      <c r="J42" s="3"/>
       <c r="K42" s="2"/>
       <c r="L42" s="2"/>
       <c r="M42" s="2"/>
@@ -3590,7 +3275,7 @@
       <c r="G43" s="2"/>
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
-      <c r="J43" s="6"/>
+      <c r="J43" s="3"/>
       <c r="K43" s="2"/>
       <c r="L43" s="2"/>
       <c r="M43" s="2"/>
@@ -3618,7 +3303,7 @@
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
       <c r="I44" s="2"/>
-      <c r="J44" s="6"/>
+      <c r="J44" s="3"/>
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
       <c r="M44" s="2"/>
@@ -3646,7 +3331,7 @@
       <c r="G45" s="2"/>
       <c r="H45" s="2"/>
       <c r="I45" s="2"/>
-      <c r="J45" s="6"/>
+      <c r="J45" s="3"/>
       <c r="K45" s="2"/>
       <c r="L45" s="2"/>
       <c r="M45" s="2"/>
@@ -3674,7 +3359,7 @@
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
       <c r="I46" s="2"/>
-      <c r="J46" s="6"/>
+      <c r="J46" s="3"/>
       <c r="K46" s="2"/>
       <c r="L46" s="2"/>
       <c r="M46" s="2"/>
@@ -3702,7 +3387,7 @@
       <c r="G47" s="2"/>
       <c r="H47" s="2"/>
       <c r="I47" s="2"/>
-      <c r="J47" s="6"/>
+      <c r="J47" s="3"/>
       <c r="K47" s="2"/>
       <c r="L47" s="2"/>
       <c r="M47" s="2"/>
@@ -3730,7 +3415,7 @@
       <c r="G48" s="2"/>
       <c r="H48" s="2"/>
       <c r="I48" s="2"/>
-      <c r="J48" s="6"/>
+      <c r="J48" s="3"/>
       <c r="K48" s="2"/>
       <c r="L48" s="2"/>
       <c r="M48" s="2"/>
@@ -3758,7 +3443,7 @@
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
       <c r="I49" s="2"/>
-      <c r="J49" s="6"/>
+      <c r="J49" s="3"/>
       <c r="K49" s="2"/>
       <c r="L49" s="2"/>
       <c r="M49" s="2"/>
@@ -3786,7 +3471,7 @@
       <c r="G50" s="2"/>
       <c r="H50" s="2"/>
       <c r="I50" s="2"/>
-      <c r="J50" s="6"/>
+      <c r="J50" s="3"/>
       <c r="K50" s="2"/>
       <c r="L50" s="2"/>
       <c r="M50" s="2"/>
@@ -3814,7 +3499,7 @@
       <c r="G51" s="2"/>
       <c r="H51" s="2"/>
       <c r="I51" s="2"/>
-      <c r="J51" s="6"/>
+      <c r="J51" s="3"/>
       <c r="K51" s="2"/>
       <c r="L51" s="2"/>
       <c r="M51" s="2"/>
@@ -3842,7 +3527,7 @@
       <c r="G52" s="2"/>
       <c r="H52" s="2"/>
       <c r="I52" s="2"/>
-      <c r="J52" s="6"/>
+      <c r="J52" s="3"/>
       <c r="K52" s="2"/>
       <c r="L52" s="2"/>
       <c r="M52" s="2"/>
@@ -3870,7 +3555,7 @@
       <c r="G53" s="2"/>
       <c r="H53" s="2"/>
       <c r="I53" s="2"/>
-      <c r="J53" s="6"/>
+      <c r="J53" s="3"/>
       <c r="K53" s="2"/>
       <c r="L53" s="2"/>
       <c r="M53" s="2"/>
@@ -3898,7 +3583,7 @@
       <c r="G54" s="2"/>
       <c r="H54" s="2"/>
       <c r="I54" s="2"/>
-      <c r="J54" s="6"/>
+      <c r="J54" s="3"/>
       <c r="K54" s="2"/>
       <c r="L54" s="2"/>
       <c r="M54" s="2"/>
@@ -3926,7 +3611,7 @@
       <c r="G55" s="2"/>
       <c r="H55" s="2"/>
       <c r="I55" s="2"/>
-      <c r="J55" s="6"/>
+      <c r="J55" s="3"/>
       <c r="K55" s="2"/>
       <c r="L55" s="2"/>
       <c r="M55" s="2"/>
@@ -3954,7 +3639,7 @@
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
       <c r="I56" s="2"/>
-      <c r="J56" s="6"/>
+      <c r="J56" s="3"/>
       <c r="K56" s="2"/>
       <c r="L56" s="2"/>
       <c r="M56" s="2"/>
@@ -3982,7 +3667,7 @@
       <c r="G57" s="2"/>
       <c r="H57" s="2"/>
       <c r="I57" s="2"/>
-      <c r="J57" s="6"/>
+      <c r="J57" s="3"/>
       <c r="K57" s="2"/>
       <c r="L57" s="2"/>
       <c r="M57" s="2"/>
@@ -4010,7 +3695,7 @@
       <c r="G58" s="2"/>
       <c r="H58" s="2"/>
       <c r="I58" s="2"/>
-      <c r="J58" s="6"/>
+      <c r="J58" s="3"/>
       <c r="K58" s="2"/>
       <c r="L58" s="2"/>
       <c r="M58" s="2"/>
@@ -4038,7 +3723,7 @@
       <c r="G59" s="2"/>
       <c r="H59" s="2"/>
       <c r="I59" s="2"/>
-      <c r="J59" s="6"/>
+      <c r="J59" s="3"/>
       <c r="K59" s="2"/>
       <c r="L59" s="2"/>
       <c r="M59" s="2"/>
@@ -4066,7 +3751,7 @@
       <c r="G60" s="2"/>
       <c r="H60" s="2"/>
       <c r="I60" s="2"/>
-      <c r="J60" s="6"/>
+      <c r="J60" s="3"/>
       <c r="K60" s="2"/>
       <c r="L60" s="2"/>
       <c r="M60" s="2"/>
@@ -4094,7 +3779,7 @@
       <c r="G61" s="2"/>
       <c r="H61" s="2"/>
       <c r="I61" s="2"/>
-      <c r="J61" s="6"/>
+      <c r="J61" s="3"/>
       <c r="K61" s="2"/>
       <c r="L61" s="2"/>
       <c r="M61" s="2"/>
@@ -4122,7 +3807,7 @@
       <c r="G62" s="2"/>
       <c r="H62" s="2"/>
       <c r="I62" s="2"/>
-      <c r="J62" s="6"/>
+      <c r="J62" s="3"/>
       <c r="K62" s="2"/>
       <c r="L62" s="2"/>
       <c r="M62" s="2"/>
@@ -4150,7 +3835,7 @@
       <c r="G63" s="2"/>
       <c r="H63" s="2"/>
       <c r="I63" s="2"/>
-      <c r="J63" s="6"/>
+      <c r="J63" s="3"/>
       <c r="K63" s="2"/>
       <c r="L63" s="2"/>
       <c r="M63" s="2"/>
@@ -4178,7 +3863,7 @@
       <c r="G64" s="2"/>
       <c r="H64" s="2"/>
       <c r="I64" s="2"/>
-      <c r="J64" s="6"/>
+      <c r="J64" s="3"/>
       <c r="K64" s="2"/>
       <c r="L64" s="2"/>
       <c r="M64" s="2"/>
@@ -4206,7 +3891,7 @@
       <c r="G65" s="2"/>
       <c r="H65" s="2"/>
       <c r="I65" s="2"/>
-      <c r="J65" s="6"/>
+      <c r="J65" s="3"/>
       <c r="K65" s="2"/>
       <c r="L65" s="2"/>
       <c r="M65" s="2"/>
@@ -4234,7 +3919,7 @@
       <c r="G66" s="2"/>
       <c r="H66" s="2"/>
       <c r="I66" s="2"/>
-      <c r="J66" s="6"/>
+      <c r="J66" s="3"/>
       <c r="K66" s="2"/>
       <c r="L66" s="2"/>
       <c r="M66" s="2"/>
@@ -4262,7 +3947,7 @@
       <c r="G67" s="2"/>
       <c r="H67" s="2"/>
       <c r="I67" s="2"/>
-      <c r="J67" s="6"/>
+      <c r="J67" s="3"/>
       <c r="K67" s="2"/>
       <c r="L67" s="2"/>
       <c r="M67" s="2"/>
@@ -4290,7 +3975,7 @@
       <c r="G68" s="2"/>
       <c r="H68" s="2"/>
       <c r="I68" s="2"/>
-      <c r="J68" s="6"/>
+      <c r="J68" s="3"/>
       <c r="K68" s="2"/>
       <c r="L68" s="2"/>
       <c r="M68" s="2"/>
@@ -4318,7 +4003,7 @@
       <c r="G69" s="2"/>
       <c r="H69" s="2"/>
       <c r="I69" s="2"/>
-      <c r="J69" s="6"/>
+      <c r="J69" s="3"/>
       <c r="K69" s="2"/>
       <c r="L69" s="2"/>
       <c r="M69" s="2"/>
@@ -4346,7 +4031,7 @@
       <c r="G70" s="2"/>
       <c r="H70" s="2"/>
       <c r="I70" s="2"/>
-      <c r="J70" s="6"/>
+      <c r="J70" s="3"/>
       <c r="K70" s="2"/>
       <c r="L70" s="2"/>
       <c r="M70" s="2"/>
@@ -4374,7 +4059,7 @@
       <c r="G71" s="2"/>
       <c r="H71" s="2"/>
       <c r="I71" s="2"/>
-      <c r="J71" s="6"/>
+      <c r="J71" s="3"/>
       <c r="K71" s="2"/>
       <c r="L71" s="2"/>
       <c r="M71" s="2"/>
@@ -4402,7 +4087,7 @@
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
       <c r="I72" s="2"/>
-      <c r="J72" s="6"/>
+      <c r="J72" s="3"/>
       <c r="K72" s="2"/>
       <c r="L72" s="2"/>
       <c r="M72" s="2"/>
@@ -4430,7 +4115,7 @@
       <c r="G73" s="2"/>
       <c r="H73" s="2"/>
       <c r="I73" s="2"/>
-      <c r="J73" s="6"/>
+      <c r="J73" s="3"/>
       <c r="K73" s="2"/>
       <c r="L73" s="2"/>
       <c r="M73" s="2"/>
@@ -4458,7 +4143,7 @@
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
       <c r="I74" s="2"/>
-      <c r="J74" s="6"/>
+      <c r="J74" s="3"/>
       <c r="K74" s="2"/>
       <c r="L74" s="2"/>
       <c r="M74" s="2"/>
@@ -4486,7 +4171,7 @@
       <c r="G75" s="2"/>
       <c r="H75" s="2"/>
       <c r="I75" s="2"/>
-      <c r="J75" s="6"/>
+      <c r="J75" s="3"/>
       <c r="K75" s="2"/>
       <c r="L75" s="2"/>
       <c r="M75" s="2"/>
@@ -4514,7 +4199,7 @@
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
       <c r="I76" s="2"/>
-      <c r="J76" s="6"/>
+      <c r="J76" s="3"/>
       <c r="K76" s="2"/>
       <c r="L76" s="2"/>
       <c r="M76" s="2"/>
@@ -4542,7 +4227,7 @@
       <c r="G77" s="2"/>
       <c r="H77" s="2"/>
       <c r="I77" s="2"/>
-      <c r="J77" s="6"/>
+      <c r="J77" s="3"/>
       <c r="K77" s="2"/>
       <c r="L77" s="2"/>
       <c r="M77" s="2"/>
@@ -4570,7 +4255,7 @@
       <c r="G78" s="2"/>
       <c r="H78" s="2"/>
       <c r="I78" s="2"/>
-      <c r="J78" s="6"/>
+      <c r="J78" s="3"/>
       <c r="K78" s="2"/>
       <c r="L78" s="2"/>
       <c r="M78" s="2"/>
@@ -4598,7 +4283,7 @@
       <c r="G79" s="2"/>
       <c r="H79" s="2"/>
       <c r="I79" s="2"/>
-      <c r="J79" s="6"/>
+      <c r="J79" s="3"/>
       <c r="K79" s="2"/>
       <c r="L79" s="2"/>
       <c r="M79" s="2"/>
@@ -4626,7 +4311,7 @@
       <c r="G80" s="2"/>
       <c r="H80" s="2"/>
       <c r="I80" s="2"/>
-      <c r="J80" s="6"/>
+      <c r="J80" s="3"/>
       <c r="K80" s="2"/>
       <c r="L80" s="2"/>
       <c r="M80" s="2"/>
@@ -4654,7 +4339,7 @@
       <c r="G81" s="2"/>
       <c r="H81" s="2"/>
       <c r="I81" s="2"/>
-      <c r="J81" s="6"/>
+      <c r="J81" s="3"/>
       <c r="K81" s="2"/>
       <c r="L81" s="2"/>
       <c r="M81" s="2"/>
@@ -4682,7 +4367,7 @@
       <c r="G82" s="2"/>
       <c r="H82" s="2"/>
       <c r="I82" s="2"/>
-      <c r="J82" s="6"/>
+      <c r="J82" s="3"/>
       <c r="K82" s="2"/>
       <c r="L82" s="2"/>
       <c r="M82" s="2"/>
@@ -4710,7 +4395,7 @@
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
       <c r="I83" s="2"/>
-      <c r="J83" s="6"/>
+      <c r="J83" s="3"/>
       <c r="K83" s="2"/>
       <c r="L83" s="2"/>
       <c r="M83" s="2"/>
@@ -4738,7 +4423,7 @@
       <c r="G84" s="2"/>
       <c r="H84" s="2"/>
       <c r="I84" s="2"/>
-      <c r="J84" s="6"/>
+      <c r="J84" s="3"/>
       <c r="K84" s="2"/>
       <c r="L84" s="2"/>
       <c r="M84" s="2"/>
@@ -4766,7 +4451,7 @@
       <c r="G85" s="2"/>
       <c r="H85" s="2"/>
       <c r="I85" s="2"/>
-      <c r="J85" s="6"/>
+      <c r="J85" s="3"/>
       <c r="K85" s="2"/>
       <c r="L85" s="2"/>
       <c r="M85" s="2"/>
@@ -4794,7 +4479,7 @@
       <c r="G86" s="2"/>
       <c r="H86" s="2"/>
       <c r="I86" s="2"/>
-      <c r="J86" s="6"/>
+      <c r="J86" s="3"/>
       <c r="K86" s="2"/>
       <c r="L86" s="2"/>
       <c r="M86" s="2"/>
@@ -4822,7 +4507,7 @@
       <c r="G87" s="2"/>
       <c r="H87" s="2"/>
       <c r="I87" s="2"/>
-      <c r="J87" s="6"/>
+      <c r="J87" s="3"/>
       <c r="K87" s="2"/>
       <c r="L87" s="2"/>
       <c r="M87" s="2"/>
@@ -4850,7 +4535,7 @@
       <c r="G88" s="2"/>
       <c r="H88" s="2"/>
       <c r="I88" s="2"/>
-      <c r="J88" s="6"/>
+      <c r="J88" s="3"/>
       <c r="K88" s="2"/>
       <c r="L88" s="2"/>
       <c r="M88" s="2"/>
@@ -4878,7 +4563,7 @@
       <c r="G89" s="2"/>
       <c r="H89" s="2"/>
       <c r="I89" s="2"/>
-      <c r="J89" s="6"/>
+      <c r="J89" s="3"/>
       <c r="K89" s="2"/>
       <c r="L89" s="2"/>
       <c r="M89" s="2"/>
@@ -4906,7 +4591,7 @@
       <c r="G90" s="2"/>
       <c r="H90" s="2"/>
       <c r="I90" s="2"/>
-      <c r="J90" s="6"/>
+      <c r="J90" s="3"/>
       <c r="K90" s="2"/>
       <c r="L90" s="2"/>
       <c r="M90" s="2"/>
@@ -4934,7 +4619,7 @@
       <c r="G91" s="2"/>
       <c r="H91" s="2"/>
       <c r="I91" s="2"/>
-      <c r="J91" s="6"/>
+      <c r="J91" s="3"/>
       <c r="K91" s="2"/>
       <c r="L91" s="2"/>
       <c r="M91" s="2"/>
@@ -4962,7 +4647,7 @@
       <c r="G92" s="2"/>
       <c r="H92" s="2"/>
       <c r="I92" s="2"/>
-      <c r="J92" s="6"/>
+      <c r="J92" s="3"/>
       <c r="K92" s="2"/>
       <c r="L92" s="2"/>
       <c r="M92" s="2"/>
@@ -4990,7 +4675,7 @@
       <c r="G93" s="2"/>
       <c r="H93" s="2"/>
       <c r="I93" s="2"/>
-      <c r="J93" s="6"/>
+      <c r="J93" s="3"/>
       <c r="K93" s="2"/>
       <c r="L93" s="2"/>
       <c r="M93" s="2"/>
@@ -5018,7 +4703,7 @@
       <c r="G94" s="2"/>
       <c r="H94" s="2"/>
       <c r="I94" s="2"/>
-      <c r="J94" s="6"/>
+      <c r="J94" s="3"/>
       <c r="K94" s="2"/>
       <c r="L94" s="2"/>
       <c r="M94" s="2"/>
@@ -5046,7 +4731,7 @@
       <c r="G95" s="2"/>
       <c r="H95" s="2"/>
       <c r="I95" s="2"/>
-      <c r="J95" s="6"/>
+      <c r="J95" s="3"/>
       <c r="K95" s="2"/>
       <c r="L95" s="2"/>
       <c r="M95" s="2"/>
@@ -5074,7 +4759,7 @@
       <c r="G96" s="2"/>
       <c r="H96" s="2"/>
       <c r="I96" s="2"/>
-      <c r="J96" s="6"/>
+      <c r="J96" s="3"/>
       <c r="K96" s="2"/>
       <c r="L96" s="2"/>
       <c r="M96" s="2"/>
@@ -5102,7 +4787,7 @@
       <c r="G97" s="2"/>
       <c r="H97" s="2"/>
       <c r="I97" s="2"/>
-      <c r="J97" s="6"/>
+      <c r="J97" s="3"/>
       <c r="K97" s="2"/>
       <c r="L97" s="2"/>
       <c r="M97" s="2"/>
@@ -5130,7 +4815,7 @@
       <c r="G98" s="2"/>
       <c r="H98" s="2"/>
       <c r="I98" s="2"/>
-      <c r="J98" s="6"/>
+      <c r="J98" s="3"/>
       <c r="K98" s="2"/>
       <c r="L98" s="2"/>
       <c r="M98" s="2"/>
@@ -5158,7 +4843,7 @@
       <c r="G99" s="2"/>
       <c r="H99" s="2"/>
       <c r="I99" s="2"/>
-      <c r="J99" s="6"/>
+      <c r="J99" s="3"/>
       <c r="K99" s="2"/>
       <c r="L99" s="2"/>
       <c r="M99" s="2"/>
@@ -5186,7 +4871,7 @@
       <c r="G100" s="2"/>
       <c r="H100" s="2"/>
       <c r="I100" s="2"/>
-      <c r="J100" s="6"/>
+      <c r="J100" s="3"/>
       <c r="K100" s="2"/>
       <c r="L100" s="2"/>
       <c r="M100" s="2"/>
@@ -5214,7 +4899,7 @@
       <c r="G101" s="2"/>
       <c r="H101" s="2"/>
       <c r="I101" s="2"/>
-      <c r="J101" s="6"/>
+      <c r="J101" s="3"/>
       <c r="K101" s="2"/>
       <c r="L101" s="2"/>
       <c r="M101" s="2"/>
@@ -5242,7 +4927,7 @@
       <c r="G102" s="2"/>
       <c r="H102" s="2"/>
       <c r="I102" s="2"/>
-      <c r="J102" s="6"/>
+      <c r="J102" s="3"/>
       <c r="K102" s="2"/>
       <c r="L102" s="2"/>
       <c r="M102" s="2"/>
@@ -5270,7 +4955,7 @@
       <c r="G103" s="2"/>
       <c r="H103" s="2"/>
       <c r="I103" s="2"/>
-      <c r="J103" s="6"/>
+      <c r="J103" s="3"/>
       <c r="K103" s="2"/>
       <c r="L103" s="2"/>
       <c r="M103" s="2"/>
@@ -5298,7 +4983,7 @@
       <c r="G104" s="2"/>
       <c r="H104" s="2"/>
       <c r="I104" s="2"/>
-      <c r="J104" s="6"/>
+      <c r="J104" s="3"/>
       <c r="K104" s="2"/>
       <c r="L104" s="2"/>
       <c r="M104" s="2"/>
@@ -5326,7 +5011,7 @@
       <c r="G105" s="2"/>
       <c r="H105" s="2"/>
       <c r="I105" s="2"/>
-      <c r="J105" s="6"/>
+      <c r="J105" s="3"/>
       <c r="K105" s="2"/>
       <c r="L105" s="2"/>
       <c r="M105" s="2"/>
@@ -5354,7 +5039,7 @@
       <c r="G106" s="2"/>
       <c r="H106" s="2"/>
       <c r="I106" s="2"/>
-      <c r="J106" s="6"/>
+      <c r="J106" s="3"/>
       <c r="K106" s="2"/>
       <c r="L106" s="2"/>
       <c r="M106" s="2"/>
@@ -5382,7 +5067,7 @@
       <c r="G107" s="2"/>
       <c r="H107" s="2"/>
       <c r="I107" s="2"/>
-      <c r="J107" s="6"/>
+      <c r="J107" s="3"/>
       <c r="K107" s="2"/>
       <c r="L107" s="2"/>
       <c r="M107" s="2"/>
@@ -5410,7 +5095,7 @@
       <c r="G108" s="2"/>
       <c r="H108" s="2"/>
       <c r="I108" s="2"/>
-      <c r="J108" s="6"/>
+      <c r="J108" s="3"/>
       <c r="K108" s="2"/>
       <c r="L108" s="2"/>
       <c r="M108" s="2"/>
@@ -5438,7 +5123,7 @@
       <c r="G109" s="2"/>
       <c r="H109" s="2"/>
       <c r="I109" s="2"/>
-      <c r="J109" s="6"/>
+      <c r="J109" s="3"/>
       <c r="K109" s="2"/>
       <c r="L109" s="2"/>
       <c r="M109" s="2"/>
@@ -5466,7 +5151,7 @@
       <c r="G110" s="2"/>
       <c r="H110" s="2"/>
       <c r="I110" s="2"/>
-      <c r="J110" s="6"/>
+      <c r="J110" s="3"/>
       <c r="K110" s="2"/>
       <c r="L110" s="2"/>
       <c r="M110" s="2"/>
@@ -5494,7 +5179,7 @@
       <c r="G111" s="2"/>
       <c r="H111" s="2"/>
       <c r="I111" s="2"/>
-      <c r="J111" s="6"/>
+      <c r="J111" s="3"/>
       <c r="K111" s="2"/>
       <c r="L111" s="2"/>
       <c r="M111" s="2"/>
@@ -5522,7 +5207,7 @@
       <c r="G112" s="2"/>
       <c r="H112" s="2"/>
       <c r="I112" s="2"/>
-      <c r="J112" s="6"/>
+      <c r="J112" s="3"/>
       <c r="K112" s="2"/>
       <c r="L112" s="2"/>
       <c r="M112" s="2"/>
@@ -5550,7 +5235,7 @@
       <c r="G113" s="2"/>
       <c r="H113" s="2"/>
       <c r="I113" s="2"/>
-      <c r="J113" s="6"/>
+      <c r="J113" s="3"/>
       <c r="K113" s="2"/>
       <c r="L113" s="2"/>
       <c r="M113" s="2"/>
@@ -5578,7 +5263,7 @@
       <c r="G114" s="2"/>
       <c r="H114" s="2"/>
       <c r="I114" s="2"/>
-      <c r="J114" s="6"/>
+      <c r="J114" s="3"/>
       <c r="K114" s="2"/>
       <c r="L114" s="2"/>
       <c r="M114" s="2"/>
@@ -5606,7 +5291,7 @@
       <c r="G115" s="2"/>
       <c r="H115" s="2"/>
       <c r="I115" s="2"/>
-      <c r="J115" s="6"/>
+      <c r="J115" s="3"/>
       <c r="K115" s="2"/>
       <c r="L115" s="2"/>
       <c r="M115" s="2"/>
@@ -5634,7 +5319,7 @@
       <c r="G116" s="2"/>
       <c r="H116" s="2"/>
       <c r="I116" s="2"/>
-      <c r="J116" s="6"/>
+      <c r="J116" s="3"/>
       <c r="K116" s="2"/>
       <c r="L116" s="2"/>
       <c r="M116" s="2"/>
@@ -5662,7 +5347,7 @@
       <c r="G117" s="2"/>
       <c r="H117" s="2"/>
       <c r="I117" s="2"/>
-      <c r="J117" s="6"/>
+      <c r="J117" s="3"/>
       <c r="K117" s="2"/>
       <c r="L117" s="2"/>
       <c r="M117" s="2"/>
@@ -5690,7 +5375,7 @@
       <c r="G118" s="2"/>
       <c r="H118" s="2"/>
       <c r="I118" s="2"/>
-      <c r="J118" s="6"/>
+      <c r="J118" s="3"/>
       <c r="K118" s="2"/>
       <c r="L118" s="2"/>
       <c r="M118" s="2"/>
@@ -5718,7 +5403,7 @@
       <c r="G119" s="2"/>
       <c r="H119" s="2"/>
       <c r="I119" s="2"/>
-      <c r="J119" s="6"/>
+      <c r="J119" s="3"/>
       <c r="K119" s="2"/>
       <c r="L119" s="2"/>
       <c r="M119" s="2"/>
@@ -5746,7 +5431,7 @@
       <c r="G120" s="2"/>
       <c r="H120" s="2"/>
       <c r="I120" s="2"/>
-      <c r="J120" s="6"/>
+      <c r="J120" s="3"/>
       <c r="K120" s="2"/>
       <c r="L120" s="2"/>
       <c r="M120" s="2"/>
@@ -5774,7 +5459,7 @@
       <c r="G121" s="2"/>
       <c r="H121" s="2"/>
       <c r="I121" s="2"/>
-      <c r="J121" s="6"/>
+      <c r="J121" s="3"/>
       <c r="K121" s="2"/>
       <c r="L121" s="2"/>
       <c r="M121" s="2"/>
@@ -5802,7 +5487,7 @@
       <c r="G122" s="2"/>
       <c r="H122" s="2"/>
       <c r="I122" s="2"/>
-      <c r="J122" s="6"/>
+      <c r="J122" s="3"/>
       <c r="K122" s="2"/>
       <c r="L122" s="2"/>
       <c r="M122" s="2"/>
@@ -5830,7 +5515,7 @@
       <c r="G123" s="2"/>
       <c r="H123" s="2"/>
       <c r="I123" s="2"/>
-      <c r="J123" s="6"/>
+      <c r="J123" s="3"/>
       <c r="K123" s="2"/>
       <c r="L123" s="2"/>
       <c r="M123" s="2"/>
@@ -5858,7 +5543,7 @@
       <c r="G124" s="2"/>
       <c r="H124" s="2"/>
       <c r="I124" s="2"/>
-      <c r="J124" s="6"/>
+      <c r="J124" s="3"/>
       <c r="K124" s="2"/>
       <c r="L124" s="2"/>
       <c r="M124" s="2"/>
@@ -5886,7 +5571,7 @@
       <c r="G125" s="2"/>
       <c r="H125" s="2"/>
       <c r="I125" s="2"/>
-      <c r="J125" s="6"/>
+      <c r="J125" s="3"/>
       <c r="K125" s="2"/>
       <c r="L125" s="2"/>
       <c r="M125" s="2"/>
@@ -5914,7 +5599,7 @@
       <c r="G126" s="2"/>
       <c r="H126" s="2"/>
       <c r="I126" s="2"/>
-      <c r="J126" s="6"/>
+      <c r="J126" s="3"/>
       <c r="K126" s="2"/>
       <c r="L126" s="2"/>
       <c r="M126" s="2"/>
@@ -5942,7 +5627,7 @@
       <c r="G127" s="2"/>
       <c r="H127" s="2"/>
       <c r="I127" s="2"/>
-      <c r="J127" s="6"/>
+      <c r="J127" s="3"/>
       <c r="K127" s="2"/>
       <c r="L127" s="2"/>
       <c r="M127" s="2"/>
@@ -5970,7 +5655,7 @@
       <c r="G128" s="2"/>
       <c r="H128" s="2"/>
       <c r="I128" s="2"/>
-      <c r="J128" s="6"/>
+      <c r="J128" s="3"/>
       <c r="K128" s="2"/>
       <c r="L128" s="2"/>
       <c r="M128" s="2"/>
@@ -5998,7 +5683,7 @@
       <c r="G129" s="2"/>
       <c r="H129" s="2"/>
       <c r="I129" s="2"/>
-      <c r="J129" s="6"/>
+      <c r="J129" s="3"/>
       <c r="K129" s="2"/>
       <c r="L129" s="2"/>
       <c r="M129" s="2"/>
@@ -6026,7 +5711,7 @@
       <c r="G130" s="2"/>
       <c r="H130" s="2"/>
       <c r="I130" s="2"/>
-      <c r="J130" s="6"/>
+      <c r="J130" s="3"/>
       <c r="K130" s="2"/>
       <c r="L130" s="2"/>
       <c r="M130" s="2"/>
@@ -6054,7 +5739,7 @@
       <c r="G131" s="2"/>
       <c r="H131" s="2"/>
       <c r="I131" s="2"/>
-      <c r="J131" s="6"/>
+      <c r="J131" s="3"/>
       <c r="K131" s="2"/>
       <c r="L131" s="2"/>
       <c r="M131" s="2"/>
@@ -6082,7 +5767,7 @@
       <c r="G132" s="2"/>
       <c r="H132" s="2"/>
       <c r="I132" s="2"/>
-      <c r="J132" s="6"/>
+      <c r="J132" s="3"/>
       <c r="K132" s="2"/>
       <c r="L132" s="2"/>
       <c r="M132" s="2"/>
@@ -6110,7 +5795,7 @@
       <c r="G133" s="2"/>
       <c r="H133" s="2"/>
       <c r="I133" s="2"/>
-      <c r="J133" s="6"/>
+      <c r="J133" s="3"/>
       <c r="K133" s="2"/>
       <c r="L133" s="2"/>
       <c r="M133" s="2"/>
@@ -6138,7 +5823,7 @@
       <c r="G134" s="2"/>
       <c r="H134" s="2"/>
       <c r="I134" s="2"/>
-      <c r="J134" s="6"/>
+      <c r="J134" s="3"/>
       <c r="K134" s="2"/>
       <c r="L134" s="2"/>
       <c r="M134" s="2"/>
@@ -6166,7 +5851,7 @@
       <c r="G135" s="2"/>
       <c r="H135" s="2"/>
       <c r="I135" s="2"/>
-      <c r="J135" s="6"/>
+      <c r="J135" s="3"/>
       <c r="K135" s="2"/>
       <c r="L135" s="2"/>
       <c r="M135" s="2"/>
@@ -6194,7 +5879,7 @@
       <c r="G136" s="2"/>
       <c r="H136" s="2"/>
       <c r="I136" s="2"/>
-      <c r="J136" s="6"/>
+      <c r="J136" s="3"/>
       <c r="K136" s="2"/>
       <c r="L136" s="2"/>
       <c r="M136" s="2"/>
@@ -6222,7 +5907,7 @@
       <c r="G137" s="2"/>
       <c r="H137" s="2"/>
       <c r="I137" s="2"/>
-      <c r="J137" s="6"/>
+      <c r="J137" s="3"/>
       <c r="K137" s="2"/>
       <c r="L137" s="2"/>
       <c r="M137" s="2"/>
@@ -6250,7 +5935,7 @@
       <c r="G138" s="2"/>
       <c r="H138" s="2"/>
       <c r="I138" s="2"/>
-      <c r="J138" s="6"/>
+      <c r="J138" s="3"/>
       <c r="K138" s="2"/>
       <c r="L138" s="2"/>
       <c r="M138" s="2"/>
@@ -6278,7 +5963,7 @@
       <c r="G139" s="2"/>
       <c r="H139" s="2"/>
       <c r="I139" s="2"/>
-      <c r="J139" s="6"/>
+      <c r="J139" s="3"/>
       <c r="K139" s="2"/>
       <c r="L139" s="2"/>
       <c r="M139" s="2"/>
@@ -6306,7 +5991,7 @@
       <c r="G140" s="2"/>
       <c r="H140" s="2"/>
       <c r="I140" s="2"/>
-      <c r="J140" s="6"/>
+      <c r="J140" s="3"/>
       <c r="K140" s="2"/>
       <c r="L140" s="2"/>
       <c r="M140" s="2"/>
@@ -6334,7 +6019,7 @@
       <c r="G141" s="2"/>
       <c r="H141" s="2"/>
       <c r="I141" s="2"/>
-      <c r="J141" s="6"/>
+      <c r="J141" s="3"/>
       <c r="K141" s="2"/>
       <c r="L141" s="2"/>
       <c r="M141" s="2"/>
@@ -6362,7 +6047,7 @@
       <c r="G142" s="2"/>
       <c r="H142" s="2"/>
       <c r="I142" s="2"/>
-      <c r="J142" s="6"/>
+      <c r="J142" s="3"/>
       <c r="K142" s="2"/>
       <c r="L142" s="2"/>
       <c r="M142" s="2"/>
@@ -6390,7 +6075,7 @@
       <c r="G143" s="2"/>
       <c r="H143" s="2"/>
       <c r="I143" s="2"/>
-      <c r="J143" s="6"/>
+      <c r="J143" s="3"/>
       <c r="K143" s="2"/>
       <c r="L143" s="2"/>
       <c r="M143" s="2"/>
@@ -6418,7 +6103,7 @@
       <c r="G144" s="2"/>
       <c r="H144" s="2"/>
       <c r="I144" s="2"/>
-      <c r="J144" s="6"/>
+      <c r="J144" s="3"/>
       <c r="K144" s="2"/>
       <c r="L144" s="2"/>
       <c r="M144" s="2"/>
@@ -6446,7 +6131,7 @@
       <c r="G145" s="2"/>
       <c r="H145" s="2"/>
       <c r="I145" s="2"/>
-      <c r="J145" s="6"/>
+      <c r="J145" s="3"/>
       <c r="K145" s="2"/>
       <c r="L145" s="2"/>
       <c r="M145" s="2"/>
@@ -6474,7 +6159,7 @@
       <c r="G146" s="2"/>
       <c r="H146" s="2"/>
       <c r="I146" s="2"/>
-      <c r="J146" s="6"/>
+      <c r="J146" s="3"/>
       <c r="K146" s="2"/>
       <c r="L146" s="2"/>
       <c r="M146" s="2"/>
@@ -6502,7 +6187,7 @@
       <c r="G147" s="2"/>
       <c r="H147" s="2"/>
       <c r="I147" s="2"/>
-      <c r="J147" s="6"/>
+      <c r="J147" s="3"/>
       <c r="K147" s="2"/>
       <c r="L147" s="2"/>
       <c r="M147" s="2"/>
@@ -6530,7 +6215,7 @@
       <c r="G148" s="2"/>
       <c r="H148" s="2"/>
       <c r="I148" s="2"/>
-      <c r="J148" s="6"/>
+      <c r="J148" s="3"/>
       <c r="K148" s="2"/>
       <c r="L148" s="2"/>
       <c r="M148" s="2"/>
@@ -6558,7 +6243,7 @@
       <c r="G149" s="2"/>
       <c r="H149" s="2"/>
       <c r="I149" s="2"/>
-      <c r="J149" s="6"/>
+      <c r="J149" s="3"/>
       <c r="K149" s="2"/>
       <c r="L149" s="2"/>
       <c r="M149" s="2"/>
@@ -6586,7 +6271,7 @@
       <c r="G150" s="2"/>
       <c r="H150" s="2"/>
       <c r="I150" s="2"/>
-      <c r="J150" s="6"/>
+      <c r="J150" s="3"/>
       <c r="K150" s="2"/>
       <c r="L150" s="2"/>
       <c r="M150" s="2"/>
@@ -6614,7 +6299,7 @@
       <c r="G151" s="2"/>
       <c r="H151" s="2"/>
       <c r="I151" s="2"/>
-      <c r="J151" s="6"/>
+      <c r="J151" s="3"/>
       <c r="K151" s="2"/>
       <c r="L151" s="2"/>
       <c r="M151" s="2"/>
@@ -6642,7 +6327,7 @@
       <c r="G152" s="2"/>
       <c r="H152" s="2"/>
       <c r="I152" s="2"/>
-      <c r="J152" s="6"/>
+      <c r="J152" s="3"/>
       <c r="K152" s="2"/>
       <c r="L152" s="2"/>
       <c r="M152" s="2"/>
@@ -6670,7 +6355,7 @@
       <c r="G153" s="2"/>
       <c r="H153" s="2"/>
       <c r="I153" s="2"/>
-      <c r="J153" s="6"/>
+      <c r="J153" s="3"/>
       <c r="K153" s="2"/>
       <c r="L153" s="2"/>
       <c r="M153" s="2"/>
@@ -6698,7 +6383,7 @@
       <c r="G154" s="2"/>
       <c r="H154" s="2"/>
       <c r="I154" s="2"/>
-      <c r="J154" s="6"/>
+      <c r="J154" s="3"/>
       <c r="K154" s="2"/>
       <c r="L154" s="2"/>
       <c r="M154" s="2"/>
@@ -6726,7 +6411,7 @@
       <c r="G155" s="2"/>
       <c r="H155" s="2"/>
       <c r="I155" s="2"/>
-      <c r="J155" s="6"/>
+      <c r="J155" s="3"/>
       <c r="K155" s="2"/>
       <c r="L155" s="2"/>
       <c r="M155" s="2"/>
@@ -6754,7 +6439,7 @@
       <c r="G156" s="2"/>
       <c r="H156" s="2"/>
       <c r="I156" s="2"/>
-      <c r="J156" s="6"/>
+      <c r="J156" s="3"/>
       <c r="K156" s="2"/>
       <c r="L156" s="2"/>
       <c r="M156" s="2"/>
@@ -6782,7 +6467,7 @@
       <c r="G157" s="2"/>
       <c r="H157" s="2"/>
       <c r="I157" s="2"/>
-      <c r="J157" s="6"/>
+      <c r="J157" s="3"/>
       <c r="K157" s="2"/>
       <c r="L157" s="2"/>
       <c r="M157" s="2"/>
@@ -6810,7 +6495,7 @@
       <c r="G158" s="2"/>
       <c r="H158" s="2"/>
       <c r="I158" s="2"/>
-      <c r="J158" s="6"/>
+      <c r="J158" s="3"/>
       <c r="K158" s="2"/>
       <c r="L158" s="2"/>
       <c r="M158" s="2"/>
@@ -6838,7 +6523,7 @@
       <c r="G159" s="2"/>
       <c r="H159" s="2"/>
       <c r="I159" s="2"/>
-      <c r="J159" s="6"/>
+      <c r="J159" s="3"/>
       <c r="K159" s="2"/>
       <c r="L159" s="2"/>
       <c r="M159" s="2"/>
@@ -6866,7 +6551,7 @@
       <c r="G160" s="2"/>
       <c r="H160" s="2"/>
       <c r="I160" s="2"/>
-      <c r="J160" s="6"/>
+      <c r="J160" s="3"/>
       <c r="K160" s="2"/>
       <c r="L160" s="2"/>
       <c r="M160" s="2"/>
@@ -6894,7 +6579,7 @@
       <c r="G161" s="2"/>
       <c r="H161" s="2"/>
       <c r="I161" s="2"/>
-      <c r="J161" s="6"/>
+      <c r="J161" s="3"/>
       <c r="K161" s="2"/>
       <c r="L161" s="2"/>
       <c r="M161" s="2"/>
@@ -6922,7 +6607,7 @@
       <c r="G162" s="2"/>
       <c r="H162" s="2"/>
       <c r="I162" s="2"/>
-      <c r="J162" s="6"/>
+      <c r="J162" s="3"/>
       <c r="K162" s="2"/>
       <c r="L162" s="2"/>
       <c r="M162" s="2"/>
@@ -6950,7 +6635,7 @@
       <c r="G163" s="2"/>
       <c r="H163" s="2"/>
       <c r="I163" s="2"/>
-      <c r="J163" s="6"/>
+      <c r="J163" s="3"/>
       <c r="K163" s="2"/>
       <c r="L163" s="2"/>
       <c r="M163" s="2"/>
@@ -6978,7 +6663,7 @@
       <c r="G164" s="2"/>
       <c r="H164" s="2"/>
       <c r="I164" s="2"/>
-      <c r="J164" s="6"/>
+      <c r="J164" s="3"/>
       <c r="K164" s="2"/>
       <c r="L164" s="2"/>
       <c r="M164" s="2"/>
@@ -7006,7 +6691,7 @@
       <c r="G165" s="2"/>
       <c r="H165" s="2"/>
       <c r="I165" s="2"/>
-      <c r="J165" s="6"/>
+      <c r="J165" s="3"/>
       <c r="K165" s="2"/>
       <c r="L165" s="2"/>
       <c r="M165" s="2"/>
@@ -7034,7 +6719,7 @@
       <c r="G166" s="2"/>
       <c r="H166" s="2"/>
       <c r="I166" s="2"/>
-      <c r="J166" s="6"/>
+      <c r="J166" s="3"/>
       <c r="K166" s="2"/>
       <c r="L166" s="2"/>
       <c r="M166" s="2"/>
@@ -7062,7 +6747,7 @@
       <c r="G167" s="2"/>
       <c r="H167" s="2"/>
       <c r="I167" s="2"/>
-      <c r="J167" s="6"/>
+      <c r="J167" s="3"/>
       <c r="K167" s="2"/>
       <c r="L167" s="2"/>
       <c r="M167" s="2"/>
@@ -7090,7 +6775,7 @@
       <c r="G168" s="2"/>
       <c r="H168" s="2"/>
       <c r="I168" s="2"/>
-      <c r="J168" s="6"/>
+      <c r="J168" s="3"/>
       <c r="K168" s="2"/>
       <c r="L168" s="2"/>
       <c r="M168" s="2"/>
@@ -7118,7 +6803,7 @@
       <c r="G169" s="2"/>
       <c r="H169" s="2"/>
       <c r="I169" s="2"/>
-      <c r="J169" s="6"/>
+      <c r="J169" s="3"/>
       <c r="K169" s="2"/>
       <c r="L169" s="2"/>
       <c r="M169" s="2"/>
@@ -7146,7 +6831,7 @@
       <c r="G170" s="2"/>
       <c r="H170" s="2"/>
       <c r="I170" s="2"/>
-      <c r="J170" s="6"/>
+      <c r="J170" s="3"/>
       <c r="K170" s="2"/>
       <c r="L170" s="2"/>
       <c r="M170" s="2"/>
@@ -7174,7 +6859,7 @@
       <c r="G171" s="2"/>
       <c r="H171" s="2"/>
       <c r="I171" s="2"/>
-      <c r="J171" s="6"/>
+      <c r="J171" s="3"/>
       <c r="K171" s="2"/>
       <c r="L171" s="2"/>
       <c r="M171" s="2"/>
@@ -7202,7 +6887,7 @@
       <c r="G172" s="2"/>
       <c r="H172" s="2"/>
       <c r="I172" s="2"/>
-      <c r="J172" s="6"/>
+      <c r="J172" s="3"/>
       <c r="K172" s="2"/>
       <c r="L172" s="2"/>
       <c r="M172" s="2"/>
@@ -7230,7 +6915,7 @@
       <c r="G173" s="2"/>
       <c r="H173" s="2"/>
       <c r="I173" s="2"/>
-      <c r="J173" s="6"/>
+      <c r="J173" s="3"/>
       <c r="K173" s="2"/>
       <c r="L173" s="2"/>
       <c r="M173" s="2"/>
@@ -7258,7 +6943,7 @@
       <c r="G174" s="2"/>
       <c r="H174" s="2"/>
       <c r="I174" s="2"/>
-      <c r="J174" s="6"/>
+      <c r="J174" s="3"/>
       <c r="K174" s="2"/>
       <c r="L174" s="2"/>
       <c r="M174" s="2"/>
@@ -7286,7 +6971,7 @@
       <c r="G175" s="2"/>
       <c r="H175" s="2"/>
       <c r="I175" s="2"/>
-      <c r="J175" s="6"/>
+      <c r="J175" s="3"/>
       <c r="K175" s="2"/>
       <c r="L175" s="2"/>
       <c r="M175" s="2"/>
@@ -7314,7 +6999,7 @@
       <c r="G176" s="2"/>
       <c r="H176" s="2"/>
       <c r="I176" s="2"/>
-      <c r="J176" s="6"/>
+      <c r="J176" s="3"/>
       <c r="K176" s="2"/>
       <c r="L176" s="2"/>
       <c r="M176" s="2"/>
@@ -7342,7 +7027,7 @@
       <c r="G177" s="2"/>
       <c r="H177" s="2"/>
       <c r="I177" s="2"/>
-      <c r="J177" s="6"/>
+      <c r="J177" s="3"/>
       <c r="K177" s="2"/>
       <c r="L177" s="2"/>
       <c r="M177" s="2"/>
@@ -7370,7 +7055,7 @@
       <c r="G178" s="2"/>
       <c r="H178" s="2"/>
       <c r="I178" s="2"/>
-      <c r="J178" s="6"/>
+      <c r="J178" s="3"/>
       <c r="K178" s="2"/>
       <c r="L178" s="2"/>
       <c r="M178" s="2"/>
@@ -7398,7 +7083,7 @@
       <c r="G179" s="2"/>
       <c r="H179" s="2"/>
       <c r="I179" s="2"/>
-      <c r="J179" s="6"/>
+      <c r="J179" s="3"/>
       <c r="K179" s="2"/>
       <c r="L179" s="2"/>
       <c r="M179" s="2"/>
@@ -7426,7 +7111,7 @@
       <c r="G180" s="2"/>
       <c r="H180" s="2"/>
       <c r="I180" s="2"/>
-      <c r="J180" s="6"/>
+      <c r="J180" s="3"/>
       <c r="K180" s="2"/>
       <c r="L180" s="2"/>
       <c r="M180" s="2"/>
@@ -7454,7 +7139,7 @@
       <c r="G181" s="2"/>
       <c r="H181" s="2"/>
       <c r="I181" s="2"/>
-      <c r="J181" s="6"/>
+      <c r="J181" s="3"/>
       <c r="K181" s="2"/>
       <c r="L181" s="2"/>
       <c r="M181" s="2"/>
@@ -7482,7 +7167,7 @@
       <c r="G182" s="2"/>
       <c r="H182" s="2"/>
       <c r="I182" s="2"/>
-      <c r="J182" s="6"/>
+      <c r="J182" s="3"/>
       <c r="K182" s="2"/>
       <c r="L182" s="2"/>
       <c r="M182" s="2"/>
@@ -7510,7 +7195,7 @@
       <c r="G183" s="2"/>
       <c r="H183" s="2"/>
       <c r="I183" s="2"/>
-      <c r="J183" s="6"/>
+      <c r="J183" s="3"/>
       <c r="K183" s="2"/>
       <c r="L183" s="2"/>
       <c r="M183" s="2"/>
@@ -7538,7 +7223,7 @@
       <c r="G184" s="2"/>
       <c r="H184" s="2"/>
       <c r="I184" s="2"/>
-      <c r="J184" s="6"/>
+      <c r="J184" s="3"/>
       <c r="K184" s="2"/>
       <c r="L184" s="2"/>
       <c r="M184" s="2"/>
@@ -7566,7 +7251,7 @@
       <c r="G185" s="2"/>
       <c r="H185" s="2"/>
       <c r="I185" s="2"/>
-      <c r="J185" s="6"/>
+      <c r="J185" s="3"/>
       <c r="K185" s="2"/>
       <c r="L185" s="2"/>
       <c r="M185" s="2"/>
@@ -7594,7 +7279,7 @@
       <c r="G186" s="2"/>
       <c r="H186" s="2"/>
       <c r="I186" s="2"/>
-      <c r="J186" s="6"/>
+      <c r="J186" s="3"/>
       <c r="K186" s="2"/>
       <c r="L186" s="2"/>
       <c r="M186" s="2"/>
@@ -7622,7 +7307,7 @@
       <c r="G187" s="2"/>
       <c r="H187" s="2"/>
       <c r="I187" s="2"/>
-      <c r="J187" s="6"/>
+      <c r="J187" s="3"/>
       <c r="K187" s="2"/>
       <c r="L187" s="2"/>
       <c r="M187" s="2"/>
@@ -7650,7 +7335,7 @@
       <c r="G188" s="2"/>
       <c r="H188" s="2"/>
       <c r="I188" s="2"/>
-      <c r="J188" s="6"/>
+      <c r="J188" s="3"/>
       <c r="K188" s="2"/>
       <c r="L188" s="2"/>
       <c r="M188" s="2"/>
@@ -7678,7 +7363,7 @@
       <c r="G189" s="2"/>
       <c r="H189" s="2"/>
       <c r="I189" s="2"/>
-      <c r="J189" s="6"/>
+      <c r="J189" s="3"/>
       <c r="K189" s="2"/>
       <c r="L189" s="2"/>
       <c r="M189" s="2"/>
@@ -7706,7 +7391,7 @@
       <c r="G190" s="2"/>
       <c r="H190" s="2"/>
       <c r="I190" s="2"/>
-      <c r="J190" s="6"/>
+      <c r="J190" s="3"/>
       <c r="K190" s="2"/>
       <c r="L190" s="2"/>
       <c r="M190" s="2"/>
@@ -7734,7 +7419,7 @@
       <c r="G191" s="2"/>
       <c r="H191" s="2"/>
       <c r="I191" s="2"/>
-      <c r="J191" s="6"/>
+      <c r="J191" s="3"/>
       <c r="K191" s="2"/>
       <c r="L191" s="2"/>
       <c r="M191" s="2"/>
@@ -7762,7 +7447,7 @@
       <c r="G192" s="2"/>
       <c r="H192" s="2"/>
       <c r="I192" s="2"/>
-      <c r="J192" s="6"/>
+      <c r="J192" s="3"/>
       <c r="K192" s="2"/>
       <c r="L192" s="2"/>
       <c r="M192" s="2"/>
@@ -7790,7 +7475,7 @@
       <c r="G193" s="2"/>
       <c r="H193" s="2"/>
       <c r="I193" s="2"/>
-      <c r="J193" s="6"/>
+      <c r="J193" s="3"/>
       <c r="K193" s="2"/>
       <c r="L193" s="2"/>
       <c r="M193" s="2"/>
@@ -7818,7 +7503,7 @@
       <c r="G194" s="2"/>
       <c r="H194" s="2"/>
       <c r="I194" s="2"/>
-      <c r="J194" s="6"/>
+      <c r="J194" s="3"/>
       <c r="K194" s="2"/>
       <c r="L194" s="2"/>
       <c r="M194" s="2"/>
@@ -7846,7 +7531,7 @@
       <c r="G195" s="2"/>
       <c r="H195" s="2"/>
       <c r="I195" s="2"/>
-      <c r="J195" s="6"/>
+      <c r="J195" s="3"/>
       <c r="K195" s="2"/>
       <c r="L195" s="2"/>
       <c r="M195" s="2"/>
@@ -7874,7 +7559,7 @@
       <c r="G196" s="2"/>
       <c r="H196" s="2"/>
       <c r="I196" s="2"/>
-      <c r="J196" s="6"/>
+      <c r="J196" s="3"/>
       <c r="K196" s="2"/>
       <c r="L196" s="2"/>
       <c r="M196" s="2"/>
@@ -7902,7 +7587,7 @@
       <c r="G197" s="2"/>
       <c r="H197" s="2"/>
       <c r="I197" s="2"/>
-      <c r="J197" s="6"/>
+      <c r="J197" s="3"/>
       <c r="K197" s="2"/>
       <c r="L197" s="2"/>
       <c r="M197" s="2"/>
@@ -7930,7 +7615,7 @@
       <c r="G198" s="2"/>
       <c r="H198" s="2"/>
       <c r="I198" s="2"/>
-      <c r="J198" s="6"/>
+      <c r="J198" s="3"/>
       <c r="K198" s="2"/>
       <c r="L198" s="2"/>
       <c r="M198" s="2"/>
@@ -7958,7 +7643,7 @@
       <c r="G199" s="2"/>
       <c r="H199" s="2"/>
       <c r="I199" s="2"/>
-      <c r="J199" s="6"/>
+      <c r="J199" s="3"/>
       <c r="K199" s="2"/>
       <c r="L199" s="2"/>
       <c r="M199" s="2"/>
@@ -7986,7 +7671,7 @@
       <c r="G200" s="2"/>
       <c r="H200" s="2"/>
       <c r="I200" s="2"/>
-      <c r="J200" s="6"/>
+      <c r="J200" s="3"/>
       <c r="K200" s="2"/>
       <c r="L200" s="2"/>
       <c r="M200" s="2"/>
@@ -8014,7 +7699,7 @@
       <c r="G201" s="2"/>
       <c r="H201" s="2"/>
       <c r="I201" s="2"/>
-      <c r="J201" s="6"/>
+      <c r="J201" s="3"/>
       <c r="K201" s="2"/>
       <c r="L201" s="2"/>
       <c r="M201" s="2"/>
@@ -8042,7 +7727,7 @@
       <c r="G202" s="2"/>
       <c r="H202" s="2"/>
       <c r="I202" s="2"/>
-      <c r="J202" s="6"/>
+      <c r="J202" s="3"/>
       <c r="K202" s="2"/>
       <c r="L202" s="2"/>
       <c r="M202" s="2"/>
@@ -8070,7 +7755,7 @@
       <c r="G203" s="2"/>
       <c r="H203" s="2"/>
       <c r="I203" s="2"/>
-      <c r="J203" s="6"/>
+      <c r="J203" s="3"/>
       <c r="K203" s="2"/>
       <c r="L203" s="2"/>
       <c r="M203" s="2"/>
@@ -8098,7 +7783,7 @@
       <c r="G204" s="2"/>
       <c r="H204" s="2"/>
       <c r="I204" s="2"/>
-      <c r="J204" s="6"/>
+      <c r="J204" s="3"/>
       <c r="K204" s="2"/>
       <c r="L204" s="2"/>
       <c r="M204" s="2"/>
@@ -8126,7 +7811,7 @@
       <c r="G205" s="2"/>
       <c r="H205" s="2"/>
       <c r="I205" s="2"/>
-      <c r="J205" s="6"/>
+      <c r="J205" s="3"/>
       <c r="K205" s="2"/>
       <c r="L205" s="2"/>
       <c r="M205" s="2"/>
@@ -8154,7 +7839,7 @@
       <c r="G206" s="2"/>
       <c r="H206" s="2"/>
       <c r="I206" s="2"/>
-      <c r="J206" s="6"/>
+      <c r="J206" s="3"/>
       <c r="K206" s="2"/>
       <c r="L206" s="2"/>
       <c r="M206" s="2"/>
@@ -8182,7 +7867,7 @@
       <c r="G207" s="2"/>
       <c r="H207" s="2"/>
       <c r="I207" s="2"/>
-      <c r="J207" s="6"/>
+      <c r="J207" s="3"/>
       <c r="K207" s="2"/>
       <c r="L207" s="2"/>
       <c r="M207" s="2"/>
@@ -8210,7 +7895,7 @@
       <c r="G208" s="2"/>
       <c r="H208" s="2"/>
       <c r="I208" s="2"/>
-      <c r="J208" s="6"/>
+      <c r="J208" s="3"/>
       <c r="K208" s="2"/>
       <c r="L208" s="2"/>
       <c r="M208" s="2"/>
@@ -8238,7 +7923,7 @@
       <c r="G209" s="2"/>
       <c r="H209" s="2"/>
       <c r="I209" s="2"/>
-      <c r="J209" s="6"/>
+      <c r="J209" s="3"/>
       <c r="K209" s="2"/>
       <c r="L209" s="2"/>
       <c r="M209" s="2"/>
@@ -8266,7 +7951,7 @@
       <c r="G210" s="2"/>
       <c r="H210" s="2"/>
       <c r="I210" s="2"/>
-      <c r="J210" s="6"/>
+      <c r="J210" s="3"/>
       <c r="K210" s="2"/>
       <c r="L210" s="2"/>
       <c r="M210" s="2"/>
@@ -8294,7 +7979,7 @@
       <c r="G211" s="2"/>
       <c r="H211" s="2"/>
       <c r="I211" s="2"/>
-      <c r="J211" s="6"/>
+      <c r="J211" s="3"/>
       <c r="K211" s="2"/>
       <c r="L211" s="2"/>
       <c r="M211" s="2"/>
@@ -8322,7 +8007,7 @@
       <c r="G212" s="2"/>
       <c r="H212" s="2"/>
       <c r="I212" s="2"/>
-      <c r="J212" s="6"/>
+      <c r="J212" s="3"/>
       <c r="K212" s="2"/>
       <c r="L212" s="2"/>
       <c r="M212" s="2"/>
@@ -8350,7 +8035,7 @@
       <c r="G213" s="2"/>
       <c r="H213" s="2"/>
       <c r="I213" s="2"/>
-      <c r="J213" s="6"/>
+      <c r="J213" s="3"/>
       <c r="K213" s="2"/>
       <c r="L213" s="2"/>
       <c r="M213" s="2"/>
@@ -8378,7 +8063,7 @@
       <c r="G214" s="2"/>
       <c r="H214" s="2"/>
       <c r="I214" s="2"/>
-      <c r="J214" s="6"/>
+      <c r="J214" s="3"/>
       <c r="K214" s="2"/>
       <c r="L214" s="2"/>
       <c r="M214" s="2"/>
@@ -8406,7 +8091,7 @@
       <c r="G215" s="2"/>
       <c r="H215" s="2"/>
       <c r="I215" s="2"/>
-      <c r="J215" s="6"/>
+      <c r="J215" s="3"/>
       <c r="K215" s="2"/>
       <c r="L215" s="2"/>
       <c r="M215" s="2"/>
@@ -8434,7 +8119,7 @@
       <c r="G216" s="2"/>
       <c r="H216" s="2"/>
       <c r="I216" s="2"/>
-      <c r="J216" s="6"/>
+      <c r="J216" s="3"/>
       <c r="K216" s="2"/>
       <c r="L216" s="2"/>
       <c r="M216" s="2"/>
@@ -8462,7 +8147,7 @@
       <c r="G217" s="2"/>
       <c r="H217" s="2"/>
       <c r="I217" s="2"/>
-      <c r="J217" s="6"/>
+      <c r="J217" s="3"/>
       <c r="K217" s="2"/>
       <c r="L217" s="2"/>
       <c r="M217" s="2"/>
@@ -8490,7 +8175,7 @@
       <c r="G218" s="2"/>
       <c r="H218" s="2"/>
       <c r="I218" s="2"/>
-      <c r="J218" s="6"/>
+      <c r="J218" s="3"/>
       <c r="K218" s="2"/>
       <c r="L218" s="2"/>
       <c r="M218" s="2"/>
@@ -8518,7 +8203,7 @@
       <c r="G219" s="2"/>
       <c r="H219" s="2"/>
       <c r="I219" s="2"/>
-      <c r="J219" s="6"/>
+      <c r="J219" s="3"/>
       <c r="K219" s="2"/>
       <c r="L219" s="2"/>
       <c r="M219" s="2"/>
@@ -8546,7 +8231,7 @@
       <c r="G220" s="2"/>
       <c r="H220" s="2"/>
       <c r="I220" s="2"/>
-      <c r="J220" s="6"/>
+      <c r="J220" s="3"/>
       <c r="K220" s="2"/>
       <c r="L220" s="2"/>
       <c r="M220" s="2"/>
@@ -8574,7 +8259,7 @@
       <c r="G221" s="2"/>
       <c r="H221" s="2"/>
       <c r="I221" s="2"/>
-      <c r="J221" s="6"/>
+      <c r="J221" s="3"/>
       <c r="K221" s="2"/>
       <c r="L221" s="2"/>
       <c r="M221" s="2"/>
@@ -8602,7 +8287,7 @@
       <c r="G222" s="2"/>
       <c r="H222" s="2"/>
       <c r="I222" s="2"/>
-      <c r="J222" s="6"/>
+      <c r="J222" s="3"/>
       <c r="K222" s="2"/>
       <c r="L222" s="2"/>
       <c r="M222" s="2"/>
@@ -8630,7 +8315,7 @@
       <c r="G223" s="2"/>
       <c r="H223" s="2"/>
       <c r="I223" s="2"/>
-      <c r="J223" s="6"/>
+      <c r="J223" s="3"/>
       <c r="K223" s="2"/>
       <c r="L223" s="2"/>
       <c r="M223" s="2"/>
@@ -8658,7 +8343,7 @@
       <c r="G224" s="2"/>
       <c r="H224" s="2"/>
       <c r="I224" s="2"/>
-      <c r="J224" s="6"/>
+      <c r="J224" s="3"/>
       <c r="K224" s="2"/>
       <c r="L224" s="2"/>
       <c r="M224" s="2"/>
@@ -8686,7 +8371,7 @@
       <c r="G225" s="2"/>
       <c r="H225" s="2"/>
       <c r="I225" s="2"/>
-      <c r="J225" s="6"/>
+      <c r="J225" s="3"/>
       <c r="K225" s="2"/>
       <c r="L225" s="2"/>
       <c r="M225" s="2"/>
@@ -8714,7 +8399,7 @@
       <c r="G226" s="2"/>
       <c r="H226" s="2"/>
       <c r="I226" s="2"/>
-      <c r="J226" s="6"/>
+      <c r="J226" s="3"/>
       <c r="K226" s="2"/>
       <c r="L226" s="2"/>
       <c r="M226" s="2"/>
@@ -8742,7 +8427,7 @@
       <c r="G227" s="2"/>
       <c r="H227" s="2"/>
       <c r="I227" s="2"/>
-      <c r="J227" s="6"/>
+      <c r="J227" s="3"/>
       <c r="K227" s="2"/>
       <c r="L227" s="2"/>
       <c r="M227" s="2"/>
@@ -8770,7 +8455,7 @@
       <c r="G228" s="2"/>
       <c r="H228" s="2"/>
       <c r="I228" s="2"/>
-      <c r="J228" s="6"/>
+      <c r="J228" s="3"/>
       <c r="K228" s="2"/>
       <c r="L228" s="2"/>
       <c r="M228" s="2"/>
@@ -9562,25 +9247,15 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="A20:I20"/>
-    <mergeCell ref="A21:C22"/>
-    <mergeCell ref="D21:I22"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="D27:I27"/>
-    <mergeCell ref="F28:I28"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F23:I23"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A25:C26"/>
-    <mergeCell ref="D25:F26"/>
-    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="A1:I10"/>
+    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="A14:C14"/>
     <mergeCell ref="D18:F18"/>
     <mergeCell ref="H18:I18"/>
     <mergeCell ref="A15:C15"/>
@@ -9590,15 +9265,25 @@
     <mergeCell ref="A17:C17"/>
     <mergeCell ref="D17:F17"/>
     <mergeCell ref="A18:C18"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="A1:I10"/>
-    <mergeCell ref="A11:I11"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F23:I23"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A25:C26"/>
+    <mergeCell ref="D25:F26"/>
+    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="D27:I27"/>
+    <mergeCell ref="F28:I28"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A21:C22"/>
+    <mergeCell ref="D21:I22"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.78740157480314965" right="0.78740157480314965" top="0.59055118110236227" bottom="0.39370078740157483" header="0" footer="0"/>

</xml_diff>

<commit_message>
Cambio de botones a descarga directa de Word en Informe de Supervisión y mejoras en conversión XML a Word
</commit_message>
<xml_diff>
--- a/plantillas/CUENTA_COBRO.xlsx
+++ b/plantillas/CUENTA_COBRO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Soporte y Desarrollo\Documents\NetBeansProjects\combinacion\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81717961-126E-49D4-9AB9-C464D1D8D3E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B272AAD7-6780-4F12-9CD7-6F41FBF836E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -451,32 +451,71 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -498,56 +537,17 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -896,7 +896,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="8362950" cy="1724025"/>
+    <xdr:ext cx="8172450" cy="1724025"/>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
         <xdr:cNvPr id="7" name="Shape 2">
@@ -911,7 +911,7 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="8362950" cy="1724025"/>
+          <a:ext cx="8172450" cy="1724025"/>
           <a:chOff x="1469325" y="2884650"/>
           <a:chExt cx="7753350" cy="1790700"/>
         </a:xfrm>
@@ -2014,15 +2014,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="57"/>
-      <c r="B1" s="58"/>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
+      <c r="A1" s="22"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
@@ -2042,15 +2042,15 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58"/>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
+      <c r="A2" s="23"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
@@ -2070,15 +2070,15 @@
       <c r="Z2" s="1"/>
     </row>
     <row r="3" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="58"/>
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
+      <c r="A3" s="23"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
@@ -2098,15 +2098,15 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="58"/>
-      <c r="B4" s="58"/>
-      <c r="C4" s="58"/>
-      <c r="D4" s="58"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="58"/>
-      <c r="I4" s="58"/>
+      <c r="A4" s="23"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
@@ -2126,15 +2126,15 @@
       <c r="Z4" s="1"/>
     </row>
     <row r="5" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="58"/>
-      <c r="B5" s="58"/>
-      <c r="C5" s="58"/>
-      <c r="D5" s="58"/>
-      <c r="E5" s="58"/>
-      <c r="F5" s="58"/>
-      <c r="G5" s="58"/>
-      <c r="H5" s="58"/>
-      <c r="I5" s="58"/>
+      <c r="A5" s="23"/>
+      <c r="B5" s="23"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="23"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
@@ -2154,15 +2154,15 @@
       <c r="Z5" s="1"/>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="58"/>
-      <c r="B6" s="58"/>
-      <c r="C6" s="58"/>
-      <c r="D6" s="58"/>
-      <c r="E6" s="58"/>
-      <c r="F6" s="58"/>
-      <c r="G6" s="58"/>
-      <c r="H6" s="58"/>
-      <c r="I6" s="58"/>
+      <c r="A6" s="23"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
@@ -2182,15 +2182,15 @@
       <c r="Z6" s="1"/>
     </row>
     <row r="7" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="58"/>
-      <c r="B7" s="58"/>
-      <c r="C7" s="58"/>
-      <c r="D7" s="58"/>
-      <c r="E7" s="58"/>
-      <c r="F7" s="58"/>
-      <c r="G7" s="58"/>
-      <c r="H7" s="58"/>
-      <c r="I7" s="58"/>
+      <c r="A7" s="23"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
@@ -2210,15 +2210,15 @@
       <c r="Z7" s="1"/>
     </row>
     <row r="8" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="58"/>
-      <c r="B8" s="58"/>
-      <c r="C8" s="58"/>
-      <c r="D8" s="58"/>
-      <c r="E8" s="58"/>
-      <c r="F8" s="58"/>
-      <c r="G8" s="58"/>
-      <c r="H8" s="58"/>
-      <c r="I8" s="58"/>
+      <c r="A8" s="23"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
@@ -2238,15 +2238,15 @@
       <c r="Z8" s="1"/>
     </row>
     <row r="9" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="58"/>
-      <c r="B9" s="58"/>
-      <c r="C9" s="58"/>
-      <c r="D9" s="58"/>
-      <c r="E9" s="58"/>
-      <c r="F9" s="58"/>
-      <c r="G9" s="58"/>
-      <c r="H9" s="58"/>
-      <c r="I9" s="58"/>
+      <c r="A9" s="23"/>
+      <c r="B9" s="23"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
@@ -2266,15 +2266,15 @@
       <c r="Z9" s="1"/>
     </row>
     <row r="10" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="58"/>
-      <c r="B10" s="58"/>
-      <c r="C10" s="58"/>
-      <c r="D10" s="58"/>
-      <c r="E10" s="58"/>
-      <c r="F10" s="58"/>
-      <c r="G10" s="58"/>
-      <c r="H10" s="58"/>
-      <c r="I10" s="58"/>
+      <c r="A10" s="23"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
@@ -2294,17 +2294,17 @@
       <c r="Z10" s="1"/>
     </row>
     <row r="11" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="52" t="s">
+      <c r="A11" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="20"/>
+      <c r="B11" s="25"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="25"/>
+      <c r="I11" s="21"/>
       <c r="J11" s="5">
         <v>1</v>
       </c>
@@ -2326,13 +2326,13 @@
       <c r="Z11" s="2"/>
     </row>
     <row r="12" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="19"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="59"/>
-      <c r="E12" s="20"/>
+      <c r="B12" s="25"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="21"/>
       <c r="F12" s="11" t="s">
         <v>2</v>
       </c>
@@ -2362,16 +2362,16 @@
       <c r="Z12" s="2"/>
     </row>
     <row r="13" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="53" t="s">
+      <c r="B13" s="25"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="E13" s="54"/>
-      <c r="F13" s="54"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
       <c r="G13" s="12" t="s">
         <v>6</v>
       </c>
@@ -2400,23 +2400,23 @@
       <c r="Z13" s="2"/>
     </row>
     <row r="14" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="19"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="55" t="s">
+      <c r="B14" s="25"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="56"/>
-      <c r="F14" s="56"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="H14" s="51">
+      <c r="H14" s="20">
         <v>4121</v>
       </c>
-      <c r="I14" s="20"/>
+      <c r="I14" s="21"/>
       <c r="J14" s="3"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
@@ -2436,23 +2436,23 @@
       <c r="Z14" s="2"/>
     </row>
     <row r="15" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="19"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="50" t="s">
+      <c r="B15" s="25"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
       <c r="G15" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="51">
+      <c r="H15" s="20">
         <v>8896744</v>
       </c>
-      <c r="I15" s="20"/>
+      <c r="I15" s="21"/>
       <c r="J15" s="3"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
@@ -2472,17 +2472,17 @@
       <c r="Z15" s="2"/>
     </row>
     <row r="16" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="52" t="s">
+      <c r="A16" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="19"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="20"/>
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="25"/>
+      <c r="I16" s="21"/>
       <c r="J16" s="5">
         <v>2</v>
       </c>
@@ -2504,14 +2504,14 @@
       <c r="Z16" s="2"/>
     </row>
     <row r="17" spans="1:26" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="53"/>
-      <c r="E17" s="54"/>
-      <c r="F17" s="54"/>
+      <c r="B17" s="25"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="29"/>
       <c r="G17" s="14" t="s">
         <v>15</v>
       </c>
@@ -2536,19 +2536,19 @@
       <c r="Z17" s="2"/>
     </row>
     <row r="18" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="19"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="47"/>
-      <c r="E18" s="48"/>
-      <c r="F18" s="48"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
       <c r="G18" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="H18" s="49"/>
-      <c r="I18" s="20"/>
+      <c r="H18" s="32"/>
+      <c r="I18" s="21"/>
       <c r="J18" s="3"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
@@ -2568,19 +2568,19 @@
       <c r="Z18" s="2"/>
     </row>
     <row r="19" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="18" t="s">
+      <c r="A19" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="19"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="21"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
+      <c r="B19" s="25"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="56"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
       <c r="G19" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="H19" s="23"/>
-      <c r="I19" s="20"/>
+      <c r="H19" s="57"/>
+      <c r="I19" s="21"/>
       <c r="J19" s="3"/>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
@@ -2600,17 +2600,17 @@
       <c r="Z19" s="2"/>
     </row>
     <row r="20" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="24" t="s">
+      <c r="A20" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="20"/>
+      <c r="B20" s="25"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="25"/>
+      <c r="G20" s="25"/>
+      <c r="H20" s="25"/>
+      <c r="I20" s="21"/>
       <c r="J20" s="5">
         <v>3</v>
       </c>
@@ -2632,17 +2632,17 @@
       <c r="Z20" s="2"/>
     </row>
     <row r="21" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="25" t="s">
+      <c r="A21" s="58" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="26"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="31"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="26"/>
-      <c r="G21" s="26"/>
-      <c r="H21" s="26"/>
-      <c r="I21" s="27"/>
+      <c r="B21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="59"/>
+      <c r="E21" s="42"/>
+      <c r="F21" s="42"/>
+      <c r="G21" s="42"/>
+      <c r="H21" s="42"/>
+      <c r="I21" s="43"/>
       <c r="J21" s="5"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
@@ -2662,15 +2662,15 @@
       <c r="Z21" s="2"/>
     </row>
     <row r="22" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="28"/>
-      <c r="B22" s="29"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="28"/>
-      <c r="E22" s="29"/>
-      <c r="F22" s="29"/>
-      <c r="G22" s="29"/>
-      <c r="H22" s="29"/>
-      <c r="I22" s="30"/>
+      <c r="A22" s="44"/>
+      <c r="B22" s="38"/>
+      <c r="C22" s="39"/>
+      <c r="D22" s="44"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="38"/>
+      <c r="G22" s="38"/>
+      <c r="H22" s="38"/>
+      <c r="I22" s="39"/>
       <c r="J22" s="5"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
@@ -2690,17 +2690,17 @@
       <c r="Z22" s="2"/>
     </row>
     <row r="23" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="42" t="s">
+      <c r="A23" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="19"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="40"/>
-      <c r="F23" s="41"/>
-      <c r="G23" s="29"/>
-      <c r="H23" s="29"/>
-      <c r="I23" s="30"/>
+      <c r="B23" s="25"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="35"/>
+      <c r="E23" s="36"/>
+      <c r="F23" s="37"/>
+      <c r="G23" s="38"/>
+      <c r="H23" s="38"/>
+      <c r="I23" s="39"/>
       <c r="J23" s="5"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
@@ -2720,17 +2720,17 @@
       <c r="Z23" s="2"/>
     </row>
     <row r="24" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="24" t="s">
+      <c r="A24" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="46"/>
-      <c r="C24" s="46"/>
-      <c r="D24" s="46"/>
-      <c r="E24" s="46"/>
-      <c r="F24" s="46"/>
-      <c r="G24" s="46"/>
-      <c r="H24" s="46"/>
-      <c r="I24" s="20"/>
+      <c r="B24" s="48"/>
+      <c r="C24" s="48"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="48"/>
+      <c r="F24" s="48"/>
+      <c r="G24" s="48"/>
+      <c r="H24" s="48"/>
+      <c r="I24" s="21"/>
       <c r="J24" s="5">
         <v>4</v>
       </c>
@@ -2752,19 +2752,19 @@
       <c r="Z24" s="2"/>
     </row>
     <row r="25" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="43" t="s">
+      <c r="A25" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="26"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="44"/>
-      <c r="E25" s="40"/>
-      <c r="F25" s="45"/>
+      <c r="B25" s="42"/>
+      <c r="C25" s="43"/>
+      <c r="D25" s="45"/>
+      <c r="E25" s="36"/>
+      <c r="F25" s="46"/>
       <c r="G25" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="H25" s="34"/>
-      <c r="I25" s="20"/>
+      <c r="H25" s="51"/>
+      <c r="I25" s="21"/>
       <c r="J25" s="5"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
@@ -2784,17 +2784,17 @@
       <c r="Z25" s="2"/>
     </row>
     <row r="26" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="28"/>
-      <c r="B26" s="29"/>
-      <c r="C26" s="30"/>
-      <c r="D26" s="40"/>
-      <c r="E26" s="40"/>
-      <c r="F26" s="45"/>
+      <c r="A26" s="44"/>
+      <c r="B26" s="38"/>
+      <c r="C26" s="39"/>
+      <c r="D26" s="36"/>
+      <c r="E26" s="36"/>
+      <c r="F26" s="46"/>
       <c r="G26" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="H26" s="34"/>
-      <c r="I26" s="20"/>
+      <c r="H26" s="51"/>
+      <c r="I26" s="21"/>
       <c r="J26" s="5"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
@@ -2814,17 +2814,17 @@
       <c r="Z26" s="2"/>
     </row>
     <row r="27" spans="1:26" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="32" t="s">
+      <c r="A27" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="B27" s="19"/>
-      <c r="C27" s="20"/>
-      <c r="D27" s="35"/>
-      <c r="E27" s="36"/>
-      <c r="F27" s="36"/>
-      <c r="G27" s="36"/>
-      <c r="H27" s="36"/>
-      <c r="I27" s="37"/>
+      <c r="B27" s="25"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="52"/>
+      <c r="E27" s="53"/>
+      <c r="F27" s="53"/>
+      <c r="G27" s="53"/>
+      <c r="H27" s="53"/>
+      <c r="I27" s="54"/>
       <c r="J27" s="5"/>
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
@@ -2844,17 +2844,17 @@
       <c r="Z27" s="2"/>
     </row>
     <row r="28" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="32" t="s">
+      <c r="A28" s="49" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="19"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="33"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="38"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="19"/>
-      <c r="I28" s="20"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="50"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="55"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="25"/>
+      <c r="I28" s="21"/>
       <c r="J28" s="5"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
@@ -9247,6 +9247,34 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="37">
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A21:C22"/>
+    <mergeCell ref="D21:I22"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="D27:I27"/>
+    <mergeCell ref="F28:I28"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F23:I23"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A25:C26"/>
+    <mergeCell ref="D25:F26"/>
+    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="A16:I16"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="A18:C18"/>
     <mergeCell ref="D14:F14"/>
     <mergeCell ref="H14:I14"/>
     <mergeCell ref="A1:I10"/>
@@ -9256,34 +9284,6 @@
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="D13:F13"/>
     <mergeCell ref="A14:C14"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="A16:I16"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F23:I23"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A25:C26"/>
-    <mergeCell ref="D25:F26"/>
-    <mergeCell ref="A24:I24"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="D27:I27"/>
-    <mergeCell ref="F28:I28"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="A20:I20"/>
-    <mergeCell ref="A21:C22"/>
-    <mergeCell ref="D21:I22"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.78740157480314965" right="0.78740157480314965" top="0.59055118110236227" bottom="0.39370078740157483" header="0" footer="0"/>

</xml_diff>

<commit_message>
Actualizar plantillas y utilidades para generación de cuenta de cobro y PDF
</commit_message>
<xml_diff>
--- a/plantillas/CUENTA_COBRO.xlsx
+++ b/plantillas/CUENTA_COBRO.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Soporte y Desarrollo\Documents\NetBeansProjects\combinacion\plantillas\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B272AAD7-6780-4F12-9CD7-6F41FBF836E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11160"/>
   </bookViews>
   <sheets>
     <sheet name="Documento Equivalente" sheetId="1" r:id="rId1"/>
@@ -121,13 +115,13 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="5">
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;\ * #,##0.00_);_(&quot;$&quot;\ * \(#,##0.00\);_(&quot;$&quot;\ * &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="dd\-mm\-yyyy"/>
-    <numFmt numFmtId="165" formatCode="##,###"/>
-    <numFmt numFmtId="166" formatCode="&quot;$&quot;\ #,##0"/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;\ * #,##0.00_);_(&quot;$&quot;\ * \(#,##0.00\);_(&quot;$&quot;\ * &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="dd\-mm\-yyyy"/>
+    <numFmt numFmtId="167" formatCode="##,###"/>
+    <numFmt numFmtId="168" formatCode="&quot;$&quot;\ #,##0"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -409,7 +403,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -436,10 +430,10 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -448,7 +442,7 @@
     <xf numFmtId="1" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -472,7 +466,7 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -490,11 +484,11 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
@@ -519,7 +513,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -581,7 +575,7 @@
         <xdr:cNvPr id="3" name="Shape 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -636,7 +630,7 @@
         <xdr:cNvPr id="4" name="Shape 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -691,7 +685,7 @@
         <xdr:cNvPr id="2" name="Shape 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -746,7 +740,7 @@
         <xdr:cNvPr id="5" name="Shape 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -801,7 +795,7 @@
         <xdr:cNvPr id="6" name="Shape 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -902,7 +896,7 @@
         <xdr:cNvPr id="7" name="Shape 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000007000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000007000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -921,7 +915,7 @@
           <xdr:cNvPr id="8" name="Shape 6">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000008000000}"/>
+                <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000008000000}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
@@ -940,7 +934,7 @@
             <xdr:cNvPr id="9" name="Shape 7">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
+                  <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -983,7 +977,7 @@
             <xdr:cNvPr id="10" name="Shape 8">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000A000000}"/>
+                  <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000A000000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1002,7 +996,7 @@
               <xdr:cNvPr id="11" name="Shape 9">
                 <a:extLst>
                   <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000B000000}"/>
+                    <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000B000000}"/>
                   </a:ext>
                 </a:extLst>
               </xdr:cNvPr>
@@ -1047,7 +1041,7 @@
               <xdr:cNvPr id="12" name="Shape 10">
                 <a:extLst>
                   <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000C000000}"/>
+                    <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000C000000}"/>
                   </a:ext>
                 </a:extLst>
               </xdr:cNvPr>
@@ -1066,7 +1060,7 @@
                 <xdr:cNvPr id="13" name="Shape 11">
                   <a:extLst>
                     <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000D000000}"/>
+                      <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000D000000}"/>
                     </a:ext>
                   </a:extLst>
                 </xdr:cNvPr>
@@ -1111,7 +1105,7 @@
                 <xdr:cNvPr id="14" name="Shape 12">
                   <a:extLst>
                     <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000E000000}"/>
+                      <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000E000000}"/>
                     </a:ext>
                   </a:extLst>
                 </xdr:cNvPr>
@@ -1130,7 +1124,7 @@
                   <xdr:cNvPr id="15" name="Shape 13">
                     <a:extLst>
                       <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000F000000}"/>
+                        <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000F000000}"/>
                       </a:ext>
                     </a:extLst>
                   </xdr:cNvPr>
@@ -1175,7 +1169,7 @@
                   <xdr:cNvPr id="16" name="Shape 14">
                     <a:extLst>
                       <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000010000000}"/>
+                        <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000010000000}"/>
                       </a:ext>
                     </a:extLst>
                   </xdr:cNvPr>
@@ -1194,7 +1188,7 @@
                     <xdr:cNvPr id="17" name="Shape 15">
                       <a:extLst>
                         <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                          <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000011000000}"/>
+                          <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000011000000}"/>
                         </a:ext>
                       </a:extLst>
                     </xdr:cNvPr>
@@ -1239,7 +1233,7 @@
                     <xdr:cNvPr id="18" name="Shape 16">
                       <a:extLst>
                         <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                          <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000012000000}"/>
+                          <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000012000000}"/>
                         </a:ext>
                       </a:extLst>
                     </xdr:cNvPr>
@@ -1258,7 +1252,7 @@
                       <xdr:cNvPr id="19" name="Shape 17">
                         <a:extLst>
                           <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                            <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000013000000}"/>
+                            <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000013000000}"/>
                           </a:ext>
                         </a:extLst>
                       </xdr:cNvPr>
@@ -1303,7 +1297,7 @@
                       <xdr:cNvPr id="20" name="Shape 18">
                         <a:extLst>
                           <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                            <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000014000000}"/>
+                            <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000014000000}"/>
                           </a:ext>
                         </a:extLst>
                       </xdr:cNvPr>
@@ -1322,7 +1316,7 @@
                         <xdr:cNvPr id="21" name="Shape 19">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000015000000}"/>
+                              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000015000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -1373,7 +1367,7 @@
                         <xdr:cNvPr id="22" name="Shape 20">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000016000000}"/>
+                              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000016000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -1449,7 +1443,7 @@
                         <xdr:cNvPr id="23" name="Shape 21">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000017000000}"/>
+                              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000017000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -1517,7 +1511,7 @@
                         <xdr:cNvPr id="24" name="Shape 22">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000018000000}"/>
+                              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000018000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -1585,7 +1579,7 @@
                         <xdr:cNvPr id="25" name="Shape 23">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000019000000}"/>
+                              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000019000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -1634,14 +1628,17 @@
                           </a:pPr>
                           <a:r>
                             <a:rPr lang="en-US" sz="1000" b="0" i="0">
-                              <a:latin typeface="Arial"/>
+                              <a:latin typeface="Arial" pitchFamily="34" charset="0"/>
                               <a:ea typeface="Arial"/>
-                              <a:cs typeface="Arial"/>
+                              <a:cs typeface="Arial" pitchFamily="34" charset="0"/>
                               <a:sym typeface="Arial"/>
                             </a:rPr>
                             <a:t>MODELO INTEGRADO DE PLANEACIÓN Y GESTIÓN</a:t>
                           </a:r>
-                          <a:endParaRPr sz="1400"/>
+                          <a:endParaRPr sz="1400">
+                            <a:latin typeface="Arial" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Arial" pitchFamily="34" charset="0"/>
+                          </a:endParaRPr>
                         </a:p>
                         <a:p>
                           <a:pPr marL="0" lvl="0" indent="0" algn="ctr" rtl="1">
@@ -1659,18 +1656,18 @@
                             <a:buNone/>
                           </a:pPr>
                           <a:r>
-                            <a:rPr lang="en-US" sz="1000" b="0" i="0">
-                              <a:latin typeface="Arial"/>
+                            <a:rPr lang="es-MX" sz="1000">
+                              <a:latin typeface="Arial" pitchFamily="34" charset="0"/>
                               <a:ea typeface="Arial"/>
-                              <a:cs typeface="Arial"/>
+                              <a:cs typeface="Arial" pitchFamily="34" charset="0"/>
                               <a:sym typeface="Arial"/>
                             </a:rPr>
-                            <a:t>(MIPG)</a:t>
+                            <a:t> (MIPG)</a:t>
                           </a:r>
                           <a:endParaRPr sz="1000">
-                            <a:latin typeface="Arial"/>
+                            <a:latin typeface="Arial" pitchFamily="34" charset="0"/>
                             <a:ea typeface="Arial"/>
-                            <a:cs typeface="Arial"/>
+                            <a:cs typeface="Arial" pitchFamily="34" charset="0"/>
                             <a:sym typeface="Arial"/>
                           </a:endParaRPr>
                         </a:p>
@@ -1760,7 +1757,7 @@
                       <xdr:cNvPr id="26" name="Shape 24" descr="escudo">
                         <a:extLst>
                           <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                            <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001A000000}"/>
+                            <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001A000000}"/>
                           </a:ext>
                         </a:extLst>
                       </xdr:cNvPr>
@@ -1996,24 +1993,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="3" width="10.7109375" customWidth="1"/>
-    <col min="4" max="4" width="8.7109375" customWidth="1"/>
+    <col min="1" max="3" width="10.6640625" customWidth="1"/>
+    <col min="4" max="4" width="8.6640625" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
-    <col min="6" max="6" width="23.42578125" customWidth="1"/>
-    <col min="7" max="7" width="16.7109375" customWidth="1"/>
-    <col min="8" max="8" width="17.42578125" customWidth="1"/>
-    <col min="9" max="9" width="9.7109375" customWidth="1"/>
-    <col min="10" max="10" width="0.42578125" customWidth="1"/>
-    <col min="11" max="12" width="11.42578125" customWidth="1"/>
-    <col min="13" max="13" width="21.28515625" customWidth="1"/>
-    <col min="14" max="26" width="10.7109375" customWidth="1"/>
+    <col min="6" max="6" width="23.44140625" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="8" width="17.44140625" customWidth="1"/>
+    <col min="9" max="9" width="9.6640625" customWidth="1"/>
+    <col min="10" max="10" width="0.44140625" customWidth="1"/>
+    <col min="11" max="12" width="11.44140625" customWidth="1"/>
+    <col min="13" max="13" width="21.33203125" customWidth="1"/>
+    <col min="14" max="26" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="22"/>
       <c r="B1" s="23"/>
       <c r="C1" s="23"/>
@@ -2041,7 +2038,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="23"/>
       <c r="B2" s="23"/>
       <c r="C2" s="23"/>
@@ -2069,7 +2066,7 @@
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
     </row>
-    <row r="3" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="23"/>
       <c r="B3" s="23"/>
       <c r="C3" s="23"/>
@@ -2097,7 +2094,7 @@
       <c r="Y3" s="1"/>
       <c r="Z3" s="1"/>
     </row>
-    <row r="4" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="23"/>
       <c r="B4" s="23"/>
       <c r="C4" s="23"/>
@@ -2125,7 +2122,7 @@
       <c r="Y4" s="1"/>
       <c r="Z4" s="1"/>
     </row>
-    <row r="5" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="23"/>
       <c r="B5" s="23"/>
       <c r="C5" s="23"/>
@@ -2153,7 +2150,7 @@
       <c r="Y5" s="1"/>
       <c r="Z5" s="1"/>
     </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23"/>
       <c r="B6" s="23"/>
       <c r="C6" s="23"/>
@@ -2181,7 +2178,7 @@
       <c r="Y6" s="1"/>
       <c r="Z6" s="1"/>
     </row>
-    <row r="7" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="23"/>
       <c r="B7" s="23"/>
       <c r="C7" s="23"/>
@@ -2209,7 +2206,7 @@
       <c r="Y7" s="1"/>
       <c r="Z7" s="1"/>
     </row>
-    <row r="8" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="23"/>
       <c r="B8" s="23"/>
       <c r="C8" s="23"/>
@@ -2237,7 +2234,7 @@
       <c r="Y8" s="1"/>
       <c r="Z8" s="1"/>
     </row>
-    <row r="9" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="23"/>
       <c r="B9" s="23"/>
       <c r="C9" s="23"/>
@@ -2265,7 +2262,7 @@
       <c r="Y9" s="1"/>
       <c r="Z9" s="1"/>
     </row>
-    <row r="10" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="23"/>
       <c r="B10" s="23"/>
       <c r="C10" s="23"/>
@@ -2293,7 +2290,7 @@
       <c r="Y10" s="1"/>
       <c r="Z10" s="1"/>
     </row>
-    <row r="11" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="24" t="s">
         <v>0</v>
       </c>
@@ -2325,7 +2322,7 @@
       <c r="Y11" s="2"/>
       <c r="Z11" s="2"/>
     </row>
-    <row r="12" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="26" t="s">
         <v>1</v>
       </c>
@@ -2361,7 +2358,7 @@
       <c r="Y12" s="2"/>
       <c r="Z12" s="2"/>
     </row>
-    <row r="13" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="26" t="s">
         <v>4</v>
       </c>
@@ -2399,7 +2396,7 @@
       <c r="Y13" s="2"/>
       <c r="Z13" s="2"/>
     </row>
-    <row r="14" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="26" t="s">
         <v>7</v>
       </c>
@@ -2435,7 +2432,7 @@
       <c r="Y14" s="2"/>
       <c r="Z14" s="2"/>
     </row>
-    <row r="15" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="26" t="s">
         <v>10</v>
       </c>
@@ -2471,7 +2468,7 @@
       <c r="Y15" s="2"/>
       <c r="Z15" s="2"/>
     </row>
-    <row r="16" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="24" t="s">
         <v>13</v>
       </c>
@@ -2503,7 +2500,7 @@
       <c r="Y16" s="2"/>
       <c r="Z16" s="2"/>
     </row>
-    <row r="17" spans="1:26" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:26" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="26" t="s">
         <v>14</v>
       </c>
@@ -2535,7 +2532,7 @@
       <c r="Y17" s="2"/>
       <c r="Z17" s="2"/>
     </row>
-    <row r="18" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="26" t="s">
         <v>16</v>
       </c>
@@ -2567,7 +2564,7 @@
       <c r="Y18" s="2"/>
       <c r="Z18" s="2"/>
     </row>
-    <row r="19" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="26" t="s">
         <v>18</v>
       </c>
@@ -2599,7 +2596,7 @@
       <c r="Y19" s="2"/>
       <c r="Z19" s="2"/>
     </row>
-    <row r="20" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="47" t="s">
         <v>20</v>
       </c>
@@ -2631,7 +2628,7 @@
       <c r="Y20" s="2"/>
       <c r="Z20" s="2"/>
     </row>
-    <row r="21" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="58" t="s">
         <v>21</v>
       </c>
@@ -2661,7 +2658,7 @@
       <c r="Y21" s="2"/>
       <c r="Z21" s="2"/>
     </row>
-    <row r="22" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="44"/>
       <c r="B22" s="38"/>
       <c r="C22" s="39"/>
@@ -2689,7 +2686,7 @@
       <c r="Y22" s="2"/>
       <c r="Z22" s="2"/>
     </row>
-    <row r="23" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="40" t="s">
         <v>22</v>
       </c>
@@ -2719,7 +2716,7 @@
       <c r="Y23" s="2"/>
       <c r="Z23" s="2"/>
     </row>
-    <row r="24" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="47" t="s">
         <v>23</v>
       </c>
@@ -2751,7 +2748,7 @@
       <c r="Y24" s="2"/>
       <c r="Z24" s="2"/>
     </row>
-    <row r="25" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="41" t="s">
         <v>24</v>
       </c>
@@ -2783,7 +2780,7 @@
       <c r="Y25" s="2"/>
       <c r="Z25" s="2"/>
     </row>
-    <row r="26" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="44"/>
       <c r="B26" s="38"/>
       <c r="C26" s="39"/>
@@ -2813,7 +2810,7 @@
       <c r="Y26" s="2"/>
       <c r="Z26" s="2"/>
     </row>
-    <row r="27" spans="1:26" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:26" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="49" t="s">
         <v>27</v>
       </c>
@@ -2843,7 +2840,7 @@
       <c r="Y27" s="2"/>
       <c r="Z27" s="2"/>
     </row>
-    <row r="28" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="49" t="s">
         <v>28</v>
       </c>
@@ -2873,7 +2870,7 @@
       <c r="Y28" s="2"/>
       <c r="Z28" s="2"/>
     </row>
-    <row r="29" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -2901,7 +2898,7 @@
       <c r="Y29" s="2"/>
       <c r="Z29" s="2"/>
     </row>
-    <row r="30" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -2929,7 +2926,7 @@
       <c r="Y30" s="2"/>
       <c r="Z30" s="2"/>
     </row>
-    <row r="31" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -2957,7 +2954,7 @@
       <c r="Y31" s="2"/>
       <c r="Z31" s="2"/>
     </row>
-    <row r="32" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -2985,7 +2982,7 @@
       <c r="Y32" s="2"/>
       <c r="Z32" s="2"/>
     </row>
-    <row r="33" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -3013,7 +3010,7 @@
       <c r="Y33" s="2"/>
       <c r="Z33" s="2"/>
     </row>
-    <row r="34" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -3041,7 +3038,7 @@
       <c r="Y34" s="2"/>
       <c r="Z34" s="2"/>
     </row>
-    <row r="35" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -3069,7 +3066,7 @@
       <c r="Y35" s="2"/>
       <c r="Z35" s="2"/>
     </row>
-    <row r="36" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -3097,7 +3094,7 @@
       <c r="Y36" s="2"/>
       <c r="Z36" s="2"/>
     </row>
-    <row r="37" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -3125,7 +3122,7 @@
       <c r="Y37" s="2"/>
       <c r="Z37" s="2"/>
     </row>
-    <row r="38" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -3153,7 +3150,7 @@
       <c r="Y38" s="2"/>
       <c r="Z38" s="2"/>
     </row>
-    <row r="39" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -3181,7 +3178,7 @@
       <c r="Y39" s="2"/>
       <c r="Z39" s="2"/>
     </row>
-    <row r="40" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -3209,7 +3206,7 @@
       <c r="Y40" s="2"/>
       <c r="Z40" s="2"/>
     </row>
-    <row r="41" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -3237,7 +3234,7 @@
       <c r="Y41" s="2"/>
       <c r="Z41" s="2"/>
     </row>
-    <row r="42" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -3265,7 +3262,7 @@
       <c r="Y42" s="2"/>
       <c r="Z42" s="2"/>
     </row>
-    <row r="43" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -3293,7 +3290,7 @@
       <c r="Y43" s="2"/>
       <c r="Z43" s="2"/>
     </row>
-    <row r="44" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -3321,7 +3318,7 @@
       <c r="Y44" s="2"/>
       <c r="Z44" s="2"/>
     </row>
-    <row r="45" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -3349,7 +3346,7 @@
       <c r="Y45" s="2"/>
       <c r="Z45" s="2"/>
     </row>
-    <row r="46" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -3377,7 +3374,7 @@
       <c r="Y46" s="2"/>
       <c r="Z46" s="2"/>
     </row>
-    <row r="47" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
@@ -3405,7 +3402,7 @@
       <c r="Y47" s="2"/>
       <c r="Z47" s="2"/>
     </row>
-    <row r="48" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -3433,7 +3430,7 @@
       <c r="Y48" s="2"/>
       <c r="Z48" s="2"/>
     </row>
-    <row r="49" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -3461,7 +3458,7 @@
       <c r="Y49" s="2"/>
       <c r="Z49" s="2"/>
     </row>
-    <row r="50" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -3489,7 +3486,7 @@
       <c r="Y50" s="2"/>
       <c r="Z50" s="2"/>
     </row>
-    <row r="51" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
@@ -3517,7 +3514,7 @@
       <c r="Y51" s="2"/>
       <c r="Z51" s="2"/>
     </row>
-    <row r="52" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
@@ -3545,7 +3542,7 @@
       <c r="Y52" s="2"/>
       <c r="Z52" s="2"/>
     </row>
-    <row r="53" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
@@ -3573,7 +3570,7 @@
       <c r="Y53" s="2"/>
       <c r="Z53" s="2"/>
     </row>
-    <row r="54" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
@@ -3601,7 +3598,7 @@
       <c r="Y54" s="2"/>
       <c r="Z54" s="2"/>
     </row>
-    <row r="55" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -3629,7 +3626,7 @@
       <c r="Y55" s="2"/>
       <c r="Z55" s="2"/>
     </row>
-    <row r="56" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
@@ -3657,7 +3654,7 @@
       <c r="Y56" s="2"/>
       <c r="Z56" s="2"/>
     </row>
-    <row r="57" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
@@ -3685,7 +3682,7 @@
       <c r="Y57" s="2"/>
       <c r="Z57" s="2"/>
     </row>
-    <row r="58" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
@@ -3713,7 +3710,7 @@
       <c r="Y58" s="2"/>
       <c r="Z58" s="2"/>
     </row>
-    <row r="59" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
@@ -3741,7 +3738,7 @@
       <c r="Y59" s="2"/>
       <c r="Z59" s="2"/>
     </row>
-    <row r="60" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
@@ -3769,7 +3766,7 @@
       <c r="Y60" s="2"/>
       <c r="Z60" s="2"/>
     </row>
-    <row r="61" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
@@ -3797,7 +3794,7 @@
       <c r="Y61" s="2"/>
       <c r="Z61" s="2"/>
     </row>
-    <row r="62" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
@@ -3825,7 +3822,7 @@
       <c r="Y62" s="2"/>
       <c r="Z62" s="2"/>
     </row>
-    <row r="63" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -3853,7 +3850,7 @@
       <c r="Y63" s="2"/>
       <c r="Z63" s="2"/>
     </row>
-    <row r="64" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
@@ -3881,7 +3878,7 @@
       <c r="Y64" s="2"/>
       <c r="Z64" s="2"/>
     </row>
-    <row r="65" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
@@ -3909,7 +3906,7 @@
       <c r="Y65" s="2"/>
       <c r="Z65" s="2"/>
     </row>
-    <row r="66" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
@@ -3937,7 +3934,7 @@
       <c r="Y66" s="2"/>
       <c r="Z66" s="2"/>
     </row>
-    <row r="67" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
@@ -3965,7 +3962,7 @@
       <c r="Y67" s="2"/>
       <c r="Z67" s="2"/>
     </row>
-    <row r="68" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
@@ -3993,7 +3990,7 @@
       <c r="Y68" s="2"/>
       <c r="Z68" s="2"/>
     </row>
-    <row r="69" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
@@ -4021,7 +4018,7 @@
       <c r="Y69" s="2"/>
       <c r="Z69" s="2"/>
     </row>
-    <row r="70" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
@@ -4049,7 +4046,7 @@
       <c r="Y70" s="2"/>
       <c r="Z70" s="2"/>
     </row>
-    <row r="71" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
@@ -4077,7 +4074,7 @@
       <c r="Y71" s="2"/>
       <c r="Z71" s="2"/>
     </row>
-    <row r="72" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
@@ -4105,7 +4102,7 @@
       <c r="Y72" s="2"/>
       <c r="Z72" s="2"/>
     </row>
-    <row r="73" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
@@ -4133,7 +4130,7 @@
       <c r="Y73" s="2"/>
       <c r="Z73" s="2"/>
     </row>
-    <row r="74" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="2"/>
       <c r="B74" s="2"/>
       <c r="C74" s="2"/>
@@ -4161,7 +4158,7 @@
       <c r="Y74" s="2"/>
       <c r="Z74" s="2"/>
     </row>
-    <row r="75" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
@@ -4189,7 +4186,7 @@
       <c r="Y75" s="2"/>
       <c r="Z75" s="2"/>
     </row>
-    <row r="76" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
@@ -4217,7 +4214,7 @@
       <c r="Y76" s="2"/>
       <c r="Z76" s="2"/>
     </row>
-    <row r="77" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
@@ -4245,7 +4242,7 @@
       <c r="Y77" s="2"/>
       <c r="Z77" s="2"/>
     </row>
-    <row r="78" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
@@ -4273,7 +4270,7 @@
       <c r="Y78" s="2"/>
       <c r="Z78" s="2"/>
     </row>
-    <row r="79" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
@@ -4301,7 +4298,7 @@
       <c r="Y79" s="2"/>
       <c r="Z79" s="2"/>
     </row>
-    <row r="80" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="2"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
@@ -4329,7 +4326,7 @@
       <c r="Y80" s="2"/>
       <c r="Z80" s="2"/>
     </row>
-    <row r="81" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
@@ -4357,7 +4354,7 @@
       <c r="Y81" s="2"/>
       <c r="Z81" s="2"/>
     </row>
-    <row r="82" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
@@ -4385,7 +4382,7 @@
       <c r="Y82" s="2"/>
       <c r="Z82" s="2"/>
     </row>
-    <row r="83" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
@@ -4413,7 +4410,7 @@
       <c r="Y83" s="2"/>
       <c r="Z83" s="2"/>
     </row>
-    <row r="84" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
@@ -4441,7 +4438,7 @@
       <c r="Y84" s="2"/>
       <c r="Z84" s="2"/>
     </row>
-    <row r="85" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
@@ -4469,7 +4466,7 @@
       <c r="Y85" s="2"/>
       <c r="Z85" s="2"/>
     </row>
-    <row r="86" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
@@ -4497,7 +4494,7 @@
       <c r="Y86" s="2"/>
       <c r="Z86" s="2"/>
     </row>
-    <row r="87" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
@@ -4525,7 +4522,7 @@
       <c r="Y87" s="2"/>
       <c r="Z87" s="2"/>
     </row>
-    <row r="88" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
@@ -4553,7 +4550,7 @@
       <c r="Y88" s="2"/>
       <c r="Z88" s="2"/>
     </row>
-    <row r="89" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
@@ -4581,7 +4578,7 @@
       <c r="Y89" s="2"/>
       <c r="Z89" s="2"/>
     </row>
-    <row r="90" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
@@ -4609,7 +4606,7 @@
       <c r="Y90" s="2"/>
       <c r="Z90" s="2"/>
     </row>
-    <row r="91" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
@@ -4637,7 +4634,7 @@
       <c r="Y91" s="2"/>
       <c r="Z91" s="2"/>
     </row>
-    <row r="92" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
@@ -4665,7 +4662,7 @@
       <c r="Y92" s="2"/>
       <c r="Z92" s="2"/>
     </row>
-    <row r="93" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
@@ -4693,7 +4690,7 @@
       <c r="Y93" s="2"/>
       <c r="Z93" s="2"/>
     </row>
-    <row r="94" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
@@ -4721,7 +4718,7 @@
       <c r="Y94" s="2"/>
       <c r="Z94" s="2"/>
     </row>
-    <row r="95" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
@@ -4749,7 +4746,7 @@
       <c r="Y95" s="2"/>
       <c r="Z95" s="2"/>
     </row>
-    <row r="96" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
@@ -4777,7 +4774,7 @@
       <c r="Y96" s="2"/>
       <c r="Z96" s="2"/>
     </row>
-    <row r="97" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
@@ -4805,7 +4802,7 @@
       <c r="Y97" s="2"/>
       <c r="Z97" s="2"/>
     </row>
-    <row r="98" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
@@ -4833,7 +4830,7 @@
       <c r="Y98" s="2"/>
       <c r="Z98" s="2"/>
     </row>
-    <row r="99" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
@@ -4861,7 +4858,7 @@
       <c r="Y99" s="2"/>
       <c r="Z99" s="2"/>
     </row>
-    <row r="100" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
@@ -4889,7 +4886,7 @@
       <c r="Y100" s="2"/>
       <c r="Z100" s="2"/>
     </row>
-    <row r="101" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="2"/>
       <c r="B101" s="2"/>
       <c r="C101" s="2"/>
@@ -4917,7 +4914,7 @@
       <c r="Y101" s="2"/>
       <c r="Z101" s="2"/>
     </row>
-    <row r="102" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="2"/>
       <c r="B102" s="2"/>
       <c r="C102" s="2"/>
@@ -4945,7 +4942,7 @@
       <c r="Y102" s="2"/>
       <c r="Z102" s="2"/>
     </row>
-    <row r="103" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="2"/>
       <c r="B103" s="2"/>
       <c r="C103" s="2"/>
@@ -4973,7 +4970,7 @@
       <c r="Y103" s="2"/>
       <c r="Z103" s="2"/>
     </row>
-    <row r="104" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="2"/>
       <c r="B104" s="2"/>
       <c r="C104" s="2"/>
@@ -5001,7 +4998,7 @@
       <c r="Y104" s="2"/>
       <c r="Z104" s="2"/>
     </row>
-    <row r="105" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="2"/>
       <c r="B105" s="2"/>
       <c r="C105" s="2"/>
@@ -5029,7 +5026,7 @@
       <c r="Y105" s="2"/>
       <c r="Z105" s="2"/>
     </row>
-    <row r="106" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="2"/>
       <c r="B106" s="2"/>
       <c r="C106" s="2"/>
@@ -5057,7 +5054,7 @@
       <c r="Y106" s="2"/>
       <c r="Z106" s="2"/>
     </row>
-    <row r="107" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="2"/>
       <c r="B107" s="2"/>
       <c r="C107" s="2"/>
@@ -5085,7 +5082,7 @@
       <c r="Y107" s="2"/>
       <c r="Z107" s="2"/>
     </row>
-    <row r="108" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="2"/>
       <c r="B108" s="2"/>
       <c r="C108" s="2"/>
@@ -5113,7 +5110,7 @@
       <c r="Y108" s="2"/>
       <c r="Z108" s="2"/>
     </row>
-    <row r="109" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="2"/>
       <c r="B109" s="2"/>
       <c r="C109" s="2"/>
@@ -5141,7 +5138,7 @@
       <c r="Y109" s="2"/>
       <c r="Z109" s="2"/>
     </row>
-    <row r="110" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="2"/>
       <c r="B110" s="2"/>
       <c r="C110" s="2"/>
@@ -5169,7 +5166,7 @@
       <c r="Y110" s="2"/>
       <c r="Z110" s="2"/>
     </row>
-    <row r="111" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
       <c r="C111" s="2"/>
@@ -5197,7 +5194,7 @@
       <c r="Y111" s="2"/>
       <c r="Z111" s="2"/>
     </row>
-    <row r="112" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="C112" s="2"/>
@@ -5225,7 +5222,7 @@
       <c r="Y112" s="2"/>
       <c r="Z112" s="2"/>
     </row>
-    <row r="113" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="2"/>
@@ -5253,7 +5250,7 @@
       <c r="Y113" s="2"/>
       <c r="Z113" s="2"/>
     </row>
-    <row r="114" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="2"/>
@@ -5281,7 +5278,7 @@
       <c r="Y114" s="2"/>
       <c r="Z114" s="2"/>
     </row>
-    <row r="115" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="2"/>
       <c r="B115" s="2"/>
       <c r="C115" s="2"/>
@@ -5309,7 +5306,7 @@
       <c r="Y115" s="2"/>
       <c r="Z115" s="2"/>
     </row>
-    <row r="116" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="2"/>
       <c r="B116" s="2"/>
       <c r="C116" s="2"/>
@@ -5337,7 +5334,7 @@
       <c r="Y116" s="2"/>
       <c r="Z116" s="2"/>
     </row>
-    <row r="117" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="2"/>
       <c r="B117" s="2"/>
       <c r="C117" s="2"/>
@@ -5365,7 +5362,7 @@
       <c r="Y117" s="2"/>
       <c r="Z117" s="2"/>
     </row>
-    <row r="118" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="2"/>
       <c r="B118" s="2"/>
       <c r="C118" s="2"/>
@@ -5393,7 +5390,7 @@
       <c r="Y118" s="2"/>
       <c r="Z118" s="2"/>
     </row>
-    <row r="119" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="2"/>
       <c r="B119" s="2"/>
       <c r="C119" s="2"/>
@@ -5421,7 +5418,7 @@
       <c r="Y119" s="2"/>
       <c r="Z119" s="2"/>
     </row>
-    <row r="120" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="2"/>
       <c r="B120" s="2"/>
       <c r="C120" s="2"/>
@@ -5449,7 +5446,7 @@
       <c r="Y120" s="2"/>
       <c r="Z120" s="2"/>
     </row>
-    <row r="121" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="2"/>
       <c r="B121" s="2"/>
       <c r="C121" s="2"/>
@@ -5477,7 +5474,7 @@
       <c r="Y121" s="2"/>
       <c r="Z121" s="2"/>
     </row>
-    <row r="122" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="2"/>
       <c r="B122" s="2"/>
       <c r="C122" s="2"/>
@@ -5505,7 +5502,7 @@
       <c r="Y122" s="2"/>
       <c r="Z122" s="2"/>
     </row>
-    <row r="123" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A123" s="2"/>
       <c r="B123" s="2"/>
       <c r="C123" s="2"/>
@@ -5533,7 +5530,7 @@
       <c r="Y123" s="2"/>
       <c r="Z123" s="2"/>
     </row>
-    <row r="124" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A124" s="2"/>
       <c r="B124" s="2"/>
       <c r="C124" s="2"/>
@@ -5561,7 +5558,7 @@
       <c r="Y124" s="2"/>
       <c r="Z124" s="2"/>
     </row>
-    <row r="125" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A125" s="2"/>
       <c r="B125" s="2"/>
       <c r="C125" s="2"/>
@@ -5589,7 +5586,7 @@
       <c r="Y125" s="2"/>
       <c r="Z125" s="2"/>
     </row>
-    <row r="126" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="2"/>
       <c r="B126" s="2"/>
       <c r="C126" s="2"/>
@@ -5617,7 +5614,7 @@
       <c r="Y126" s="2"/>
       <c r="Z126" s="2"/>
     </row>
-    <row r="127" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="2"/>
       <c r="B127" s="2"/>
       <c r="C127" s="2"/>
@@ -5645,7 +5642,7 @@
       <c r="Y127" s="2"/>
       <c r="Z127" s="2"/>
     </row>
-    <row r="128" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A128" s="2"/>
       <c r="B128" s="2"/>
       <c r="C128" s="2"/>
@@ -5673,7 +5670,7 @@
       <c r="Y128" s="2"/>
       <c r="Z128" s="2"/>
     </row>
-    <row r="129" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A129" s="2"/>
       <c r="B129" s="2"/>
       <c r="C129" s="2"/>
@@ -5701,7 +5698,7 @@
       <c r="Y129" s="2"/>
       <c r="Z129" s="2"/>
     </row>
-    <row r="130" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="2"/>
       <c r="B130" s="2"/>
       <c r="C130" s="2"/>
@@ -5729,7 +5726,7 @@
       <c r="Y130" s="2"/>
       <c r="Z130" s="2"/>
     </row>
-    <row r="131" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="2"/>
       <c r="B131" s="2"/>
       <c r="C131" s="2"/>
@@ -5757,7 +5754,7 @@
       <c r="Y131" s="2"/>
       <c r="Z131" s="2"/>
     </row>
-    <row r="132" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A132" s="2"/>
       <c r="B132" s="2"/>
       <c r="C132" s="2"/>
@@ -5785,7 +5782,7 @@
       <c r="Y132" s="2"/>
       <c r="Z132" s="2"/>
     </row>
-    <row r="133" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A133" s="2"/>
       <c r="B133" s="2"/>
       <c r="C133" s="2"/>
@@ -5813,7 +5810,7 @@
       <c r="Y133" s="2"/>
       <c r="Z133" s="2"/>
     </row>
-    <row r="134" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" s="2"/>
       <c r="B134" s="2"/>
       <c r="C134" s="2"/>
@@ -5841,7 +5838,7 @@
       <c r="Y134" s="2"/>
       <c r="Z134" s="2"/>
     </row>
-    <row r="135" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A135" s="2"/>
       <c r="B135" s="2"/>
       <c r="C135" s="2"/>
@@ -5869,7 +5866,7 @@
       <c r="Y135" s="2"/>
       <c r="Z135" s="2"/>
     </row>
-    <row r="136" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A136" s="2"/>
       <c r="B136" s="2"/>
       <c r="C136" s="2"/>
@@ -5897,7 +5894,7 @@
       <c r="Y136" s="2"/>
       <c r="Z136" s="2"/>
     </row>
-    <row r="137" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A137" s="2"/>
       <c r="B137" s="2"/>
       <c r="C137" s="2"/>
@@ -5925,7 +5922,7 @@
       <c r="Y137" s="2"/>
       <c r="Z137" s="2"/>
     </row>
-    <row r="138" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" s="2"/>
       <c r="B138" s="2"/>
       <c r="C138" s="2"/>
@@ -5953,7 +5950,7 @@
       <c r="Y138" s="2"/>
       <c r="Z138" s="2"/>
     </row>
-    <row r="139" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A139" s="2"/>
       <c r="B139" s="2"/>
       <c r="C139" s="2"/>
@@ -5981,7 +5978,7 @@
       <c r="Y139" s="2"/>
       <c r="Z139" s="2"/>
     </row>
-    <row r="140" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A140" s="2"/>
       <c r="B140" s="2"/>
       <c r="C140" s="2"/>
@@ -6009,7 +6006,7 @@
       <c r="Y140" s="2"/>
       <c r="Z140" s="2"/>
     </row>
-    <row r="141" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A141" s="2"/>
       <c r="B141" s="2"/>
       <c r="C141" s="2"/>
@@ -6037,7 +6034,7 @@
       <c r="Y141" s="2"/>
       <c r="Z141" s="2"/>
     </row>
-    <row r="142" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="2"/>
       <c r="B142" s="2"/>
       <c r="C142" s="2"/>
@@ -6065,7 +6062,7 @@
       <c r="Y142" s="2"/>
       <c r="Z142" s="2"/>
     </row>
-    <row r="143" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A143" s="2"/>
       <c r="B143" s="2"/>
       <c r="C143" s="2"/>
@@ -6093,7 +6090,7 @@
       <c r="Y143" s="2"/>
       <c r="Z143" s="2"/>
     </row>
-    <row r="144" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A144" s="2"/>
       <c r="B144" s="2"/>
       <c r="C144" s="2"/>
@@ -6121,7 +6118,7 @@
       <c r="Y144" s="2"/>
       <c r="Z144" s="2"/>
     </row>
-    <row r="145" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A145" s="2"/>
       <c r="B145" s="2"/>
       <c r="C145" s="2"/>
@@ -6149,7 +6146,7 @@
       <c r="Y145" s="2"/>
       <c r="Z145" s="2"/>
     </row>
-    <row r="146" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" s="2"/>
       <c r="B146" s="2"/>
       <c r="C146" s="2"/>
@@ -6177,7 +6174,7 @@
       <c r="Y146" s="2"/>
       <c r="Z146" s="2"/>
     </row>
-    <row r="147" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="2"/>
       <c r="B147" s="2"/>
       <c r="C147" s="2"/>
@@ -6205,7 +6202,7 @@
       <c r="Y147" s="2"/>
       <c r="Z147" s="2"/>
     </row>
-    <row r="148" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A148" s="2"/>
       <c r="B148" s="2"/>
       <c r="C148" s="2"/>
@@ -6233,7 +6230,7 @@
       <c r="Y148" s="2"/>
       <c r="Z148" s="2"/>
     </row>
-    <row r="149" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A149" s="2"/>
       <c r="B149" s="2"/>
       <c r="C149" s="2"/>
@@ -6261,7 +6258,7 @@
       <c r="Y149" s="2"/>
       <c r="Z149" s="2"/>
     </row>
-    <row r="150" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="2"/>
       <c r="B150" s="2"/>
       <c r="C150" s="2"/>
@@ -6289,7 +6286,7 @@
       <c r="Y150" s="2"/>
       <c r="Z150" s="2"/>
     </row>
-    <row r="151" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A151" s="2"/>
       <c r="B151" s="2"/>
       <c r="C151" s="2"/>
@@ -6317,7 +6314,7 @@
       <c r="Y151" s="2"/>
       <c r="Z151" s="2"/>
     </row>
-    <row r="152" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A152" s="2"/>
       <c r="B152" s="2"/>
       <c r="C152" s="2"/>
@@ -6345,7 +6342,7 @@
       <c r="Y152" s="2"/>
       <c r="Z152" s="2"/>
     </row>
-    <row r="153" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A153" s="2"/>
       <c r="B153" s="2"/>
       <c r="C153" s="2"/>
@@ -6373,7 +6370,7 @@
       <c r="Y153" s="2"/>
       <c r="Z153" s="2"/>
     </row>
-    <row r="154" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A154" s="2"/>
       <c r="B154" s="2"/>
       <c r="C154" s="2"/>
@@ -6401,7 +6398,7 @@
       <c r="Y154" s="2"/>
       <c r="Z154" s="2"/>
     </row>
-    <row r="155" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A155" s="2"/>
       <c r="B155" s="2"/>
       <c r="C155" s="2"/>
@@ -6429,7 +6426,7 @@
       <c r="Y155" s="2"/>
       <c r="Z155" s="2"/>
     </row>
-    <row r="156" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A156" s="2"/>
       <c r="B156" s="2"/>
       <c r="C156" s="2"/>
@@ -6457,7 +6454,7 @@
       <c r="Y156" s="2"/>
       <c r="Z156" s="2"/>
     </row>
-    <row r="157" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A157" s="2"/>
       <c r="B157" s="2"/>
       <c r="C157" s="2"/>
@@ -6485,7 +6482,7 @@
       <c r="Y157" s="2"/>
       <c r="Z157" s="2"/>
     </row>
-    <row r="158" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" s="2"/>
       <c r="B158" s="2"/>
       <c r="C158" s="2"/>
@@ -6513,7 +6510,7 @@
       <c r="Y158" s="2"/>
       <c r="Z158" s="2"/>
     </row>
-    <row r="159" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A159" s="2"/>
       <c r="B159" s="2"/>
       <c r="C159" s="2"/>
@@ -6541,7 +6538,7 @@
       <c r="Y159" s="2"/>
       <c r="Z159" s="2"/>
     </row>
-    <row r="160" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A160" s="2"/>
       <c r="B160" s="2"/>
       <c r="C160" s="2"/>
@@ -6569,7 +6566,7 @@
       <c r="Y160" s="2"/>
       <c r="Z160" s="2"/>
     </row>
-    <row r="161" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A161" s="2"/>
       <c r="B161" s="2"/>
       <c r="C161" s="2"/>
@@ -6597,7 +6594,7 @@
       <c r="Y161" s="2"/>
       <c r="Z161" s="2"/>
     </row>
-    <row r="162" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A162" s="2"/>
       <c r="B162" s="2"/>
       <c r="C162" s="2"/>
@@ -6625,7 +6622,7 @@
       <c r="Y162" s="2"/>
       <c r="Z162" s="2"/>
     </row>
-    <row r="163" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A163" s="2"/>
       <c r="B163" s="2"/>
       <c r="C163" s="2"/>
@@ -6653,7 +6650,7 @@
       <c r="Y163" s="2"/>
       <c r="Z163" s="2"/>
     </row>
-    <row r="164" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A164" s="2"/>
       <c r="B164" s="2"/>
       <c r="C164" s="2"/>
@@ -6681,7 +6678,7 @@
       <c r="Y164" s="2"/>
       <c r="Z164" s="2"/>
     </row>
-    <row r="165" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A165" s="2"/>
       <c r="B165" s="2"/>
       <c r="C165" s="2"/>
@@ -6709,7 +6706,7 @@
       <c r="Y165" s="2"/>
       <c r="Z165" s="2"/>
     </row>
-    <row r="166" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A166" s="2"/>
       <c r="B166" s="2"/>
       <c r="C166" s="2"/>
@@ -6737,7 +6734,7 @@
       <c r="Y166" s="2"/>
       <c r="Z166" s="2"/>
     </row>
-    <row r="167" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A167" s="2"/>
       <c r="B167" s="2"/>
       <c r="C167" s="2"/>
@@ -6765,7 +6762,7 @@
       <c r="Y167" s="2"/>
       <c r="Z167" s="2"/>
     </row>
-    <row r="168" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A168" s="2"/>
       <c r="B168" s="2"/>
       <c r="C168" s="2"/>
@@ -6793,7 +6790,7 @@
       <c r="Y168" s="2"/>
       <c r="Z168" s="2"/>
     </row>
-    <row r="169" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A169" s="2"/>
       <c r="B169" s="2"/>
       <c r="C169" s="2"/>
@@ -6821,7 +6818,7 @@
       <c r="Y169" s="2"/>
       <c r="Z169" s="2"/>
     </row>
-    <row r="170" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A170" s="2"/>
       <c r="B170" s="2"/>
       <c r="C170" s="2"/>
@@ -6849,7 +6846,7 @@
       <c r="Y170" s="2"/>
       <c r="Z170" s="2"/>
     </row>
-    <row r="171" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A171" s="2"/>
       <c r="B171" s="2"/>
       <c r="C171" s="2"/>
@@ -6877,7 +6874,7 @@
       <c r="Y171" s="2"/>
       <c r="Z171" s="2"/>
     </row>
-    <row r="172" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A172" s="2"/>
       <c r="B172" s="2"/>
       <c r="C172" s="2"/>
@@ -6905,7 +6902,7 @@
       <c r="Y172" s="2"/>
       <c r="Z172" s="2"/>
     </row>
-    <row r="173" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A173" s="2"/>
       <c r="B173" s="2"/>
       <c r="C173" s="2"/>
@@ -6933,7 +6930,7 @@
       <c r="Y173" s="2"/>
       <c r="Z173" s="2"/>
     </row>
-    <row r="174" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A174" s="2"/>
       <c r="B174" s="2"/>
       <c r="C174" s="2"/>
@@ -6961,7 +6958,7 @@
       <c r="Y174" s="2"/>
       <c r="Z174" s="2"/>
     </row>
-    <row r="175" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A175" s="2"/>
       <c r="B175" s="2"/>
       <c r="C175" s="2"/>
@@ -6989,7 +6986,7 @@
       <c r="Y175" s="2"/>
       <c r="Z175" s="2"/>
     </row>
-    <row r="176" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A176" s="2"/>
       <c r="B176" s="2"/>
       <c r="C176" s="2"/>
@@ -7017,7 +7014,7 @@
       <c r="Y176" s="2"/>
       <c r="Z176" s="2"/>
     </row>
-    <row r="177" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A177" s="2"/>
       <c r="B177" s="2"/>
       <c r="C177" s="2"/>
@@ -7045,7 +7042,7 @@
       <c r="Y177" s="2"/>
       <c r="Z177" s="2"/>
     </row>
-    <row r="178" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A178" s="2"/>
       <c r="B178" s="2"/>
       <c r="C178" s="2"/>
@@ -7073,7 +7070,7 @@
       <c r="Y178" s="2"/>
       <c r="Z178" s="2"/>
     </row>
-    <row r="179" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A179" s="2"/>
       <c r="B179" s="2"/>
       <c r="C179" s="2"/>
@@ -7101,7 +7098,7 @@
       <c r="Y179" s="2"/>
       <c r="Z179" s="2"/>
     </row>
-    <row r="180" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A180" s="2"/>
       <c r="B180" s="2"/>
       <c r="C180" s="2"/>
@@ -7129,7 +7126,7 @@
       <c r="Y180" s="2"/>
       <c r="Z180" s="2"/>
     </row>
-    <row r="181" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A181" s="2"/>
       <c r="B181" s="2"/>
       <c r="C181" s="2"/>
@@ -7157,7 +7154,7 @@
       <c r="Y181" s="2"/>
       <c r="Z181" s="2"/>
     </row>
-    <row r="182" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A182" s="2"/>
       <c r="B182" s="2"/>
       <c r="C182" s="2"/>
@@ -7185,7 +7182,7 @@
       <c r="Y182" s="2"/>
       <c r="Z182" s="2"/>
     </row>
-    <row r="183" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A183" s="2"/>
       <c r="B183" s="2"/>
       <c r="C183" s="2"/>
@@ -7213,7 +7210,7 @@
       <c r="Y183" s="2"/>
       <c r="Z183" s="2"/>
     </row>
-    <row r="184" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A184" s="2"/>
       <c r="B184" s="2"/>
       <c r="C184" s="2"/>
@@ -7241,7 +7238,7 @@
       <c r="Y184" s="2"/>
       <c r="Z184" s="2"/>
     </row>
-    <row r="185" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A185" s="2"/>
       <c r="B185" s="2"/>
       <c r="C185" s="2"/>
@@ -7269,7 +7266,7 @@
       <c r="Y185" s="2"/>
       <c r="Z185" s="2"/>
     </row>
-    <row r="186" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A186" s="2"/>
       <c r="B186" s="2"/>
       <c r="C186" s="2"/>
@@ -7297,7 +7294,7 @@
       <c r="Y186" s="2"/>
       <c r="Z186" s="2"/>
     </row>
-    <row r="187" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A187" s="2"/>
       <c r="B187" s="2"/>
       <c r="C187" s="2"/>
@@ -7325,7 +7322,7 @@
       <c r="Y187" s="2"/>
       <c r="Z187" s="2"/>
     </row>
-    <row r="188" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A188" s="2"/>
       <c r="B188" s="2"/>
       <c r="C188" s="2"/>
@@ -7353,7 +7350,7 @@
       <c r="Y188" s="2"/>
       <c r="Z188" s="2"/>
     </row>
-    <row r="189" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A189" s="2"/>
       <c r="B189" s="2"/>
       <c r="C189" s="2"/>
@@ -7381,7 +7378,7 @@
       <c r="Y189" s="2"/>
       <c r="Z189" s="2"/>
     </row>
-    <row r="190" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A190" s="2"/>
       <c r="B190" s="2"/>
       <c r="C190" s="2"/>
@@ -7409,7 +7406,7 @@
       <c r="Y190" s="2"/>
       <c r="Z190" s="2"/>
     </row>
-    <row r="191" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A191" s="2"/>
       <c r="B191" s="2"/>
       <c r="C191" s="2"/>
@@ -7437,7 +7434,7 @@
       <c r="Y191" s="2"/>
       <c r="Z191" s="2"/>
     </row>
-    <row r="192" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A192" s="2"/>
       <c r="B192" s="2"/>
       <c r="C192" s="2"/>
@@ -7465,7 +7462,7 @@
       <c r="Y192" s="2"/>
       <c r="Z192" s="2"/>
     </row>
-    <row r="193" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A193" s="2"/>
       <c r="B193" s="2"/>
       <c r="C193" s="2"/>
@@ -7493,7 +7490,7 @@
       <c r="Y193" s="2"/>
       <c r="Z193" s="2"/>
     </row>
-    <row r="194" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A194" s="2"/>
       <c r="B194" s="2"/>
       <c r="C194" s="2"/>
@@ -7521,7 +7518,7 @@
       <c r="Y194" s="2"/>
       <c r="Z194" s="2"/>
     </row>
-    <row r="195" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A195" s="2"/>
       <c r="B195" s="2"/>
       <c r="C195" s="2"/>
@@ -7549,7 +7546,7 @@
       <c r="Y195" s="2"/>
       <c r="Z195" s="2"/>
     </row>
-    <row r="196" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A196" s="2"/>
       <c r="B196" s="2"/>
       <c r="C196" s="2"/>
@@ -7577,7 +7574,7 @@
       <c r="Y196" s="2"/>
       <c r="Z196" s="2"/>
     </row>
-    <row r="197" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A197" s="2"/>
       <c r="B197" s="2"/>
       <c r="C197" s="2"/>
@@ -7605,7 +7602,7 @@
       <c r="Y197" s="2"/>
       <c r="Z197" s="2"/>
     </row>
-    <row r="198" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A198" s="2"/>
       <c r="B198" s="2"/>
       <c r="C198" s="2"/>
@@ -7633,7 +7630,7 @@
       <c r="Y198" s="2"/>
       <c r="Z198" s="2"/>
     </row>
-    <row r="199" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A199" s="2"/>
       <c r="B199" s="2"/>
       <c r="C199" s="2"/>
@@ -7661,7 +7658,7 @@
       <c r="Y199" s="2"/>
       <c r="Z199" s="2"/>
     </row>
-    <row r="200" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A200" s="2"/>
       <c r="B200" s="2"/>
       <c r="C200" s="2"/>
@@ -7689,7 +7686,7 @@
       <c r="Y200" s="2"/>
       <c r="Z200" s="2"/>
     </row>
-    <row r="201" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A201" s="2"/>
       <c r="B201" s="2"/>
       <c r="C201" s="2"/>
@@ -7717,7 +7714,7 @@
       <c r="Y201" s="2"/>
       <c r="Z201" s="2"/>
     </row>
-    <row r="202" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A202" s="2"/>
       <c r="B202" s="2"/>
       <c r="C202" s="2"/>
@@ -7745,7 +7742,7 @@
       <c r="Y202" s="2"/>
       <c r="Z202" s="2"/>
     </row>
-    <row r="203" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A203" s="2"/>
       <c r="B203" s="2"/>
       <c r="C203" s="2"/>
@@ -7773,7 +7770,7 @@
       <c r="Y203" s="2"/>
       <c r="Z203" s="2"/>
     </row>
-    <row r="204" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A204" s="2"/>
       <c r="B204" s="2"/>
       <c r="C204" s="2"/>
@@ -7801,7 +7798,7 @@
       <c r="Y204" s="2"/>
       <c r="Z204" s="2"/>
     </row>
-    <row r="205" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A205" s="2"/>
       <c r="B205" s="2"/>
       <c r="C205" s="2"/>
@@ -7829,7 +7826,7 @@
       <c r="Y205" s="2"/>
       <c r="Z205" s="2"/>
     </row>
-    <row r="206" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A206" s="2"/>
       <c r="B206" s="2"/>
       <c r="C206" s="2"/>
@@ -7857,7 +7854,7 @@
       <c r="Y206" s="2"/>
       <c r="Z206" s="2"/>
     </row>
-    <row r="207" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A207" s="2"/>
       <c r="B207" s="2"/>
       <c r="C207" s="2"/>
@@ -7885,7 +7882,7 @@
       <c r="Y207" s="2"/>
       <c r="Z207" s="2"/>
     </row>
-    <row r="208" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A208" s="2"/>
       <c r="B208" s="2"/>
       <c r="C208" s="2"/>
@@ -7913,7 +7910,7 @@
       <c r="Y208" s="2"/>
       <c r="Z208" s="2"/>
     </row>
-    <row r="209" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A209" s="2"/>
       <c r="B209" s="2"/>
       <c r="C209" s="2"/>
@@ -7941,7 +7938,7 @@
       <c r="Y209" s="2"/>
       <c r="Z209" s="2"/>
     </row>
-    <row r="210" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A210" s="2"/>
       <c r="B210" s="2"/>
       <c r="C210" s="2"/>
@@ -7969,7 +7966,7 @@
       <c r="Y210" s="2"/>
       <c r="Z210" s="2"/>
     </row>
-    <row r="211" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A211" s="2"/>
       <c r="B211" s="2"/>
       <c r="C211" s="2"/>
@@ -7997,7 +7994,7 @@
       <c r="Y211" s="2"/>
       <c r="Z211" s="2"/>
     </row>
-    <row r="212" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A212" s="2"/>
       <c r="B212" s="2"/>
       <c r="C212" s="2"/>
@@ -8025,7 +8022,7 @@
       <c r="Y212" s="2"/>
       <c r="Z212" s="2"/>
     </row>
-    <row r="213" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A213" s="2"/>
       <c r="B213" s="2"/>
       <c r="C213" s="2"/>
@@ -8053,7 +8050,7 @@
       <c r="Y213" s="2"/>
       <c r="Z213" s="2"/>
     </row>
-    <row r="214" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A214" s="2"/>
       <c r="B214" s="2"/>
       <c r="C214" s="2"/>
@@ -8081,7 +8078,7 @@
       <c r="Y214" s="2"/>
       <c r="Z214" s="2"/>
     </row>
-    <row r="215" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A215" s="2"/>
       <c r="B215" s="2"/>
       <c r="C215" s="2"/>
@@ -8109,7 +8106,7 @@
       <c r="Y215" s="2"/>
       <c r="Z215" s="2"/>
     </row>
-    <row r="216" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A216" s="2"/>
       <c r="B216" s="2"/>
       <c r="C216" s="2"/>
@@ -8137,7 +8134,7 @@
       <c r="Y216" s="2"/>
       <c r="Z216" s="2"/>
     </row>
-    <row r="217" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A217" s="2"/>
       <c r="B217" s="2"/>
       <c r="C217" s="2"/>
@@ -8165,7 +8162,7 @@
       <c r="Y217" s="2"/>
       <c r="Z217" s="2"/>
     </row>
-    <row r="218" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A218" s="2"/>
       <c r="B218" s="2"/>
       <c r="C218" s="2"/>
@@ -8193,7 +8190,7 @@
       <c r="Y218" s="2"/>
       <c r="Z218" s="2"/>
     </row>
-    <row r="219" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A219" s="2"/>
       <c r="B219" s="2"/>
       <c r="C219" s="2"/>
@@ -8221,7 +8218,7 @@
       <c r="Y219" s="2"/>
       <c r="Z219" s="2"/>
     </row>
-    <row r="220" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A220" s="2"/>
       <c r="B220" s="2"/>
       <c r="C220" s="2"/>
@@ -8249,7 +8246,7 @@
       <c r="Y220" s="2"/>
       <c r="Z220" s="2"/>
     </row>
-    <row r="221" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A221" s="2"/>
       <c r="B221" s="2"/>
       <c r="C221" s="2"/>
@@ -8277,7 +8274,7 @@
       <c r="Y221" s="2"/>
       <c r="Z221" s="2"/>
     </row>
-    <row r="222" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A222" s="2"/>
       <c r="B222" s="2"/>
       <c r="C222" s="2"/>
@@ -8305,7 +8302,7 @@
       <c r="Y222" s="2"/>
       <c r="Z222" s="2"/>
     </row>
-    <row r="223" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A223" s="2"/>
       <c r="B223" s="2"/>
       <c r="C223" s="2"/>
@@ -8333,7 +8330,7 @@
       <c r="Y223" s="2"/>
       <c r="Z223" s="2"/>
     </row>
-    <row r="224" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A224" s="2"/>
       <c r="B224" s="2"/>
       <c r="C224" s="2"/>
@@ -8361,7 +8358,7 @@
       <c r="Y224" s="2"/>
       <c r="Z224" s="2"/>
     </row>
-    <row r="225" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A225" s="2"/>
       <c r="B225" s="2"/>
       <c r="C225" s="2"/>
@@ -8389,7 +8386,7 @@
       <c r="Y225" s="2"/>
       <c r="Z225" s="2"/>
     </row>
-    <row r="226" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A226" s="2"/>
       <c r="B226" s="2"/>
       <c r="C226" s="2"/>
@@ -8417,7 +8414,7 @@
       <c r="Y226" s="2"/>
       <c r="Z226" s="2"/>
     </row>
-    <row r="227" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A227" s="2"/>
       <c r="B227" s="2"/>
       <c r="C227" s="2"/>
@@ -8445,7 +8442,7 @@
       <c r="Y227" s="2"/>
       <c r="Z227" s="2"/>
     </row>
-    <row r="228" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A228" s="2"/>
       <c r="B228" s="2"/>
       <c r="C228" s="2"/>
@@ -8473,778 +8470,778 @@
       <c r="Y228" s="2"/>
       <c r="Z228" s="2"/>
     </row>
-    <row r="229" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="230" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="231" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="232" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="233" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="234" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="235" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="236" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="237" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="238" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="239" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="240" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="229" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="230" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="231" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="232" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="233" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="234" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="235" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="236" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="237" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="238" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="239" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="240" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="37">
     <mergeCell ref="A19:C19"/>

</xml_diff>

<commit_message>
fix: actualizar plantilla CUENTA_COBRO.xlsx
</commit_message>
<xml_diff>
--- a/plantillas/CUENTA_COBRO.xlsx
+++ b/plantillas/CUENTA_COBRO.xlsx
@@ -445,71 +445,32 @@
     <xf numFmtId="167" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -531,17 +492,56 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -575,7 +575,7 @@
         <xdr:cNvPr id="3" name="Shape 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -630,7 +630,7 @@
         <xdr:cNvPr id="4" name="Shape 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -685,7 +685,7 @@
         <xdr:cNvPr id="2" name="Shape 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -740,7 +740,7 @@
         <xdr:cNvPr id="5" name="Shape 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000005000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -782,1017 +782,61 @@
     </xdr:sp>
     <xdr:clientData fLocksWithSheet="0"/>
   </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1790700" cy="419100"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="6" name="Shape 5">
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="27" name="26 Imagen"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
           <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
             </a:ext>
           </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="4455413" y="3575213"/>
-          <a:ext cx="1781175" cy="409575"/>
+          <a:off x="0" y="30480"/>
+          <a:ext cx="8023860" cy="1752600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="FFFFFF"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
       </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr spcFirstLastPara="1" wrap="square" lIns="27425" tIns="18275" rIns="27425" bIns="18275" anchor="ctr" anchorCtr="0">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" rtl="1">
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClr>
-              <a:srgbClr val="000000"/>
-            </a:buClr>
-            <a:buSzPts val="800"/>
-            <a:buFont typeface="Arial"/>
-            <a:buNone/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:ea typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-              <a:sym typeface="Arial"/>
-            </a:rPr>
-            <a:t>GESTIÓN DE HACIENDA PÚBLICA</a:t>
-          </a:r>
-          <a:endParaRPr sz="1400"/>
-        </a:p>
-        <a:p>
-          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" rtl="1">
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClr>
-              <a:srgbClr val="000000"/>
-            </a:buClr>
-            <a:buSzPts val="800"/>
-            <a:buFont typeface="Arial"/>
-            <a:buNone/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:ea typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-              <a:sym typeface="Arial"/>
-            </a:rPr>
-            <a:t>CONTABILIDAD GENERAL</a:t>
-          </a:r>
-          <a:endParaRPr sz="1400"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="8172450" cy="1724025"/>
-    <xdr:grpSp>
-      <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="7" name="Shape 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000007000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGrpSpPr/>
-      </xdr:nvGrpSpPr>
-      <xdr:grpSpPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="8172450" cy="1724025"/>
-          <a:chOff x="1469325" y="2884650"/>
-          <a:chExt cx="7753350" cy="1790700"/>
-        </a:xfrm>
-      </xdr:grpSpPr>
-      <xdr:grpSp>
-        <xdr:nvGrpSpPr>
-          <xdr:cNvPr id="8" name="Shape 6">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000008000000}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvGrpSpPr/>
-        </xdr:nvGrpSpPr>
-        <xdr:grpSpPr>
-          <a:xfrm>
-            <a:off x="1469325" y="2884650"/>
-            <a:ext cx="7753350" cy="1790700"/>
-            <a:chOff x="1445513" y="2908463"/>
-            <a:chExt cx="7800975" cy="1743075"/>
-          </a:xfrm>
-        </xdr:grpSpPr>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="9" name="Shape 7">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="1445513" y="2908463"/>
-              <a:ext cx="7800975" cy="1743075"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr spcFirstLastPara="1" wrap="square" lIns="91425" tIns="91425" rIns="91425" bIns="91425" anchor="ctr" anchorCtr="0">
-              <a:noAutofit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr marL="0" lvl="0" indent="0" algn="l" rtl="0">
-                <a:spcBef>
-                  <a:spcPts val="0"/>
-                </a:spcBef>
-                <a:spcAft>
-                  <a:spcPts val="0"/>
-                </a:spcAft>
-                <a:buNone/>
-              </a:pPr>
-              <a:endParaRPr sz="1400"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-        <xdr:grpSp>
-          <xdr:nvGrpSpPr>
-            <xdr:cNvPr id="10" name="Shape 8">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000A000000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGrpSpPr/>
-          </xdr:nvGrpSpPr>
-          <xdr:grpSpPr>
-            <a:xfrm>
-              <a:off x="1445513" y="2908463"/>
-              <a:ext cx="7800975" cy="1743075"/>
-              <a:chOff x="1445513" y="2908463"/>
-              <a:chExt cx="7800975" cy="1743075"/>
-            </a:xfrm>
-          </xdr:grpSpPr>
-          <xdr:sp macro="" textlink="">
-            <xdr:nvSpPr>
-              <xdr:cNvPr id="11" name="Shape 9">
-                <a:extLst>
-                  <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                    <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000B000000}"/>
-                  </a:ext>
-                </a:extLst>
-              </xdr:cNvPr>
-              <xdr:cNvSpPr/>
-            </xdr:nvSpPr>
-            <xdr:spPr>
-              <a:xfrm>
-                <a:off x="1445513" y="2908463"/>
-                <a:ext cx="7800975" cy="1743075"/>
-              </a:xfrm>
-              <a:prstGeom prst="rect">
-                <a:avLst/>
-              </a:prstGeom>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-            </xdr:spPr>
-            <xdr:txBody>
-              <a:bodyPr spcFirstLastPara="1" wrap="square" lIns="91425" tIns="91425" rIns="91425" bIns="91425" anchor="ctr" anchorCtr="0">
-                <a:noAutofit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr marL="0" lvl="0" indent="0" algn="l" rtl="0">
-                  <a:spcBef>
-                    <a:spcPts val="0"/>
-                  </a:spcBef>
-                  <a:spcAft>
-                    <a:spcPts val="0"/>
-                  </a:spcAft>
-                  <a:buSzPts val="1400"/>
-                  <a:buFont typeface="Arial"/>
-                  <a:buNone/>
-                </a:pPr>
-                <a:endParaRPr sz="1400"/>
-              </a:p>
-            </xdr:txBody>
-          </xdr:sp>
-          <xdr:grpSp>
-            <xdr:nvGrpSpPr>
-              <xdr:cNvPr id="12" name="Shape 10">
-                <a:extLst>
-                  <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                    <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000C000000}"/>
-                  </a:ext>
-                </a:extLst>
-              </xdr:cNvPr>
-              <xdr:cNvGrpSpPr/>
-            </xdr:nvGrpSpPr>
-            <xdr:grpSpPr>
-              <a:xfrm>
-                <a:off x="1445513" y="2908463"/>
-                <a:ext cx="7800975" cy="1743075"/>
-                <a:chOff x="1445513" y="2908463"/>
-                <a:chExt cx="7800975" cy="1743075"/>
-              </a:xfrm>
-            </xdr:grpSpPr>
-            <xdr:sp macro="" textlink="">
-              <xdr:nvSpPr>
-                <xdr:cNvPr id="13" name="Shape 11">
-                  <a:extLst>
-                    <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                      <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000D000000}"/>
-                    </a:ext>
-                  </a:extLst>
-                </xdr:cNvPr>
-                <xdr:cNvSpPr/>
-              </xdr:nvSpPr>
-              <xdr:spPr>
-                <a:xfrm>
-                  <a:off x="1445513" y="2908463"/>
-                  <a:ext cx="7800975" cy="1743075"/>
-                </a:xfrm>
-                <a:prstGeom prst="rect">
-                  <a:avLst/>
-                </a:prstGeom>
-                <a:noFill/>
-                <a:ln>
-                  <a:noFill/>
-                </a:ln>
-              </xdr:spPr>
-              <xdr:txBody>
-                <a:bodyPr spcFirstLastPara="1" wrap="square" lIns="91425" tIns="91425" rIns="91425" bIns="91425" anchor="ctr" anchorCtr="0">
-                  <a:noAutofit/>
-                </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
-                  <a:pPr marL="0" lvl="0" indent="0" algn="l" rtl="0">
-                    <a:spcBef>
-                      <a:spcPts val="0"/>
-                    </a:spcBef>
-                    <a:spcAft>
-                      <a:spcPts val="0"/>
-                    </a:spcAft>
-                    <a:buSzPts val="1400"/>
-                    <a:buFont typeface="Arial"/>
-                    <a:buNone/>
-                  </a:pPr>
-                  <a:endParaRPr sz="1400"/>
-                </a:p>
-              </xdr:txBody>
-            </xdr:sp>
-            <xdr:grpSp>
-              <xdr:nvGrpSpPr>
-                <xdr:cNvPr id="14" name="Shape 12">
-                  <a:extLst>
-                    <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                      <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000E000000}"/>
-                    </a:ext>
-                  </a:extLst>
-                </xdr:cNvPr>
-                <xdr:cNvGrpSpPr/>
-              </xdr:nvGrpSpPr>
-              <xdr:grpSpPr>
-                <a:xfrm>
-                  <a:off x="1445513" y="2908463"/>
-                  <a:ext cx="7800975" cy="1743075"/>
-                  <a:chOff x="1445513" y="2908463"/>
-                  <a:chExt cx="7800975" cy="1743075"/>
-                </a:xfrm>
-              </xdr:grpSpPr>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="15" name="Shape 13">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000F000000}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="1445513" y="2908463"/>
-                    <a:ext cx="7800975" cy="1743075"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                </xdr:spPr>
-                <xdr:txBody>
-                  <a:bodyPr spcFirstLastPara="1" wrap="square" lIns="91425" tIns="91425" rIns="91425" bIns="91425" anchor="ctr" anchorCtr="0">
-                    <a:noAutofit/>
-                  </a:bodyPr>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr marL="0" lvl="0" indent="0" algn="l" rtl="0">
-                      <a:spcBef>
-                        <a:spcPts val="0"/>
-                      </a:spcBef>
-                      <a:spcAft>
-                        <a:spcPts val="0"/>
-                      </a:spcAft>
-                      <a:buSzPts val="1400"/>
-                      <a:buFont typeface="Arial"/>
-                      <a:buNone/>
-                    </a:pPr>
-                    <a:endParaRPr sz="1400"/>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:grpSp>
-                <xdr:nvGrpSpPr>
-                  <xdr:cNvPr id="16" name="Shape 14">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000010000000}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvGrpSpPr/>
-                </xdr:nvGrpSpPr>
-                <xdr:grpSpPr>
-                  <a:xfrm>
-                    <a:off x="1445513" y="2908463"/>
-                    <a:ext cx="7800975" cy="1743075"/>
-                    <a:chOff x="1445513" y="2908463"/>
-                    <a:chExt cx="7800975" cy="1743075"/>
-                  </a:xfrm>
-                </xdr:grpSpPr>
-                <xdr:sp macro="" textlink="">
-                  <xdr:nvSpPr>
-                    <xdr:cNvPr id="17" name="Shape 15">
-                      <a:extLst>
-                        <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                          <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000011000000}"/>
-                        </a:ext>
-                      </a:extLst>
-                    </xdr:cNvPr>
-                    <xdr:cNvSpPr/>
-                  </xdr:nvSpPr>
-                  <xdr:spPr>
-                    <a:xfrm>
-                      <a:off x="1445513" y="2908463"/>
-                      <a:ext cx="7800975" cy="1743075"/>
-                    </a:xfrm>
-                    <a:prstGeom prst="rect">
-                      <a:avLst/>
-                    </a:prstGeom>
-                    <a:noFill/>
-                    <a:ln>
-                      <a:noFill/>
-                    </a:ln>
-                  </xdr:spPr>
-                  <xdr:txBody>
-                    <a:bodyPr spcFirstLastPara="1" wrap="square" lIns="91425" tIns="91425" rIns="91425" bIns="91425" anchor="ctr" anchorCtr="0">
-                      <a:noAutofit/>
-                    </a:bodyPr>
-                    <a:lstStyle/>
-                    <a:p>
-                      <a:pPr marL="0" lvl="0" indent="0" algn="l" rtl="0">
-                        <a:spcBef>
-                          <a:spcPts val="0"/>
-                        </a:spcBef>
-                        <a:spcAft>
-                          <a:spcPts val="0"/>
-                        </a:spcAft>
-                        <a:buSzPts val="1400"/>
-                        <a:buFont typeface="Arial"/>
-                        <a:buNone/>
-                      </a:pPr>
-                      <a:endParaRPr sz="1400"/>
-                    </a:p>
-                  </xdr:txBody>
-                </xdr:sp>
-                <xdr:grpSp>
-                  <xdr:nvGrpSpPr>
-                    <xdr:cNvPr id="18" name="Shape 16">
-                      <a:extLst>
-                        <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                          <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000012000000}"/>
-                        </a:ext>
-                      </a:extLst>
-                    </xdr:cNvPr>
-                    <xdr:cNvGrpSpPr/>
-                  </xdr:nvGrpSpPr>
-                  <xdr:grpSpPr>
-                    <a:xfrm>
-                      <a:off x="1445513" y="2908463"/>
-                      <a:ext cx="7800975" cy="1743075"/>
-                      <a:chOff x="0" y="0"/>
-                      <a:chExt cx="13148642" cy="1152525"/>
-                    </a:xfrm>
-                  </xdr:grpSpPr>
-                  <xdr:sp macro="" textlink="">
-                    <xdr:nvSpPr>
-                      <xdr:cNvPr id="19" name="Shape 17">
-                        <a:extLst>
-                          <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                            <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000013000000}"/>
-                          </a:ext>
-                        </a:extLst>
-                      </xdr:cNvPr>
-                      <xdr:cNvSpPr/>
-                    </xdr:nvSpPr>
-                    <xdr:spPr>
-                      <a:xfrm>
-                        <a:off x="0" y="0"/>
-                        <a:ext cx="13148625" cy="1152525"/>
-                      </a:xfrm>
-                      <a:prstGeom prst="rect">
-                        <a:avLst/>
-                      </a:prstGeom>
-                      <a:noFill/>
-                      <a:ln>
-                        <a:noFill/>
-                      </a:ln>
-                    </xdr:spPr>
-                    <xdr:txBody>
-                      <a:bodyPr spcFirstLastPara="1" wrap="square" lIns="91425" tIns="91425" rIns="91425" bIns="91425" anchor="ctr" anchorCtr="0">
-                        <a:noAutofit/>
-                      </a:bodyPr>
-                      <a:lstStyle/>
-                      <a:p>
-                        <a:pPr marL="0" lvl="0" indent="0" algn="l" rtl="0">
-                          <a:spcBef>
-                            <a:spcPts val="0"/>
-                          </a:spcBef>
-                          <a:spcAft>
-                            <a:spcPts val="0"/>
-                          </a:spcAft>
-                          <a:buSzPts val="1400"/>
-                          <a:buFont typeface="Arial"/>
-                          <a:buNone/>
-                        </a:pPr>
-                        <a:endParaRPr sz="1400"/>
-                      </a:p>
-                    </xdr:txBody>
-                  </xdr:sp>
-                  <xdr:grpSp>
-                    <xdr:nvGrpSpPr>
-                      <xdr:cNvPr id="20" name="Shape 18">
-                        <a:extLst>
-                          <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                            <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000014000000}"/>
-                          </a:ext>
-                        </a:extLst>
-                      </xdr:cNvPr>
-                      <xdr:cNvGrpSpPr/>
-                    </xdr:nvGrpSpPr>
-                    <xdr:grpSpPr>
-                      <a:xfrm>
-                        <a:off x="0" y="0"/>
-                        <a:ext cx="13148642" cy="1152525"/>
-                        <a:chOff x="0" y="0"/>
-                        <a:chExt cx="762" cy="102"/>
-                      </a:xfrm>
-                    </xdr:grpSpPr>
-                    <xdr:sp macro="" textlink="">
-                      <xdr:nvSpPr>
-                        <xdr:cNvPr id="21" name="Shape 19">
-                          <a:extLst>
-                            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000015000000}"/>
-                            </a:ext>
-                          </a:extLst>
-                        </xdr:cNvPr>
-                        <xdr:cNvSpPr/>
-                      </xdr:nvSpPr>
-                      <xdr:spPr>
-                        <a:xfrm>
-                          <a:off x="0" y="0"/>
-                          <a:ext cx="759" cy="102"/>
-                        </a:xfrm>
-                        <a:prstGeom prst="rect">
-                          <a:avLst/>
-                        </a:prstGeom>
-                        <a:noFill/>
-                        <a:ln w="9525" cap="flat" cmpd="sng">
-                          <a:solidFill>
-                            <a:srgbClr val="000000"/>
-                          </a:solidFill>
-                          <a:prstDash val="solid"/>
-                          <a:miter lim="800000"/>
-                          <a:headEnd type="none" w="sm" len="sm"/>
-                          <a:tailEnd type="none" w="sm" len="sm"/>
-                        </a:ln>
-                      </xdr:spPr>
-                      <xdr:txBody>
-                        <a:bodyPr spcFirstLastPara="1" wrap="square" lIns="91425" tIns="91425" rIns="91425" bIns="91425" anchor="ctr" anchorCtr="0">
-                          <a:noAutofit/>
-                        </a:bodyPr>
-                        <a:lstStyle/>
-                        <a:p>
-                          <a:pPr marL="0" lvl="0" indent="0" algn="l" rtl="0">
-                            <a:spcBef>
-                              <a:spcPts val="0"/>
-                            </a:spcBef>
-                            <a:spcAft>
-                              <a:spcPts val="0"/>
-                            </a:spcAft>
-                            <a:buSzPts val="1400"/>
-                            <a:buFont typeface="Arial"/>
-                            <a:buNone/>
-                          </a:pPr>
-                          <a:endParaRPr sz="1400"/>
-                        </a:p>
-                      </xdr:txBody>
-                    </xdr:sp>
-                    <xdr:sp macro="" textlink="">
-                      <xdr:nvSpPr>
-                        <xdr:cNvPr id="22" name="Shape 20">
-                          <a:extLst>
-                            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000016000000}"/>
-                            </a:ext>
-                          </a:extLst>
-                        </xdr:cNvPr>
-                        <xdr:cNvSpPr txBox="1"/>
-                      </xdr:nvSpPr>
-                      <xdr:spPr>
-                        <a:xfrm>
-                          <a:off x="557" y="0"/>
-                          <a:ext cx="205" cy="47"/>
-                        </a:xfrm>
-                        <a:prstGeom prst="rect">
-                          <a:avLst/>
-                        </a:prstGeom>
-                        <a:solidFill>
-                          <a:srgbClr val="FFFFFF"/>
-                        </a:solidFill>
-                        <a:ln w="9525" cap="flat" cmpd="sng">
-                          <a:solidFill>
-                            <a:srgbClr val="000000"/>
-                          </a:solidFill>
-                          <a:prstDash val="solid"/>
-                          <a:miter lim="800000"/>
-                          <a:headEnd type="none" w="sm" len="sm"/>
-                          <a:tailEnd type="none" w="sm" len="sm"/>
-                        </a:ln>
-                      </xdr:spPr>
-                      <xdr:txBody>
-                        <a:bodyPr spcFirstLastPara="1" wrap="square" lIns="27425" tIns="22850" rIns="27425" bIns="0" anchor="ctr" anchorCtr="0">
-                          <a:noAutofit/>
-                        </a:bodyPr>
-                        <a:lstStyle/>
-                        <a:p>
-                          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" rtl="1">
-                            <a:spcBef>
-                              <a:spcPts val="0"/>
-                            </a:spcBef>
-                            <a:spcAft>
-                              <a:spcPts val="0"/>
-                            </a:spcAft>
-                            <a:buClr>
-                              <a:srgbClr val="000000"/>
-                            </a:buClr>
-                            <a:buSzPts val="1000"/>
-                            <a:buFont typeface="Arial"/>
-                            <a:buNone/>
-                          </a:pPr>
-                          <a:r>
-                            <a:rPr lang="en-US" sz="1000" b="0" i="0">
-                              <a:solidFill>
-                                <a:srgbClr val="000000"/>
-                              </a:solidFill>
-                              <a:latin typeface="Arial"/>
-                              <a:ea typeface="Arial"/>
-                              <a:cs typeface="Arial"/>
-                              <a:sym typeface="Arial"/>
-                            </a:rPr>
-                            <a:t>MAHP03.03.01.P011.F001</a:t>
-                          </a:r>
-                          <a:endParaRPr sz="1000">
-                            <a:solidFill>
-                              <a:srgbClr val="000000"/>
-                            </a:solidFill>
-                            <a:latin typeface="Arial"/>
-                            <a:ea typeface="Arial"/>
-                            <a:cs typeface="Arial"/>
-                            <a:sym typeface="Arial"/>
-                          </a:endParaRPr>
-                        </a:p>
-                      </xdr:txBody>
-                    </xdr:sp>
-                    <xdr:sp macro="" textlink="">
-                      <xdr:nvSpPr>
-                        <xdr:cNvPr id="23" name="Shape 21">
-                          <a:extLst>
-                            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000017000000}"/>
-                            </a:ext>
-                          </a:extLst>
-                        </xdr:cNvPr>
-                        <xdr:cNvSpPr/>
-                      </xdr:nvSpPr>
-                      <xdr:spPr>
-                        <a:xfrm>
-                          <a:off x="664" y="47"/>
-                          <a:ext cx="98" cy="55"/>
-                        </a:xfrm>
-                        <a:prstGeom prst="rect">
-                          <a:avLst/>
-                        </a:prstGeom>
-                        <a:solidFill>
-                          <a:srgbClr val="FFFFFF"/>
-                        </a:solidFill>
-                        <a:ln w="9525" cap="flat" cmpd="sng">
-                          <a:solidFill>
-                            <a:srgbClr val="000000"/>
-                          </a:solidFill>
-                          <a:prstDash val="solid"/>
-                          <a:miter lim="800000"/>
-                          <a:headEnd type="none" w="sm" len="sm"/>
-                          <a:tailEnd type="none" w="sm" len="sm"/>
-                        </a:ln>
-                      </xdr:spPr>
-                      <xdr:txBody>
-                        <a:bodyPr spcFirstLastPara="1" wrap="square" lIns="27425" tIns="22850" rIns="27425" bIns="0" anchor="ctr" anchorCtr="0">
-                          <a:noAutofit/>
-                        </a:bodyPr>
-                        <a:lstStyle/>
-                        <a:p>
-                          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" rtl="0">
-                            <a:spcBef>
-                              <a:spcPts val="0"/>
-                            </a:spcBef>
-                            <a:spcAft>
-                              <a:spcPts val="0"/>
-                            </a:spcAft>
-                            <a:buClr>
-                              <a:srgbClr val="000000"/>
-                            </a:buClr>
-                            <a:buSzPts val="800"/>
-                            <a:buFont typeface="Arial"/>
-                            <a:buNone/>
-                          </a:pPr>
-                          <a:r>
-                            <a:rPr lang="en-US" sz="800" b="0" i="0" strike="noStrike">
-                              <a:solidFill>
-                                <a:srgbClr val="000000"/>
-                              </a:solidFill>
-                              <a:latin typeface="Arial"/>
-                              <a:ea typeface="Arial"/>
-                              <a:cs typeface="Arial"/>
-                              <a:sym typeface="Arial"/>
-                            </a:rPr>
-                            <a:t>004</a:t>
-                          </a:r>
-                          <a:endParaRPr sz="1400"/>
-                        </a:p>
-                      </xdr:txBody>
-                    </xdr:sp>
-                    <xdr:sp macro="" textlink="">
-                      <xdr:nvSpPr>
-                        <xdr:cNvPr id="24" name="Shape 22">
-                          <a:extLst>
-                            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000018000000}"/>
-                            </a:ext>
-                          </a:extLst>
-                        </xdr:cNvPr>
-                        <xdr:cNvSpPr/>
-                      </xdr:nvSpPr>
-                      <xdr:spPr>
-                        <a:xfrm>
-                          <a:off x="556" y="47"/>
-                          <a:ext cx="109" cy="55"/>
-                        </a:xfrm>
-                        <a:prstGeom prst="rect">
-                          <a:avLst/>
-                        </a:prstGeom>
-                        <a:solidFill>
-                          <a:srgbClr val="FFFFFF"/>
-                        </a:solidFill>
-                        <a:ln w="9525" cap="flat" cmpd="sng">
-                          <a:solidFill>
-                            <a:srgbClr val="000000"/>
-                          </a:solidFill>
-                          <a:prstDash val="solid"/>
-                          <a:miter lim="800000"/>
-                          <a:headEnd type="none" w="sm" len="sm"/>
-                          <a:tailEnd type="none" w="sm" len="sm"/>
-                        </a:ln>
-                      </xdr:spPr>
-                      <xdr:txBody>
-                        <a:bodyPr spcFirstLastPara="1" wrap="square" lIns="27425" tIns="22850" rIns="27425" bIns="0" anchor="ctr" anchorCtr="0">
-                          <a:noAutofit/>
-                        </a:bodyPr>
-                        <a:lstStyle/>
-                        <a:p>
-                          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" rtl="0">
-                            <a:spcBef>
-                              <a:spcPts val="0"/>
-                            </a:spcBef>
-                            <a:spcAft>
-                              <a:spcPts val="0"/>
-                            </a:spcAft>
-                            <a:buClr>
-                              <a:srgbClr val="000000"/>
-                            </a:buClr>
-                            <a:buSzPts val="800"/>
-                            <a:buFont typeface="Arial"/>
-                            <a:buNone/>
-                          </a:pPr>
-                          <a:r>
-                            <a:rPr lang="en-US" sz="800" b="0" i="0" strike="noStrike">
-                              <a:solidFill>
-                                <a:srgbClr val="000000"/>
-                              </a:solidFill>
-                              <a:latin typeface="Arial"/>
-                              <a:ea typeface="Arial"/>
-                              <a:cs typeface="Arial"/>
-                              <a:sym typeface="Arial"/>
-                            </a:rPr>
-                            <a:t>VERSIÓN</a:t>
-                          </a:r>
-                          <a:endParaRPr sz="1400"/>
-                        </a:p>
-                      </xdr:txBody>
-                    </xdr:sp>
-                    <xdr:sp macro="" textlink="">
-                      <xdr:nvSpPr>
-                        <xdr:cNvPr id="25" name="Shape 23">
-                          <a:extLst>
-                            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000019000000}"/>
-                            </a:ext>
-                          </a:extLst>
-                        </xdr:cNvPr>
-                        <xdr:cNvSpPr txBox="1"/>
-                      </xdr:nvSpPr>
-                      <xdr:spPr>
-                        <a:xfrm>
-                          <a:off x="177" y="0"/>
-                          <a:ext cx="380" cy="102"/>
-                        </a:xfrm>
-                        <a:prstGeom prst="rect">
-                          <a:avLst/>
-                        </a:prstGeom>
-                        <a:solidFill>
-                          <a:srgbClr val="FFFFFF"/>
-                        </a:solidFill>
-                        <a:ln w="9525" cap="flat" cmpd="sng">
-                          <a:solidFill>
-                            <a:srgbClr val="000000"/>
-                          </a:solidFill>
-                          <a:prstDash val="solid"/>
-                          <a:miter lim="800000"/>
-                          <a:headEnd type="none" w="sm" len="sm"/>
-                          <a:tailEnd type="none" w="sm" len="sm"/>
-                        </a:ln>
-                      </xdr:spPr>
-                      <xdr:txBody>
-                        <a:bodyPr spcFirstLastPara="1" wrap="square" lIns="27425" tIns="22850" rIns="27425" bIns="22850" anchor="ctr" anchorCtr="0">
-                          <a:noAutofit/>
-                        </a:bodyPr>
-                        <a:lstStyle/>
-                        <a:p>
-                          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" rtl="1">
-                            <a:lnSpc>
-                              <a:spcPct val="110000"/>
-                            </a:lnSpc>
-                            <a:spcBef>
-                              <a:spcPts val="0"/>
-                            </a:spcBef>
-                            <a:spcAft>
-                              <a:spcPts val="0"/>
-                            </a:spcAft>
-                            <a:buSzPts val="1000"/>
-                            <a:buFont typeface="Arial"/>
-                            <a:buNone/>
-                          </a:pPr>
-                          <a:r>
-                            <a:rPr lang="en-US" sz="1000" b="0" i="0">
-                              <a:latin typeface="Arial" pitchFamily="34" charset="0"/>
-                              <a:ea typeface="Arial"/>
-                              <a:cs typeface="Arial" pitchFamily="34" charset="0"/>
-                              <a:sym typeface="Arial"/>
-                            </a:rPr>
-                            <a:t>MODELO INTEGRADO DE PLANEACIÓN Y GESTIÓN</a:t>
-                          </a:r>
-                          <a:endParaRPr sz="1400">
-                            <a:latin typeface="Arial" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Arial" pitchFamily="34" charset="0"/>
-                          </a:endParaRPr>
-                        </a:p>
-                        <a:p>
-                          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" rtl="1">
-                            <a:lnSpc>
-                              <a:spcPct val="110000"/>
-                            </a:lnSpc>
-                            <a:spcBef>
-                              <a:spcPts val="0"/>
-                            </a:spcBef>
-                            <a:spcAft>
-                              <a:spcPts val="0"/>
-                            </a:spcAft>
-                            <a:buSzPts val="1000"/>
-                            <a:buFont typeface="Arial"/>
-                            <a:buNone/>
-                          </a:pPr>
-                          <a:r>
-                            <a:rPr lang="es-MX" sz="1000">
-                              <a:latin typeface="Arial" pitchFamily="34" charset="0"/>
-                              <a:ea typeface="Arial"/>
-                              <a:cs typeface="Arial" pitchFamily="34" charset="0"/>
-                              <a:sym typeface="Arial"/>
-                            </a:rPr>
-                            <a:t> (MIPG)</a:t>
-                          </a:r>
-                          <a:endParaRPr sz="1000">
-                            <a:latin typeface="Arial" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Arial"/>
-                            <a:cs typeface="Arial" pitchFamily="34" charset="0"/>
-                            <a:sym typeface="Arial"/>
-                          </a:endParaRPr>
-                        </a:p>
-                        <a:p>
-                          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" rtl="1">
-                            <a:spcBef>
-                              <a:spcPts val="0"/>
-                            </a:spcBef>
-                            <a:spcAft>
-                              <a:spcPts val="0"/>
-                            </a:spcAft>
-                            <a:buSzPts val="1200"/>
-                            <a:buFont typeface="Arial"/>
-                            <a:buNone/>
-                          </a:pPr>
-                          <a:endParaRPr sz="1200" b="0" i="0" strike="noStrike">
-                            <a:solidFill>
-                              <a:srgbClr val="000000"/>
-                            </a:solidFill>
-                            <a:latin typeface="Arial"/>
-                            <a:ea typeface="Arial"/>
-                            <a:cs typeface="Arial"/>
-                            <a:sym typeface="Arial"/>
-                          </a:endParaRPr>
-                        </a:p>
-                        <a:p>
-                          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" rtl="0">
-                            <a:spcBef>
-                              <a:spcPts val="0"/>
-                            </a:spcBef>
-                            <a:spcAft>
-                              <a:spcPts val="0"/>
-                            </a:spcAft>
-                            <a:buSzPts val="1200"/>
-                            <a:buFont typeface="Arial"/>
-                            <a:buNone/>
-                          </a:pPr>
-                          <a:r>
-                            <a:rPr lang="en-US" sz="1200" b="1">
-                              <a:latin typeface="Arial"/>
-                              <a:ea typeface="Arial"/>
-                              <a:cs typeface="Arial"/>
-                              <a:sym typeface="Arial"/>
-                            </a:rPr>
-                            <a:t>DOCUMENTO SOPORTE</a:t>
-                          </a:r>
-                          <a:endParaRPr sz="1200">
-                            <a:latin typeface="Arial"/>
-                            <a:ea typeface="Arial"/>
-                            <a:cs typeface="Arial"/>
-                            <a:sym typeface="Arial"/>
-                          </a:endParaRPr>
-                        </a:p>
-                        <a:p>
-                          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" rtl="0">
-                            <a:spcBef>
-                              <a:spcPts val="0"/>
-                            </a:spcBef>
-                            <a:spcAft>
-                              <a:spcPts val="0"/>
-                            </a:spcAft>
-                            <a:buSzPts val="1200"/>
-                            <a:buFont typeface="Arial"/>
-                            <a:buNone/>
-                          </a:pPr>
-                          <a:r>
-                            <a:rPr lang="en-US" sz="1200" b="1">
-                              <a:latin typeface="Arial"/>
-                              <a:ea typeface="Arial"/>
-                              <a:cs typeface="Arial"/>
-                              <a:sym typeface="Arial"/>
-                            </a:rPr>
-                            <a:t>EN ADQUISICIONES EFECTUADAS A SUJETOS NO OBLIGADOS A EXPEDIR FACTURA DE VENTA O DOCUMENTO EQUIVALENTE</a:t>
-                          </a:r>
-                          <a:endParaRPr sz="1200">
-                            <a:latin typeface="Arial"/>
-                            <a:ea typeface="Arial"/>
-                            <a:cs typeface="Arial"/>
-                            <a:sym typeface="Arial"/>
-                          </a:endParaRPr>
-                        </a:p>
-                      </xdr:txBody>
-                    </xdr:sp>
-                  </xdr:grpSp>
-                  <xdr:pic>
-                    <xdr:nvPicPr>
-                      <xdr:cNvPr id="26" name="Shape 24" descr="escudo">
-                        <a:extLst>
-                          <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                            <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001A000000}"/>
-                          </a:ext>
-                        </a:extLst>
-                      </xdr:cNvPr>
-                      <xdr:cNvPicPr preferRelativeResize="0"/>
-                    </xdr:nvPicPr>
-                    <xdr:blipFill rotWithShape="1">
-                      <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-                        <a:alphaModFix/>
-                      </a:blip>
-                      <a:srcRect/>
-                      <a:stretch/>
-                    </xdr:blipFill>
-                    <xdr:spPr>
-                      <a:xfrm>
-                        <a:off x="448978" y="75414"/>
-                        <a:ext cx="2196786" cy="776651"/>
-                      </a:xfrm>
-                      <a:prstGeom prst="rect">
-                        <a:avLst/>
-                      </a:prstGeom>
-                      <a:noFill/>
-                      <a:ln>
-                        <a:noFill/>
-                      </a:ln>
-                    </xdr:spPr>
-                  </xdr:pic>
-                </xdr:grpSp>
-              </xdr:grpSp>
-            </xdr:grpSp>
-          </xdr:grpSp>
-        </xdr:grpSp>
-      </xdr:grpSp>
-    </xdr:grpSp>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2011,15 +1055,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="22"/>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
+      <c r="A1" s="57"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="58"/>
+      <c r="I1" s="58"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
@@ -2039,15 +1083,15 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="23"/>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
+      <c r="A2" s="58"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
@@ -2067,15 +1111,15 @@
       <c r="Z2" s="1"/>
     </row>
     <row r="3" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="23"/>
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="23"/>
-      <c r="G3" s="23"/>
-      <c r="H3" s="23"/>
-      <c r="I3" s="23"/>
+      <c r="A3" s="58"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="58"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
@@ -2095,15 +1139,15 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="23"/>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
+      <c r="A4" s="58"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="58"/>
+      <c r="H4" s="58"/>
+      <c r="I4" s="58"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
@@ -2123,15 +1167,15 @@
       <c r="Z4" s="1"/>
     </row>
     <row r="5" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="23"/>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23"/>
-      <c r="H5" s="23"/>
-      <c r="I5" s="23"/>
+      <c r="A5" s="58"/>
+      <c r="B5" s="58"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="58"/>
+      <c r="E5" s="58"/>
+      <c r="F5" s="58"/>
+      <c r="G5" s="58"/>
+      <c r="H5" s="58"/>
+      <c r="I5" s="58"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
@@ -2151,15 +1195,15 @@
       <c r="Z5" s="1"/>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="23"/>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="23"/>
-      <c r="I6" s="23"/>
+      <c r="A6" s="58"/>
+      <c r="B6" s="58"/>
+      <c r="C6" s="58"/>
+      <c r="D6" s="58"/>
+      <c r="E6" s="58"/>
+      <c r="F6" s="58"/>
+      <c r="G6" s="58"/>
+      <c r="H6" s="58"/>
+      <c r="I6" s="58"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
@@ -2179,15 +1223,15 @@
       <c r="Z6" s="1"/>
     </row>
     <row r="7" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="23"/>
-      <c r="B7" s="23"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="23"/>
-      <c r="G7" s="23"/>
-      <c r="H7" s="23"/>
-      <c r="I7" s="23"/>
+      <c r="A7" s="58"/>
+      <c r="B7" s="58"/>
+      <c r="C7" s="58"/>
+      <c r="D7" s="58"/>
+      <c r="E7" s="58"/>
+      <c r="F7" s="58"/>
+      <c r="G7" s="58"/>
+      <c r="H7" s="58"/>
+      <c r="I7" s="58"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
@@ -2207,15 +1251,15 @@
       <c r="Z7" s="1"/>
     </row>
     <row r="8" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="23"/>
-      <c r="B8" s="23"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="23"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="23"/>
-      <c r="G8" s="23"/>
-      <c r="H8" s="23"/>
-      <c r="I8" s="23"/>
+      <c r="A8" s="58"/>
+      <c r="B8" s="58"/>
+      <c r="C8" s="58"/>
+      <c r="D8" s="58"/>
+      <c r="E8" s="58"/>
+      <c r="F8" s="58"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="58"/>
+      <c r="I8" s="58"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
@@ -2235,15 +1279,15 @@
       <c r="Z8" s="1"/>
     </row>
     <row r="9" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="23"/>
-      <c r="B9" s="23"/>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="23"/>
+      <c r="A9" s="58"/>
+      <c r="B9" s="58"/>
+      <c r="C9" s="58"/>
+      <c r="D9" s="58"/>
+      <c r="E9" s="58"/>
+      <c r="F9" s="58"/>
+      <c r="G9" s="58"/>
+      <c r="H9" s="58"/>
+      <c r="I9" s="58"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
@@ -2263,15 +1307,15 @@
       <c r="Z9" s="1"/>
     </row>
     <row r="10" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="23"/>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
+      <c r="A10" s="58"/>
+      <c r="B10" s="58"/>
+      <c r="C10" s="58"/>
+      <c r="D10" s="58"/>
+      <c r="E10" s="58"/>
+      <c r="F10" s="58"/>
+      <c r="G10" s="58"/>
+      <c r="H10" s="58"/>
+      <c r="I10" s="58"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
@@ -2291,17 +1335,17 @@
       <c r="Z10" s="1"/>
     </row>
     <row r="11" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="24" t="s">
+      <c r="A11" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="25"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="21"/>
+      <c r="B11" s="19"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="20"/>
       <c r="J11" s="5">
         <v>1</v>
       </c>
@@ -2323,13 +1367,13 @@
       <c r="Z11" s="2"/>
     </row>
     <row r="12" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="26" t="s">
+      <c r="A12" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="25"/>
-      <c r="C12" s="21"/>
-      <c r="D12" s="27"/>
-      <c r="E12" s="21"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="59"/>
+      <c r="E12" s="20"/>
       <c r="F12" s="11" t="s">
         <v>2</v>
       </c>
@@ -2359,16 +1403,16 @@
       <c r="Z12" s="2"/>
     </row>
     <row r="13" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="26" t="s">
+      <c r="A13" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="B13" s="25"/>
-      <c r="C13" s="21"/>
-      <c r="D13" s="28" t="s">
+      <c r="B13" s="19"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="E13" s="29"/>
-      <c r="F13" s="29"/>
+      <c r="E13" s="54"/>
+      <c r="F13" s="54"/>
       <c r="G13" s="12" t="s">
         <v>6</v>
       </c>
@@ -2397,23 +1441,23 @@
       <c r="Z13" s="2"/>
     </row>
     <row r="14" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="26" t="s">
+      <c r="A14" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="25"/>
-      <c r="C14" s="21"/>
-      <c r="D14" s="18" t="s">
+      <c r="B14" s="19"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="E14" s="56"/>
+      <c r="F14" s="56"/>
       <c r="G14" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="H14" s="20">
+      <c r="H14" s="51">
         <v>4121</v>
       </c>
-      <c r="I14" s="21"/>
+      <c r="I14" s="20"/>
       <c r="J14" s="3"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
@@ -2433,23 +1477,23 @@
       <c r="Z14" s="2"/>
     </row>
     <row r="15" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="26" t="s">
+      <c r="A15" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="25"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="33" t="s">
+      <c r="B15" s="19"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="34"/>
-      <c r="F15" s="34"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
       <c r="G15" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="20">
+      <c r="H15" s="51">
         <v>8896744</v>
       </c>
-      <c r="I15" s="21"/>
+      <c r="I15" s="20"/>
       <c r="J15" s="3"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
@@ -2469,17 +1513,17 @@
       <c r="Z15" s="2"/>
     </row>
     <row r="16" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="24" t="s">
+      <c r="A16" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="25"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
-      <c r="I16" s="21"/>
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="20"/>
       <c r="J16" s="5">
         <v>2</v>
       </c>
@@ -2501,14 +1545,14 @@
       <c r="Z16" s="2"/>
     </row>
     <row r="17" spans="1:26" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="26" t="s">
+      <c r="A17" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="25"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="29"/>
-      <c r="F17" s="29"/>
+      <c r="B17" s="19"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="53"/>
+      <c r="E17" s="54"/>
+      <c r="F17" s="54"/>
       <c r="G17" s="14" t="s">
         <v>15</v>
       </c>
@@ -2533,19 +1577,19 @@
       <c r="Z17" s="2"/>
     </row>
     <row r="18" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="26" t="s">
+      <c r="A18" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="25"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="31"/>
-      <c r="F18" s="31"/>
+      <c r="B18" s="19"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="47"/>
+      <c r="E18" s="48"/>
+      <c r="F18" s="48"/>
       <c r="G18" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="H18" s="32"/>
-      <c r="I18" s="21"/>
+      <c r="H18" s="49"/>
+      <c r="I18" s="20"/>
       <c r="J18" s="3"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
@@ -2565,19 +1609,19 @@
       <c r="Z18" s="2"/>
     </row>
     <row r="19" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="26" t="s">
+      <c r="A19" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="25"/>
-      <c r="C19" s="21"/>
-      <c r="D19" s="56"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="34"/>
+      <c r="B19" s="19"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
       <c r="G19" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="H19" s="57"/>
-      <c r="I19" s="21"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="20"/>
       <c r="J19" s="3"/>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
@@ -2597,17 +1641,17 @@
       <c r="Z19" s="2"/>
     </row>
     <row r="20" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="47" t="s">
+      <c r="A20" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="21"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="20"/>
       <c r="J20" s="5">
         <v>3</v>
       </c>
@@ -2629,17 +1673,17 @@
       <c r="Z20" s="2"/>
     </row>
     <row r="21" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="58" t="s">
+      <c r="A21" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="42"/>
-      <c r="C21" s="43"/>
-      <c r="D21" s="59"/>
-      <c r="E21" s="42"/>
-      <c r="F21" s="42"/>
-      <c r="G21" s="42"/>
-      <c r="H21" s="42"/>
-      <c r="I21" s="43"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="26"/>
+      <c r="I21" s="27"/>
       <c r="J21" s="5"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
@@ -2659,15 +1703,15 @@
       <c r="Z21" s="2"/>
     </row>
     <row r="22" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="44"/>
-      <c r="B22" s="38"/>
-      <c r="C22" s="39"/>
-      <c r="D22" s="44"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="38"/>
-      <c r="G22" s="38"/>
-      <c r="H22" s="38"/>
-      <c r="I22" s="39"/>
+      <c r="A22" s="28"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="29"/>
+      <c r="I22" s="30"/>
       <c r="J22" s="5"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
@@ -2687,17 +1731,17 @@
       <c r="Z22" s="2"/>
     </row>
     <row r="23" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="40" t="s">
+      <c r="A23" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="25"/>
-      <c r="C23" s="21"/>
-      <c r="D23" s="35"/>
-      <c r="E23" s="36"/>
-      <c r="F23" s="37"/>
-      <c r="G23" s="38"/>
-      <c r="H23" s="38"/>
-      <c r="I23" s="39"/>
+      <c r="B23" s="19"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="39"/>
+      <c r="E23" s="40"/>
+      <c r="F23" s="41"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="29"/>
+      <c r="I23" s="30"/>
       <c r="J23" s="5"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
@@ -2717,17 +1761,17 @@
       <c r="Z23" s="2"/>
     </row>
     <row r="24" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="47" t="s">
+      <c r="A24" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="48"/>
-      <c r="C24" s="48"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="48"/>
-      <c r="F24" s="48"/>
-      <c r="G24" s="48"/>
-      <c r="H24" s="48"/>
-      <c r="I24" s="21"/>
+      <c r="B24" s="46"/>
+      <c r="C24" s="46"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="46"/>
+      <c r="G24" s="46"/>
+      <c r="H24" s="46"/>
+      <c r="I24" s="20"/>
       <c r="J24" s="5">
         <v>4</v>
       </c>
@@ -2749,19 +1793,19 @@
       <c r="Z24" s="2"/>
     </row>
     <row r="25" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="41" t="s">
+      <c r="A25" s="43" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="42"/>
-      <c r="C25" s="43"/>
-      <c r="D25" s="45"/>
-      <c r="E25" s="36"/>
-      <c r="F25" s="46"/>
+      <c r="B25" s="26"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="45"/>
       <c r="G25" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="H25" s="51"/>
-      <c r="I25" s="21"/>
+      <c r="H25" s="34"/>
+      <c r="I25" s="20"/>
       <c r="J25" s="5"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
@@ -2781,17 +1825,17 @@
       <c r="Z25" s="2"/>
     </row>
     <row r="26" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="44"/>
-      <c r="B26" s="38"/>
-      <c r="C26" s="39"/>
-      <c r="D26" s="36"/>
-      <c r="E26" s="36"/>
-      <c r="F26" s="46"/>
+      <c r="A26" s="28"/>
+      <c r="B26" s="29"/>
+      <c r="C26" s="30"/>
+      <c r="D26" s="40"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="45"/>
       <c r="G26" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="H26" s="51"/>
-      <c r="I26" s="21"/>
+      <c r="H26" s="34"/>
+      <c r="I26" s="20"/>
       <c r="J26" s="5"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
@@ -2811,17 +1855,17 @@
       <c r="Z26" s="2"/>
     </row>
     <row r="27" spans="1:26" ht="90" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="49" t="s">
+      <c r="A27" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="B27" s="25"/>
-      <c r="C27" s="21"/>
-      <c r="D27" s="52"/>
-      <c r="E27" s="53"/>
-      <c r="F27" s="53"/>
-      <c r="G27" s="53"/>
-      <c r="H27" s="53"/>
-      <c r="I27" s="54"/>
+      <c r="B27" s="19"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="35"/>
+      <c r="E27" s="36"/>
+      <c r="F27" s="36"/>
+      <c r="G27" s="36"/>
+      <c r="H27" s="36"/>
+      <c r="I27" s="37"/>
       <c r="J27" s="5"/>
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
@@ -2841,17 +1885,17 @@
       <c r="Z27" s="2"/>
     </row>
     <row r="28" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="49" t="s">
+      <c r="A28" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="21"/>
-      <c r="D28" s="50"/>
-      <c r="E28" s="21"/>
-      <c r="F28" s="55"/>
-      <c r="G28" s="25"/>
-      <c r="H28" s="25"/>
-      <c r="I28" s="21"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="38"/>
+      <c r="G28" s="19"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="20"/>
       <c r="J28" s="5"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
@@ -9244,25 +8288,15 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="A20:I20"/>
-    <mergeCell ref="A21:C22"/>
-    <mergeCell ref="D21:I22"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="D27:I27"/>
-    <mergeCell ref="F28:I28"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F23:I23"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A25:C26"/>
-    <mergeCell ref="D25:F26"/>
-    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="A1:I10"/>
+    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="A14:C14"/>
     <mergeCell ref="D18:F18"/>
     <mergeCell ref="H18:I18"/>
     <mergeCell ref="A15:C15"/>
@@ -9272,15 +8306,25 @@
     <mergeCell ref="A17:C17"/>
     <mergeCell ref="D17:F17"/>
     <mergeCell ref="A18:C18"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="A1:I10"/>
-    <mergeCell ref="A11:I11"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F23:I23"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A25:C26"/>
+    <mergeCell ref="D25:F26"/>
+    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="D27:I27"/>
+    <mergeCell ref="F28:I28"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A21:C22"/>
+    <mergeCell ref="D21:I22"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.78740157480314965" right="0.78740157480314965" top="0.59055118110236227" bottom="0.39370078740157483" header="0" footer="0"/>

</xml_diff>